<commit_message>
Flash v5.6: MILA OPEX refresh + EBITDA Access location filter and compare
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/excel/ebidta-calculation-mila-lounge.xlsx
+++ b/data/excel/ebidta-calculation-mila-lounge.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MatthiasLavenant\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F0C1C3DA-03B2-424D-AE20-1EADCD705682}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0E39B955-071A-4DC3-A5E1-F65E01621503}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="855" windowWidth="29040" windowHeight="15720" xr2:uid="{A5C5C43F-777E-4BD2-AA0D-D786741A5E2A}"/>
+    <workbookView xWindow="-28920" yWindow="855" windowWidth="29040" windowHeight="15720" xr2:uid="{3C90C578-B115-41AD-8F85-41FE68FE49FA}"/>
   </bookViews>
   <sheets>
     <sheet name="EBIDTA 2" sheetId="1" r:id="rId1"/>
@@ -5580,18 +5580,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80B81ADA-8354-4531-9AEF-1BAE92BBF514}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B26BDD18-EC06-4B8C-8F68-C4E97E1A8EA4}">
   <sheetPr>
     <tabColor rgb="FFE8E05D"/>
   </sheetPr>
-  <dimension ref="B1:FS250"/>
+  <dimension ref="B1:FS290"/>
   <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.75" outlineLevelRow="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.875" style="1" customWidth="1"/>
     <col min="2" max="2" width="37.125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="2.875" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.75" style="20" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.625" style="20" customWidth="1"/>
     <col min="6" max="6" width="2.125" style="20" customWidth="1"/>
     <col min="7" max="7" width="7.5" style="20" customWidth="1"/>
     <col min="10" max="10" width="2.125" customWidth="1"/>
@@ -5600,8 +5600,8 @@
     <col min="15" max="15" width="7.5" customWidth="1"/>
     <col min="18" max="18" width="2.125" customWidth="1"/>
     <col min="19" max="19" width="7.5" customWidth="1"/>
-    <col min="20" max="20" width="10.875" customWidth="1"/>
-    <col min="21" max="21" width="12.5" customWidth="1"/>
+    <col min="20" max="20" width="12.75" customWidth="1"/>
+    <col min="21" max="21" width="18.375" customWidth="1"/>
     <col min="22" max="22" width="2.125" customWidth="1"/>
     <col min="23" max="23" width="7.5" customWidth="1"/>
     <col min="26" max="26" width="2.125" customWidth="1"/>
@@ -6241,8 +6241,7 @@
         <v>11</v>
       </c>
       <c r="D5" s="11">
-        <f>VLOOKUP(D$2,'[1]Overview 2026'!$B$7:$AC$52,$C5,FALSE)</f>
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="E5" s="12"/>
       <c r="F5" s="13"/>
@@ -6423,7 +6422,7 @@
       <c r="C6" s="2"/>
       <c r="D6" s="14">
         <f>IFERROR(D5/D8,"")</f>
-        <v>0.45454545454545453</v>
+        <v>0.14285714285714285</v>
       </c>
       <c r="E6" s="15"/>
       <c r="F6" s="16"/>
@@ -6782,9 +6781,13 @@
       </c>
       <c r="D8" s="19">
         <f>D15+D16</f>
-        <v>220000</v>
+        <v>28000</v>
       </c>
       <c r="E8" s="19"/>
+      <c r="T8" t="str">
+        <f>IFERROR(B8+E8+H8+K8+N8+Q8, "NA")</f>
+        <v>NA</v>
+      </c>
     </row>
     <row r="9" spans="2:175" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
@@ -6799,6 +6802,10 @@
         <v>101500</v>
       </c>
       <c r="E9" s="19"/>
+      <c r="W9">
+        <f>4+4+5</f>
+        <v>13</v>
+      </c>
     </row>
     <row r="10" spans="2:175" x14ac:dyDescent="0.25">
       <c r="B10" s="21" t="s">
@@ -6806,10 +6813,13 @@
       </c>
       <c r="C10" s="22"/>
       <c r="D10" s="23">
-        <f>SUM(D8:E9)</f>
-        <v>321500</v>
+        <v>61500</v>
       </c>
       <c r="E10" s="23"/>
+      <c r="W10">
+        <f>W9*2</f>
+        <v>26</v>
+      </c>
     </row>
     <row r="11" spans="2:175" x14ac:dyDescent="0.25">
       <c r="B11" s="24" t="s">
@@ -6877,7 +6887,7 @@
       </c>
       <c r="D16" s="34">
         <f>IFERROR(D5*E16,0)</f>
-        <v>200000</v>
+        <v>8000</v>
       </c>
       <c r="E16" s="35">
         <f>VLOOKUP(D$2,'[1]Overview 2026'!$B$7:$AC$52,$C16,FALSE)</f>
@@ -6914,7 +6924,7 @@
       </c>
       <c r="D20" s="39">
         <f>D16/D19</f>
-        <v>7142.8571428571431</v>
+        <v>285.71428571428572</v>
       </c>
       <c r="E20" s="39"/>
     </row>
@@ -7111,7 +7121,7 @@
       </c>
       <c r="D33" s="34">
         <f>D$36*E33</f>
-        <v>199330</v>
+        <v>38130</v>
       </c>
       <c r="E33" s="20">
         <v>0.62</v>
@@ -7123,7 +7133,7 @@
       </c>
       <c r="D34" s="34">
         <f t="shared" ref="D34" si="0">D$36*E34</f>
-        <v>109310.00000000001</v>
+        <v>20910</v>
       </c>
       <c r="E34" s="20">
         <f>E36-E33-E35</f>
@@ -7136,7 +7146,7 @@
       </c>
       <c r="D35" s="34">
         <f>D$36*E35</f>
-        <v>12860</v>
+        <v>2460</v>
       </c>
       <c r="E35" s="20">
         <v>0.04</v>
@@ -7149,7 +7159,7 @@
       <c r="C36" s="22"/>
       <c r="D36" s="45">
         <f>D10</f>
-        <v>321500</v>
+        <v>61500</v>
       </c>
       <c r="E36" s="46">
         <v>1</v>
@@ -7164,7 +7174,7 @@
       </c>
       <c r="D38" s="34">
         <f>E38*D33</f>
-        <v>29899.5</v>
+        <v>5719.5</v>
       </c>
       <c r="E38" s="20">
         <v>0.15</v>
@@ -7176,7 +7186,7 @@
       </c>
       <c r="D39" s="34">
         <f t="shared" ref="D39:D40" si="1">E39*D34</f>
-        <v>28967.150000000005</v>
+        <v>5541.1500000000005</v>
       </c>
       <c r="E39" s="20">
         <v>0.26500000000000001</v>
@@ -7188,7 +7198,7 @@
       </c>
       <c r="D40" s="34">
         <f t="shared" si="1"/>
-        <v>3600.8</v>
+        <v>688.80000000000007</v>
       </c>
       <c r="E40" s="20">
         <v>0.28000000000000003</v>
@@ -7201,11 +7211,11 @@
       <c r="C41" s="22"/>
       <c r="D41" s="45">
         <f>SUM(D38:D40)</f>
-        <v>62467.450000000012</v>
+        <v>11949.45</v>
       </c>
       <c r="E41" s="46">
         <f>D41/D36</f>
-        <v>0.19430000000000003</v>
+        <v>0.1943</v>
       </c>
     </row>
     <row r="42" spans="2:175" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
@@ -7218,11 +7228,11 @@
       <c r="C43" s="22"/>
       <c r="D43" s="45">
         <f>D36-D41</f>
-        <v>259032.55</v>
+        <v>49550.55</v>
       </c>
       <c r="E43" s="46">
         <f>D43/D36</f>
-        <v>0.80569999999999997</v>
+        <v>0.80570000000000008</v>
       </c>
     </row>
     <row r="45" spans="2:175" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -7407,12 +7417,12 @@
         <v>22</v>
       </c>
       <c r="D46" s="34">
-        <f>56000/7</f>
-        <v>8000</v>
+        <f>'OPEX DATA 2'!U139+'OPEX DATA 2'!U141+'OPEX DATA 2'!U142</f>
+        <v>4344.7518131868128</v>
       </c>
       <c r="E46" s="20">
         <f>D46/D$36</f>
-        <v>2.4883359253499222E-2</v>
+        <v>7.0646370946127038E-2</v>
       </c>
     </row>
     <row r="47" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7420,12 +7430,12 @@
         <v>23</v>
       </c>
       <c r="D47" s="34">
-        <f>30000/7</f>
-        <v>4285.7142857142853</v>
+        <f>'OPEX DATA 2'!U123+'OPEX DATA 2'!U97+'OPEX DATA 2'!U98+'OPEX DATA 2'!U110+'OPEX DATA 2'!U112</f>
+        <v>1423.4991208791207</v>
       </c>
       <c r="E47" s="20">
         <f t="shared" ref="E47:E50" si="2">D47/D$36</f>
-        <v>1.3330371028660297E-2</v>
+        <v>2.314632716876619E-2</v>
       </c>
     </row>
     <row r="48" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7433,12 +7443,12 @@
         <v>24</v>
       </c>
       <c r="D48" s="34">
-        <f>70000/7</f>
-        <v>10000</v>
+        <f>'OPEX DATA 2'!U85+'OPEX DATA 2'!U86+'OPEX DATA 2'!U87+'OPEX DATA 2'!U88+'OPEX DATA 2'!U92+'OPEX DATA 2'!U124</f>
+        <v>3049.357857142857</v>
       </c>
       <c r="E48" s="20">
         <f t="shared" si="2"/>
-        <v>3.110419906687403E-2</v>
+        <v>4.9583054587688732E-2</v>
       </c>
     </row>
     <row r="49" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7446,12 +7456,12 @@
         <v>25</v>
       </c>
       <c r="D49" s="34">
-        <f>SUM(D46:D48)*18.7%</f>
-        <v>4167.4285714285716</v>
+        <f>'OPEX DATA 2'!U151+'OPEX DATA 2'!U153+'OPEX DATA 2'!U154</f>
+        <v>2499.9871978021974</v>
       </c>
       <c r="E49" s="20">
         <f t="shared" si="2"/>
-        <v>1.2962452788269274E-2</v>
+        <v>4.0650198338247116E-2</v>
       </c>
     </row>
     <row r="50" spans="2:175" x14ac:dyDescent="0.25">
@@ -7461,11 +7471,11 @@
       <c r="C50" s="22"/>
       <c r="D50" s="45">
         <f>SUM(D46:D49)</f>
-        <v>26453.142857142859</v>
+        <v>11317.595989010988</v>
       </c>
       <c r="E50" s="46">
         <f t="shared" si="2"/>
-        <v>8.2280382137302821E-2</v>
+        <v>0.18402595104082908</v>
       </c>
     </row>
     <row r="52" spans="2:175" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -7658,7 +7668,7 @@
       </c>
       <c r="E53" s="20">
         <f t="shared" ref="E53:E101" si="3">D53/D$36</f>
-        <v>4.7989335703177072E-7</v>
+        <v>2.5087108013937279E-6</v>
       </c>
     </row>
     <row r="54" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7672,7 +7682,7 @@
       </c>
       <c r="E54" s="20">
         <f t="shared" si="3"/>
-        <v>2.7107343667219248E-4</v>
+        <v>1.4170749575627623E-3</v>
       </c>
     </row>
     <row r="55" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7686,7 +7696,7 @@
       </c>
       <c r="E55" s="20">
         <f t="shared" si="3"/>
-        <v>4.3659374839779202E-4</v>
+        <v>2.2823559367461809E-3</v>
       </c>
     </row>
     <row r="56" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7700,7 +7710,7 @@
       </c>
       <c r="E56" s="20">
         <f t="shared" si="3"/>
-        <v>6.836976398407191E-5</v>
+        <v>3.574126686321808E-4</v>
       </c>
     </row>
     <row r="57" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7714,7 +7724,7 @@
       </c>
       <c r="E57" s="20">
         <f t="shared" si="3"/>
-        <v>7.3182027925418276E-5</v>
+        <v>3.8256946305726791E-4</v>
       </c>
     </row>
     <row r="58" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7728,7 +7738,7 @@
       </c>
       <c r="E58" s="20">
         <f t="shared" si="3"/>
-        <v>4.1002751525302079E-4</v>
+        <v>2.143477173233271E-3</v>
       </c>
     </row>
     <row r="59" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7742,7 +7752,7 @@
       </c>
       <c r="E59" s="20">
         <f t="shared" si="3"/>
-        <v>3.0751679114043038E-4</v>
+        <v>1.6075877780755831E-3</v>
       </c>
     </row>
     <row r="60" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7756,7 +7766,7 @@
       </c>
       <c r="E60" s="20">
         <f t="shared" si="3"/>
-        <v>1.2595481346025672E-3</v>
+        <v>6.5844670776378112E-3</v>
       </c>
     </row>
     <row r="61" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7770,7 +7780,7 @@
       </c>
       <c r="E61" s="20">
         <f t="shared" si="3"/>
-        <v>6.3966639891989822E-5</v>
+        <v>3.3439471098007685E-4</v>
       </c>
     </row>
     <row r="62" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7784,7 +7794,7 @@
       </c>
       <c r="E62" s="20">
         <f t="shared" si="3"/>
-        <v>4.4900552014082336E-4</v>
+        <v>2.3472402394353613E-3</v>
       </c>
     </row>
     <row r="63" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7798,7 +7808,7 @@
       </c>
       <c r="E63" s="20">
         <f t="shared" si="3"/>
-        <v>4.9654179413121877E-4</v>
+        <v>2.595742875011168E-3</v>
       </c>
     </row>
     <row r="64" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7854,7 +7864,7 @@
       </c>
       <c r="E67" s="20">
         <f t="shared" si="3"/>
-        <v>4.8027498162801427E-4</v>
+        <v>2.5107057982667741E-3</v>
       </c>
     </row>
     <row r="68" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7868,7 +7878,7 @@
       </c>
       <c r="E68" s="20">
         <f t="shared" si="3"/>
-        <v>4.6007553876916248E-4</v>
+        <v>2.4051103368176543E-3</v>
       </c>
     </row>
     <row r="69" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7882,7 +7892,7 @@
       </c>
       <c r="E69" s="20">
         <f t="shared" si="3"/>
-        <v>3.7136021055150136E-4</v>
+        <v>1.9413383364602875E-3</v>
       </c>
     </row>
     <row r="70" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7896,7 +7906,7 @@
       </c>
       <c r="E70" s="20">
         <f t="shared" si="3"/>
-        <v>5.2807598311486342E-4</v>
+        <v>2.760592334494774E-3</v>
       </c>
     </row>
     <row r="71" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7910,7 +7920,7 @@
       </c>
       <c r="E71" s="20">
         <f t="shared" si="3"/>
-        <v>1.7697913284227436E-4</v>
+        <v>9.2518359689091386E-4</v>
       </c>
     </row>
     <row r="72" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7924,7 +7934,7 @@
       </c>
       <c r="E72" s="20">
         <f t="shared" si="3"/>
-        <v>9.3076735084511131E-4</v>
+        <v>4.8657187527919232E-3</v>
       </c>
     </row>
     <row r="73" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7952,7 +7962,7 @@
       </c>
       <c r="E74" s="20">
         <f t="shared" si="3"/>
-        <v>6.8273716951788489E-6</v>
+        <v>3.5691056910569106E-5</v>
       </c>
     </row>
     <row r="75" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7966,7 +7976,7 @@
       </c>
       <c r="E75" s="20">
         <f t="shared" si="3"/>
-        <v>2.6041614683916395E-4</v>
+        <v>1.3613624586795319E-3</v>
       </c>
     </row>
     <row r="76" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7980,7 +7990,7 @@
       </c>
       <c r="E76" s="20">
         <f t="shared" si="3"/>
-        <v>9.0686343205783324E-5</v>
+        <v>4.740757616367372E-4</v>
       </c>
     </row>
     <row r="77" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8022,7 +8032,7 @@
       </c>
       <c r="E79" s="20">
         <f t="shared" si="3"/>
-        <v>3.7320082716661254E-5</v>
+        <v>1.9509604216921291E-4</v>
       </c>
     </row>
     <row r="80" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8036,7 +8046,7 @@
       </c>
       <c r="E80" s="20">
         <f t="shared" si="3"/>
-        <v>3.1826619725531082E-4</v>
+        <v>1.6637818279281694E-3</v>
       </c>
     </row>
     <row r="81" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8050,7 +8060,7 @@
       </c>
       <c r="E81" s="20">
         <f t="shared" si="3"/>
-        <v>5.3045032727769888E-4</v>
+        <v>2.7730045564191902E-3</v>
       </c>
     </row>
     <row r="82" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8064,7 +8074,7 @@
       </c>
       <c r="E82" s="20">
         <f t="shared" si="3"/>
-        <v>2.1250833148189292E-5</v>
+        <v>1.1109175377468061E-4</v>
       </c>
     </row>
     <row r="83" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8092,7 +8102,7 @@
       </c>
       <c r="E84" s="20">
         <f t="shared" si="3"/>
-        <v>3.0169859689299812E-4</v>
+        <v>1.5771723398552667E-3</v>
       </c>
     </row>
     <row r="85" spans="2:175" x14ac:dyDescent="0.25">
@@ -8107,7 +8117,7 @@
       </c>
       <c r="E85" s="46">
         <f t="shared" si="3"/>
-        <v>2.205946199989746E-3</v>
+        <v>1.153189761458054E-2</v>
       </c>
     </row>
     <row r="86" spans="2:175" x14ac:dyDescent="0.25">
@@ -8121,7 +8131,7 @@
       </c>
       <c r="E86" s="20">
         <f t="shared" si="3"/>
-        <v>1.0622820569787909E-3</v>
+        <v>5.553230590547663E-3</v>
       </c>
     </row>
     <row r="87" spans="2:175" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -8136,7 +8146,7 @@
       </c>
       <c r="E87" s="18">
         <f t="shared" si="3"/>
-        <v>1.3227453728231333E-4</v>
+        <v>6.9148396319128021E-4</v>
       </c>
       <c r="F87" s="18"/>
       <c r="G87" s="18"/>
@@ -8316,11 +8326,11 @@
       </c>
       <c r="D88" s="34">
         <f>D5</f>
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="E88" s="20">
         <f t="shared" si="3"/>
-        <v>0.31104199066874028</v>
+        <v>6.5040650406504072E-2</v>
       </c>
     </row>
     <row r="89" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8334,7 +8344,7 @@
       </c>
       <c r="E89" s="20">
         <f t="shared" si="3"/>
-        <v>5.1189991967596939E-5</v>
+        <v>2.6760296613955148E-4</v>
       </c>
     </row>
     <row r="90" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8390,7 +8400,7 @@
       </c>
       <c r="E93" s="20">
         <f t="shared" si="3"/>
-        <v>4.8034795686428659E-5</v>
+        <v>2.5110872866970427E-4</v>
       </c>
     </row>
     <row r="94" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8499,11 +8509,11 @@
       <c r="C101" s="48"/>
       <c r="D101" s="49">
         <f>SUM(D53:D100)</f>
-        <v>103809.92994505494</v>
+        <v>7809.9299450549461</v>
       </c>
       <c r="E101" s="50">
         <f t="shared" si="3"/>
-        <v>0.32289247261292364</v>
+        <v>0.12699073081390155</v>
       </c>
       <c r="F101" s="50"/>
       <c r="G101" s="50"/>
@@ -8530,7 +8540,7 @@
       </c>
       <c r="E104" s="20">
         <f t="shared" ref="E104:E130" si="4">D104/D$36</f>
-        <v>6.0430077076888897E-3</v>
+        <v>3.1590682569463055E-2</v>
       </c>
     </row>
     <row r="105" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8544,7 +8554,7 @@
       </c>
       <c r="E105" s="20">
         <f t="shared" si="4"/>
-        <v>8.72284791413874E-5</v>
+        <v>4.5599928526757802E-4</v>
       </c>
     </row>
     <row r="106" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8558,7 +8568,7 @@
       </c>
       <c r="E106" s="20">
         <f t="shared" si="4"/>
-        <v>1.3268748825047427E-3</v>
+        <v>6.9364272313052807E-3</v>
       </c>
     </row>
     <row r="107" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8572,7 +8582,7 @@
       </c>
       <c r="E107" s="20">
         <f t="shared" si="4"/>
-        <v>1.0655478269786202E-4</v>
+        <v>5.5703028678638438E-4</v>
       </c>
     </row>
     <row r="108" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8586,7 +8596,7 @@
       </c>
       <c r="E108" s="20">
         <f t="shared" si="4"/>
-        <v>2.4717649069437562E-3</v>
+        <v>1.2921502724917358E-2</v>
       </c>
     </row>
     <row r="109" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8600,7 +8610,7 @@
       </c>
       <c r="E109" s="20">
         <f t="shared" si="4"/>
-        <v>5.7148326013022746E-5</v>
+        <v>2.9875100509246848E-4</v>
       </c>
     </row>
     <row r="110" spans="2:175" x14ac:dyDescent="0.25">
@@ -8629,7 +8639,7 @@
       </c>
       <c r="E111" s="20">
         <f t="shared" si="4"/>
-        <v>2.7363662775793414E-5</v>
+        <v>1.4304744036451353E-4</v>
       </c>
     </row>
     <row r="112" spans="2:175" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -8644,7 +8654,7 @@
       </c>
       <c r="E112" s="18">
         <f t="shared" si="4"/>
-        <v>1.2698032915762308E-7</v>
+        <v>6.6380773697846864E-7</v>
       </c>
       <c r="F112" s="18"/>
       <c r="G112" s="18"/>
@@ -8828,7 +8838,7 @@
       </c>
       <c r="E113" s="20">
         <f t="shared" si="4"/>
-        <v>1.1838565788799071E-5</v>
+        <v>6.1887787009738235E-5</v>
       </c>
     </row>
     <row r="114" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8856,7 +8866,7 @@
       </c>
       <c r="E115" s="20">
         <f t="shared" si="4"/>
-        <v>-2.3317895168595012E-6</v>
+        <v>-1.218976145805414E-5</v>
       </c>
     </row>
     <row r="116" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8870,7 +8880,7 @@
       </c>
       <c r="E116" s="20">
         <f t="shared" si="4"/>
-        <v>3.6887067831080275E-4</v>
+        <v>1.9283239524702941E-3</v>
       </c>
     </row>
     <row r="117" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8884,7 +8894,7 @@
       </c>
       <c r="E117" s="20">
         <f t="shared" si="4"/>
-        <v>7.5609351767983192E-5</v>
+        <v>3.9525864379522921E-4</v>
       </c>
     </row>
     <row r="118" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8898,7 +8908,7 @@
       </c>
       <c r="E118" s="20">
         <f t="shared" si="4"/>
-        <v>1.8970143386939653E-6</v>
+        <v>9.9169123559367455E-6</v>
       </c>
     </row>
     <row r="119" spans="2:175" x14ac:dyDescent="0.25">
@@ -8913,7 +8923,7 @@
       </c>
       <c r="E119" s="46">
         <f t="shared" si="4"/>
-        <v>2.5484593167330336E-4</v>
+        <v>1.3322433663897077E-3</v>
       </c>
     </row>
     <row r="120" spans="2:175" x14ac:dyDescent="0.25">
@@ -8942,7 +8952,7 @@
       </c>
       <c r="E121" s="18">
         <f t="shared" si="4"/>
-        <v>8.5451096337566006E-6</v>
+        <v>4.4670776378093451E-5</v>
       </c>
       <c r="F121" s="18"/>
       <c r="G121" s="18"/>
@@ -9127,7 +9137,7 @@
       </c>
       <c r="E122" s="46">
         <f t="shared" si="4"/>
-        <v>1.5623878454360571E-6</v>
+        <v>8.1676047529706064E-6</v>
       </c>
     </row>
     <row r="123" spans="2:175" x14ac:dyDescent="0.25">
@@ -9141,7 +9151,7 @@
       </c>
       <c r="E123" s="20">
         <f t="shared" si="4"/>
-        <v>1.3527421256814726E-5</v>
+        <v>7.0716519253104617E-5</v>
       </c>
     </row>
     <row r="124" spans="2:175" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -9156,7 +9166,7 @@
       </c>
       <c r="E124" s="18">
         <f t="shared" si="4"/>
-        <v>1.1178216806521627E-4</v>
+        <v>5.8435718752791917E-4</v>
       </c>
       <c r="F124" s="18"/>
       <c r="G124" s="18"/>
@@ -9340,7 +9350,7 @@
       </c>
       <c r="E125" s="20">
         <f t="shared" si="4"/>
-        <v>3.4997219421325177E-3</v>
+        <v>1.8295294380416331E-2</v>
       </c>
     </row>
     <row r="126" spans="2:175" x14ac:dyDescent="0.25">
@@ -9355,7 +9365,7 @@
       </c>
       <c r="E126" s="46">
         <f t="shared" si="4"/>
-        <v>2.5297728709859353E-4</v>
+        <v>1.3224747610113465E-3</v>
       </c>
     </row>
     <row r="127" spans="2:175" x14ac:dyDescent="0.25">
@@ -9369,7 +9379,7 @@
       </c>
       <c r="E127" s="20">
         <f t="shared" si="4"/>
-        <v>3.6860014013979799E-5</v>
+        <v>1.9269096756901636E-4</v>
       </c>
     </row>
     <row r="128" spans="2:175" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -9583,7 +9593,7 @@
       </c>
       <c r="E130" s="50">
         <f t="shared" si="4"/>
-        <v>1.4755775810503651E-2</v>
+        <v>7.7137917448405258E-2</v>
       </c>
       <c r="F130" s="50"/>
       <c r="G130" s="50"/>
@@ -9610,7 +9620,7 @@
       </c>
       <c r="E133" s="20">
         <f t="shared" ref="E133:E141" si="5">D133/D$36</f>
-        <v>6.5192179515663167E-5</v>
+        <v>3.4080139372822294E-4</v>
       </c>
     </row>
     <row r="134" spans="2:7" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -9624,7 +9634,7 @@
       </c>
       <c r="E134" s="20">
         <f t="shared" si="5"/>
-        <v>4.673440090236357E-5</v>
+        <v>2.44310729920486E-4</v>
       </c>
     </row>
     <row r="135" spans="2:7" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -9652,7 +9662,7 @@
       </c>
       <c r="E136" s="20">
         <f t="shared" si="5"/>
-        <v>4.5040110744620857E-4</v>
+        <v>2.3545358706334317E-3</v>
       </c>
     </row>
     <row r="137" spans="2:7" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -9666,7 +9676,7 @@
       </c>
       <c r="E137" s="20">
         <f t="shared" si="5"/>
-        <v>7.732640609779024E-5</v>
+        <v>4.0423478960064328E-4</v>
       </c>
     </row>
     <row r="138" spans="2:7" x14ac:dyDescent="0.25">
@@ -9681,7 +9691,7 @@
       </c>
       <c r="E138" s="46">
         <f t="shared" si="5"/>
-        <v>4.8358057183873668E-4</v>
+        <v>2.5279862414008753E-3</v>
       </c>
     </row>
     <row r="139" spans="2:7" x14ac:dyDescent="0.25">
@@ -9725,7 +9735,7 @@
       </c>
       <c r="E141" s="50">
         <f t="shared" si="5"/>
-        <v>1.1232346658007623E-3</v>
+        <v>5.8718690252836598E-3</v>
       </c>
       <c r="F141" s="50"/>
       <c r="G141" s="50"/>
@@ -9772,7 +9782,7 @@
       </c>
       <c r="E145" s="58">
         <f t="shared" si="6"/>
-        <v>7.8015148770358735E-3</v>
+        <v>4.0783528991333876E-2</v>
       </c>
     </row>
     <row r="146" spans="2:7" x14ac:dyDescent="0.25">
@@ -9802,7 +9812,7 @@
       </c>
       <c r="E147" s="58">
         <f t="shared" si="6"/>
-        <v>3.9211559824312546E-4</v>
+        <v>2.0498400786205665E-3</v>
       </c>
     </row>
     <row r="148" spans="2:7" x14ac:dyDescent="0.25">
@@ -9847,7 +9857,7 @@
       </c>
       <c r="E150" s="58">
         <f t="shared" si="6"/>
-        <v>2.587268299352281E-3</v>
+        <v>1.3525313142142411E-2</v>
       </c>
     </row>
     <row r="151" spans="2:7" x14ac:dyDescent="0.25">
@@ -9862,7 +9872,7 @@
       </c>
       <c r="E151" s="58">
         <f t="shared" si="6"/>
-        <v>9.610363508963819E-4</v>
+        <v>5.0239542571249886E-3</v>
       </c>
     </row>
     <row r="152" spans="2:7" x14ac:dyDescent="0.25">
@@ -9877,7 +9887,7 @@
       </c>
       <c r="E152" s="50">
         <f t="shared" si="6"/>
-        <v>1.1741935125527661E-2</v>
+        <v>6.1382636469221839E-2</v>
       </c>
       <c r="F152" s="50"/>
       <c r="G152" s="50"/>
@@ -9939,7 +9949,7 @@
       </c>
       <c r="E157" s="58">
         <f t="shared" si="7"/>
-        <v>-5.6534445336933666E-7</v>
+        <v>-2.9554185651746624E-6</v>
       </c>
     </row>
     <row r="158" spans="2:7" x14ac:dyDescent="0.25">
@@ -10089,7 +10099,7 @@
       </c>
       <c r="E167" s="58">
         <f t="shared" si="7"/>
-        <v>-7.106938287218225E-3</v>
+        <v>-3.7152531046189582E-2</v>
       </c>
     </row>
     <row r="168" spans="2:7" x14ac:dyDescent="0.25">
@@ -10164,7 +10174,7 @@
       </c>
       <c r="E172" s="50">
         <f t="shared" si="7"/>
-        <v>-7.1075036316715946E-3</v>
+        <v>-3.7155486464754757E-2</v>
       </c>
       <c r="F172" s="50"/>
       <c r="G172" s="50"/>
@@ -10211,7 +10221,7 @@
       </c>
       <c r="E176" s="58">
         <f t="shared" si="8"/>
-        <v>1.1735703177071762E-3</v>
+        <v>6.1350058072009292E-3</v>
       </c>
     </row>
     <row r="177" spans="2:5" x14ac:dyDescent="0.25">
@@ -10226,7 +10236,7 @@
       </c>
       <c r="E177" s="58">
         <f t="shared" si="8"/>
-        <v>1.0099224274947447E-2</v>
+        <v>5.2795131778790312E-2</v>
       </c>
     </row>
     <row r="178" spans="2:5" x14ac:dyDescent="0.25">
@@ -10241,7 +10251,7 @@
       </c>
       <c r="E178" s="58">
         <f t="shared" si="8"/>
-        <v>1.264676225795977E-6</v>
+        <v>6.6112749039578306E-6</v>
       </c>
     </row>
     <row r="179" spans="2:5" x14ac:dyDescent="0.25">
@@ -10256,7 +10266,7 @@
       </c>
       <c r="E179" s="58">
         <f t="shared" si="8"/>
-        <v>2.6903423170919282E-4</v>
+        <v>1.4064147234878941E-3</v>
       </c>
     </row>
     <row r="180" spans="2:5" x14ac:dyDescent="0.25">
@@ -10271,7 +10281,7 @@
       </c>
       <c r="E180" s="58">
         <f t="shared" si="8"/>
-        <v>2.6020371541366874E-5</v>
+        <v>1.3602519431787723E-4</v>
       </c>
     </row>
     <row r="181" spans="2:5" x14ac:dyDescent="0.25">
@@ -10286,7 +10296,7 @@
       </c>
       <c r="E181" s="58">
         <f t="shared" si="8"/>
-        <v>6.7838668330114668E-4</v>
+        <v>3.546362905387295E-3</v>
       </c>
     </row>
     <row r="182" spans="2:5" x14ac:dyDescent="0.25">
@@ -10331,7 +10341,7 @@
       </c>
       <c r="E184" s="58">
         <f t="shared" si="8"/>
-        <v>8.2456889921897697E-6</v>
+        <v>4.3105512373805061E-5</v>
       </c>
     </row>
     <row r="185" spans="2:5" x14ac:dyDescent="0.25">
@@ -10586,7 +10596,7 @@
       </c>
       <c r="E201" s="50">
         <f t="shared" si="8"/>
-        <v>1.2255746244424316E-2</v>
+        <v>6.406865719646207E-2</v>
       </c>
       <c r="F201" s="50"/>
       <c r="G201" s="50"/>
@@ -10604,11 +10614,11 @@
       <c r="C203" s="48"/>
       <c r="D203" s="49">
         <f>D43-D50-D101-D130-D141-D152-D172-D201</f>
-        <v>118234.18318681316</v>
+        <v>19887.730054945059</v>
       </c>
       <c r="E203" s="50">
         <f>D203/D36</f>
-        <v>0.36775795703518865</v>
+        <v>0.32337772447065138</v>
       </c>
       <c r="F203" s="50"/>
       <c r="G203" s="50"/>
@@ -10634,7 +10644,7 @@
       <c r="C207" s="63"/>
       <c r="D207" s="64">
         <f>E203</f>
-        <v>0.36775795703518865</v>
+        <v>0.32337772447065138</v>
       </c>
     </row>
     <row r="208" spans="2:175" s="20" customFormat="1" x14ac:dyDescent="0.25">
@@ -18334,6 +18344,12 @@
       <c r="FR250"/>
       <c r="FS250"/>
     </row>
+    <row r="290" spans="21:21" x14ac:dyDescent="0.25">
+      <c r="U290" t="e">
+        <f>(T290/$V$1)/7</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="13">
     <mergeCell ref="D205:E205"/>
@@ -18363,31 +18379,33 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC25C6C0-3CDE-4CEC-A6B3-1740C0B3E733}">
-  <dimension ref="A1:V332"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0F99862-AB87-4CF6-8D35-9F6AF745B5F6}">
+  <dimension ref="A1:W332"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37.5" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="2" max="2" width="17.875" customWidth="1"/>
     <col min="3" max="3" width="8.25" customWidth="1"/>
-    <col min="4" max="4" width="1.25" customWidth="1"/>
-    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="4" max="4" width="14.375" customWidth="1"/>
+    <col min="5" max="5" width="18.125" customWidth="1"/>
     <col min="6" max="6" width="8.25" customWidth="1"/>
     <col min="7" max="7" width="1.25" customWidth="1"/>
-    <col min="8" max="8" width="15" customWidth="1"/>
+    <col min="8" max="8" width="17.5" customWidth="1"/>
     <col min="9" max="9" width="8.25" customWidth="1"/>
     <col min="10" max="10" width="1.25" customWidth="1"/>
-    <col min="11" max="11" width="15" customWidth="1"/>
+    <col min="11" max="11" width="19.125" customWidth="1"/>
     <col min="12" max="12" width="8.25" customWidth="1"/>
     <col min="13" max="13" width="1.25" customWidth="1"/>
-    <col min="14" max="14" width="15" customWidth="1"/>
+    <col min="14" max="14" width="20" customWidth="1"/>
     <col min="15" max="15" width="8.25" customWidth="1"/>
     <col min="16" max="16" width="1.25" customWidth="1"/>
-    <col min="17" max="17" width="15" customWidth="1"/>
+    <col min="17" max="17" width="20.875" customWidth="1"/>
     <col min="18" max="18" width="8.25" customWidth="1"/>
+    <col min="20" max="20" width="12.75" customWidth="1"/>
+    <col min="21" max="21" width="18.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>29</v>
       </c>
@@ -18398,7 +18416,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A5" s="67" t="s">
         <v>31</v>
       </c>
@@ -18460,7 +18478,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" s="71" t="s">
         <v>40</v>
       </c>
@@ -18482,7 +18500,7 @@
       <c r="Q6" s="72"/>
       <c r="R6" s="73"/>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A7" s="75" t="s">
         <v>14</v>
       </c>
@@ -18504,7 +18522,7 @@
       <c r="Q7" s="72"/>
       <c r="R7" s="73"/>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A8" s="76" t="s">
         <v>41</v>
       </c>
@@ -18564,7 +18582,7 @@
         <v>17134.665164835165</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9" s="76" t="s">
         <v>42</v>
       </c>
@@ -18623,8 +18641,12 @@
         <f t="shared" ref="U9:U72" si="1">(T9/$V$1)/7</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W9">
+        <f>4+4+5</f>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A10" s="81" t="s">
         <v>43</v>
       </c>
@@ -18689,8 +18711,12 @@
         <f t="shared" si="1"/>
         <v>17134.665164835165</v>
       </c>
-    </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W10">
+        <f>W9*2</f>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A11" s="84" t="s">
         <v>44</v>
       </c>
@@ -18750,7 +18776,7 @@
         <v>2024.687032967033</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A12" s="75" t="s">
         <v>13</v>
       </c>
@@ -18780,7 +18806,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A13" s="76" t="s">
         <v>45</v>
       </c>
@@ -18840,7 +18866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A14" s="76" t="s">
         <v>46</v>
       </c>
@@ -18900,7 +18926,7 @@
         <v>29826.415989010991</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A15" s="76" t="s">
         <v>47</v>
       </c>
@@ -18960,7 +18986,7 @@
         <v>297.74175824175825</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A16" s="76" t="s">
         <v>48</v>
       </c>
@@ -20699,7 +20725,10 @@
         <f>IFERROR(B46/B327, "NA")</f>
         <v>-1.0903096941534676E-2</v>
       </c>
-      <c r="D46" s="79"/>
+      <c r="D46" s="79">
+        <f>(11977+7579+3952)/7</f>
+        <v>3358.2857142857142</v>
+      </c>
       <c r="E46" s="77">
         <v>-19531</v>
       </c>
@@ -20939,7 +20968,10 @@
         <f>IFERROR(B50/B327, "NA")</f>
         <v>-2.0251444563342113E-3</v>
       </c>
-      <c r="D50" s="79"/>
+      <c r="D50" s="79">
+        <f>SUM(D46:D49)</f>
+        <v>3358.2857142857142</v>
+      </c>
       <c r="E50" s="77">
         <v>-3426.8</v>
       </c>
@@ -34976,7 +35008,7 @@
         <v>590935.91</v>
       </c>
       <c r="U290" s="80">
-        <f t="shared" si="9"/>
+        <f>(T290/$V$1)/7</f>
         <v>3246.9006043956042</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Flash v5.7: MILA OPEX refresh from updated EBITDA workbook
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/excel/ebidta-calculation-mila-lounge.xlsx
+++ b/data/excel/ebidta-calculation-mila-lounge.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MatthiasLavenant\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0E39B955-071A-4DC3-A5E1-F65E01621503}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1489FA02-5096-4E88-B8B1-3E6B83A97E1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="855" windowWidth="29040" windowHeight="15720" xr2:uid="{3C90C578-B115-41AD-8F85-41FE68FE49FA}"/>
   </bookViews>
@@ -7418,11 +7418,11 @@
       </c>
       <c r="D46" s="34">
         <f>'OPEX DATA 2'!U139+'OPEX DATA 2'!U141+'OPEX DATA 2'!U142</f>
-        <v>4344.7518131868128</v>
+        <v>7603.3156730769233</v>
       </c>
       <c r="E46" s="20">
         <f>D46/D$36</f>
-        <v>7.0646370946127038E-2</v>
+        <v>0.12363114915572233</v>
       </c>
     </row>
     <row r="47" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7431,11 +7431,11 @@
       </c>
       <c r="D47" s="34">
         <f>'OPEX DATA 2'!U123+'OPEX DATA 2'!U97+'OPEX DATA 2'!U98+'OPEX DATA 2'!U110+'OPEX DATA 2'!U112</f>
-        <v>1423.4991208791207</v>
+        <v>2491.1234615384615</v>
       </c>
       <c r="E47" s="20">
         <f t="shared" ref="E47:E50" si="2">D47/D$36</f>
-        <v>2.314632716876619E-2</v>
+        <v>4.0506072545340839E-2</v>
       </c>
     </row>
     <row r="48" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7444,11 +7444,11 @@
       </c>
       <c r="D48" s="34">
         <f>'OPEX DATA 2'!U85+'OPEX DATA 2'!U86+'OPEX DATA 2'!U87+'OPEX DATA 2'!U88+'OPEX DATA 2'!U92+'OPEX DATA 2'!U124</f>
-        <v>3049.357857142857</v>
+        <v>5336.3762500000003</v>
       </c>
       <c r="E48" s="20">
         <f t="shared" si="2"/>
-        <v>4.9583054587688732E-2</v>
+        <v>8.6770345528455292E-2</v>
       </c>
     </row>
     <row r="49" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7457,11 +7457,11 @@
       </c>
       <c r="D49" s="34">
         <f>'OPEX DATA 2'!U151+'OPEX DATA 2'!U153+'OPEX DATA 2'!U154</f>
-        <v>2499.9871978021974</v>
+        <v>4374.9775961538462</v>
       </c>
       <c r="E49" s="20">
         <f t="shared" si="2"/>
-        <v>4.0650198338247116E-2</v>
+        <v>7.1137847091932452E-2</v>
       </c>
     </row>
     <row r="50" spans="2:175" x14ac:dyDescent="0.25">
@@ -7471,11 +7471,11 @@
       <c r="C50" s="22"/>
       <c r="D50" s="45">
         <f>SUM(D46:D49)</f>
-        <v>11317.595989010988</v>
+        <v>19805.792980769231</v>
       </c>
       <c r="E50" s="46">
         <f t="shared" si="2"/>
-        <v>0.18402595104082908</v>
+        <v>0.3220454143214509</v>
       </c>
     </row>
     <row r="52" spans="2:175" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -7664,11 +7664,11 @@
       </c>
       <c r="D53" s="34">
         <f>'OPEX DATA 2'!U161</f>
-        <v>0.15428571428571428</v>
+        <v>0.26999999999999996</v>
       </c>
       <c r="E53" s="20">
         <f t="shared" ref="E53:E101" si="3">D53/D$36</f>
-        <v>2.5087108013937279E-6</v>
+        <v>4.3902439024390241E-6</v>
       </c>
     </row>
     <row r="54" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7678,11 +7678,11 @@
       </c>
       <c r="D54" s="34">
         <f>'OPEX DATA 2'!U162</f>
-        <v>87.150109890109889</v>
+        <v>152.5126923076923</v>
       </c>
       <c r="E54" s="20">
         <f t="shared" si="3"/>
-        <v>1.4170749575627623E-3</v>
+        <v>2.4798811757348344E-3</v>
       </c>
     </row>
     <row r="55" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7692,11 +7692,11 @@
       </c>
       <c r="D55" s="34">
         <f>'OPEX DATA 2'!U163</f>
-        <v>140.36489010989013</v>
+        <v>245.6385576923077</v>
       </c>
       <c r="E55" s="20">
         <f t="shared" si="3"/>
-        <v>2.2823559367461809E-3</v>
+        <v>3.9941228893058166E-3</v>
       </c>
     </row>
     <row r="56" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7706,11 +7706,11 @@
       </c>
       <c r="D56" s="34">
         <f>'OPEX DATA 2'!U164</f>
-        <v>21.98087912087912</v>
+        <v>38.466538461538462</v>
       </c>
       <c r="E56" s="20">
         <f t="shared" si="3"/>
-        <v>3.574126686321808E-4</v>
+        <v>6.2547217010631647E-4</v>
       </c>
     </row>
     <row r="57" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7720,11 +7720,11 @@
       </c>
       <c r="D57" s="34">
         <f>'OPEX DATA 2'!U165</f>
-        <v>23.528021978021975</v>
+        <v>41.174038461538458</v>
       </c>
       <c r="E57" s="20">
         <f t="shared" si="3"/>
-        <v>3.8256946305726791E-4</v>
+        <v>6.6949656035021881E-4</v>
       </c>
     </row>
     <row r="58" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7734,11 +7734,11 @@
       </c>
       <c r="D58" s="34">
         <f>'OPEX DATA 2'!U166</f>
-        <v>131.82384615384618</v>
+        <v>230.69173076923079</v>
       </c>
       <c r="E58" s="20">
         <f t="shared" si="3"/>
-        <v>2.143477173233271E-3</v>
+        <v>3.7510850531582243E-3</v>
       </c>
     </row>
     <row r="59" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7748,11 +7748,11 @@
       </c>
       <c r="D59" s="34">
         <f>'OPEX DATA 2'!U167</f>
-        <v>98.866648351648365</v>
+        <v>173.01663461538465</v>
       </c>
       <c r="E59" s="20">
         <f t="shared" si="3"/>
-        <v>1.6075877780755831E-3</v>
+        <v>2.8132786116322707E-3</v>
       </c>
     </row>
     <row r="60" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7762,11 +7762,11 @@
       </c>
       <c r="D60" s="34">
         <f>'OPEX DATA 2'!U168</f>
-        <v>404.94472527472539</v>
+        <v>708.65326923076941</v>
       </c>
       <c r="E60" s="20">
         <f t="shared" si="3"/>
-        <v>6.5844670776378112E-3</v>
+        <v>1.152281738586617E-2</v>
       </c>
     </row>
     <row r="61" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7776,11 +7776,11 @@
       </c>
       <c r="D61" s="34">
         <f>'OPEX DATA 2'!U169</f>
-        <v>20.565274725274726</v>
+        <v>35.989230769230772</v>
       </c>
       <c r="E61" s="20">
         <f t="shared" si="3"/>
-        <v>3.3439471098007685E-4</v>
+        <v>5.8519074421513448E-4</v>
       </c>
     </row>
     <row r="62" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7790,11 +7790,11 @@
       </c>
       <c r="D62" s="34">
         <f>'OPEX DATA 2'!U170</f>
-        <v>144.35527472527471</v>
+        <v>252.62173076923077</v>
       </c>
       <c r="E62" s="20">
         <f t="shared" si="3"/>
-        <v>2.3472402394353613E-3</v>
+        <v>4.1076704190118824E-3</v>
       </c>
     </row>
     <row r="63" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7804,11 +7804,11 @@
       </c>
       <c r="D63" s="34">
         <f>'OPEX DATA 2'!U171</f>
-        <v>159.63818681318682</v>
+        <v>279.36682692307693</v>
       </c>
       <c r="E63" s="20">
         <f t="shared" si="3"/>
-        <v>2.595742875011168E-3</v>
+        <v>4.5425500312695436E-3</v>
       </c>
     </row>
     <row r="64" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7860,11 +7860,11 @@
       </c>
       <c r="D67" s="34">
         <f>'OPEX DATA 2'!U175</f>
-        <v>154.4084065934066</v>
+        <v>270.21471153846153</v>
       </c>
       <c r="E67" s="20">
         <f t="shared" si="3"/>
-        <v>2.5107057982667741E-3</v>
+        <v>4.3937351469668538E-3</v>
       </c>
     </row>
     <row r="68" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7874,11 +7874,11 @@
       </c>
       <c r="D68" s="34">
         <f>'OPEX DATA 2'!U176</f>
-        <v>147.91428571428574</v>
+        <v>258.85000000000002</v>
       </c>
       <c r="E68" s="20">
         <f t="shared" si="3"/>
-        <v>2.4051103368176543E-3</v>
+        <v>4.2089430894308947E-3</v>
       </c>
     </row>
     <row r="69" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7888,11 +7888,11 @@
       </c>
       <c r="D69" s="34">
         <f>'OPEX DATA 2'!U177</f>
-        <v>119.39230769230768</v>
+        <v>208.93653846153845</v>
       </c>
       <c r="E69" s="20">
         <f t="shared" si="3"/>
-        <v>1.9413383364602875E-3</v>
+        <v>3.3973420888055031E-3</v>
       </c>
     </row>
     <row r="70" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7902,11 +7902,11 @@
       </c>
       <c r="D70" s="34">
         <f>'OPEX DATA 2'!U178</f>
-        <v>169.7764285714286</v>
+        <v>297.10875000000004</v>
       </c>
       <c r="E70" s="20">
         <f t="shared" si="3"/>
-        <v>2.760592334494774E-3</v>
+        <v>4.8310365853658542E-3</v>
       </c>
     </row>
     <row r="71" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7916,11 +7916,11 @@
       </c>
       <c r="D71" s="34">
         <f>'OPEX DATA 2'!U179</f>
-        <v>56.898791208791202</v>
+        <v>99.572884615384609</v>
       </c>
       <c r="E71" s="20">
         <f t="shared" si="3"/>
-        <v>9.2518359689091386E-4</v>
+        <v>1.6190712945590993E-3</v>
       </c>
     </row>
     <row r="72" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7930,11 +7930,11 @@
       </c>
       <c r="D72" s="34">
         <f>'OPEX DATA 2'!U180</f>
-        <v>299.24170329670329</v>
+        <v>523.67298076923078</v>
       </c>
       <c r="E72" s="20">
         <f t="shared" si="3"/>
-        <v>4.8657187527919232E-3</v>
+        <v>8.5150078173858671E-3</v>
       </c>
     </row>
     <row r="73" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7958,11 +7958,11 @@
       </c>
       <c r="D74" s="34">
         <f>'OPEX DATA 2'!U182</f>
-        <v>2.1949999999999998</v>
+        <v>3.8412500000000001</v>
       </c>
       <c r="E74" s="20">
         <f t="shared" si="3"/>
-        <v>3.5691056910569106E-5</v>
+        <v>6.2459349593495936E-5</v>
       </c>
     </row>
     <row r="75" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7972,11 +7972,11 @@
       </c>
       <c r="D75" s="34">
         <f>'OPEX DATA 2'!U183</f>
-        <v>83.723791208791212</v>
+        <v>146.51663461538462</v>
       </c>
       <c r="E75" s="20">
         <f t="shared" si="3"/>
-        <v>1.3613624586795319E-3</v>
+        <v>2.382384302689181E-3</v>
       </c>
     </row>
     <row r="76" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7986,11 +7986,11 @@
       </c>
       <c r="D76" s="34">
         <f>'OPEX DATA 2'!U184</f>
-        <v>29.155659340659337</v>
+        <v>51.022403846153843</v>
       </c>
       <c r="E76" s="20">
         <f t="shared" si="3"/>
-        <v>4.740757616367372E-4</v>
+        <v>8.2963258286429011E-4</v>
       </c>
     </row>
     <row r="77" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8028,11 +8028,11 @@
       </c>
       <c r="D79" s="34">
         <f>'OPEX DATA 2'!U187</f>
-        <v>11.998406593406594</v>
+        <v>20.997211538461539</v>
       </c>
       <c r="E79" s="20">
         <f t="shared" si="3"/>
-        <v>1.9509604216921291E-4</v>
+        <v>3.414180737961226E-4</v>
       </c>
     </row>
     <row r="80" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8042,11 +8042,11 @@
       </c>
       <c r="D80" s="34">
         <f>'OPEX DATA 2'!U188</f>
-        <v>102.32258241758242</v>
+        <v>179.06451923076924</v>
       </c>
       <c r="E80" s="20">
         <f t="shared" si="3"/>
-        <v>1.6637818279281694E-3</v>
+        <v>2.9116181988742963E-3</v>
       </c>
     </row>
     <row r="81" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8056,11 +8056,11 @@
       </c>
       <c r="D81" s="34">
         <f>'OPEX DATA 2'!U189</f>
-        <v>170.5397802197802</v>
+        <v>298.44461538461536</v>
       </c>
       <c r="E81" s="20">
         <f t="shared" si="3"/>
-        <v>2.7730045564191902E-3</v>
+        <v>4.8527579737335834E-3</v>
       </c>
     </row>
     <row r="82" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8070,11 +8070,11 @@
       </c>
       <c r="D82" s="34">
         <f>'OPEX DATA 2'!U190</f>
-        <v>6.8321428571428573</v>
+        <v>11.956250000000001</v>
       </c>
       <c r="E82" s="20">
         <f t="shared" si="3"/>
-        <v>1.1109175377468061E-4</v>
+        <v>1.9441056910569107E-4</v>
       </c>
     </row>
     <row r="83" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8098,11 +8098,11 @@
       </c>
       <c r="D84" s="34">
         <f>'OPEX DATA 2'!U192</f>
-        <v>96.996098901098904</v>
+        <v>169.74317307692309</v>
       </c>
       <c r="E84" s="20">
         <f t="shared" si="3"/>
-        <v>1.5771723398552667E-3</v>
+        <v>2.7600515947467166E-3</v>
       </c>
     </row>
     <row r="85" spans="2:175" x14ac:dyDescent="0.25">
@@ -8113,11 +8113,11 @@
       <c r="C85" s="22"/>
       <c r="D85" s="45">
         <f>'OPEX DATA 2'!U193</f>
-        <v>709.21170329670326</v>
+        <v>1241.1204807692307</v>
       </c>
       <c r="E85" s="46">
         <f t="shared" si="3"/>
-        <v>1.153189761458054E-2</v>
+        <v>2.0180820825515946E-2</v>
       </c>
     </row>
     <row r="86" spans="2:175" x14ac:dyDescent="0.25">
@@ -8127,11 +8127,11 @@
       </c>
       <c r="D86" s="34">
         <f>'OPEX DATA 2'!U194</f>
-        <v>341.52368131868127</v>
+        <v>597.66644230769225</v>
       </c>
       <c r="E86" s="20">
         <f t="shared" si="3"/>
-        <v>5.553230590547663E-3</v>
+        <v>9.7181535334584113E-3</v>
       </c>
     </row>
     <row r="87" spans="2:175" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -8142,11 +8142,11 @@
       <c r="C87" s="2"/>
       <c r="D87" s="28">
         <f>'OPEX DATA 2'!U195</f>
-        <v>42.526263736263736</v>
+        <v>74.42096153846154</v>
       </c>
       <c r="E87" s="18">
         <f t="shared" si="3"/>
-        <v>6.9148396319128021E-4</v>
+        <v>1.2100969355847405E-3</v>
       </c>
       <c r="F87" s="18"/>
       <c r="G87" s="18"/>
@@ -8340,11 +8340,11 @@
       </c>
       <c r="D89" s="34">
         <f>'OPEX DATA 2'!U197</f>
-        <v>16.457582417582415</v>
+        <v>28.800769230769227</v>
       </c>
       <c r="E89" s="20">
         <f t="shared" si="3"/>
-        <v>2.6760296613955148E-4</v>
+        <v>4.6830519074421504E-4</v>
       </c>
     </row>
     <row r="90" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8396,11 +8396,11 @@
       </c>
       <c r="D93" s="34">
         <f>'OPEX DATA 2'!U201</f>
-        <v>15.443186813186813</v>
+        <v>27.025576923076922</v>
       </c>
       <c r="E93" s="20">
         <f t="shared" si="3"/>
-        <v>2.5110872866970427E-4</v>
+        <v>4.3944027517198246E-4</v>
       </c>
     </row>
     <row r="94" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8509,11 +8509,11 @@
       <c r="C101" s="48"/>
       <c r="D101" s="49">
         <f>SUM(D53:D100)</f>
-        <v>7809.9299450549461</v>
+        <v>10667.377403846154</v>
       </c>
       <c r="E101" s="50">
         <f t="shared" si="3"/>
-        <v>0.12699073081390155</v>
+        <v>0.17345329111944965</v>
       </c>
       <c r="F101" s="50"/>
       <c r="G101" s="50"/>
@@ -8536,11 +8536,11 @@
       </c>
       <c r="D104" s="34">
         <f>'OPEX DATA 2'!U215</f>
-        <v>1942.826978021978</v>
+        <v>3399.9472115384615</v>
       </c>
       <c r="E104" s="20">
         <f t="shared" ref="E104:E130" si="4">D104/D$36</f>
-        <v>3.1590682569463055E-2</v>
+        <v>5.528369449656035E-2</v>
       </c>
     </row>
     <row r="105" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8550,11 +8550,11 @@
       </c>
       <c r="D105" s="34">
         <f>'OPEX DATA 2'!U216</f>
-        <v>28.043956043956047</v>
+        <v>49.07692307692308</v>
       </c>
       <c r="E105" s="20">
         <f t="shared" si="4"/>
-        <v>4.5599928526757802E-4</v>
+        <v>7.979987492182615E-4</v>
       </c>
     </row>
     <row r="106" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8564,11 +8564,11 @@
       </c>
       <c r="D106" s="34">
         <f>'OPEX DATA 2'!U217</f>
-        <v>426.59027472527475</v>
+        <v>746.53298076923079</v>
       </c>
       <c r="E106" s="20">
         <f t="shared" si="4"/>
-        <v>6.9364272313052807E-3</v>
+        <v>1.2138747654784241E-2</v>
       </c>
     </row>
     <row r="107" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8578,11 +8578,11 @@
       </c>
       <c r="D107" s="34">
         <f>'OPEX DATA 2'!U218</f>
-        <v>34.25736263736264</v>
+        <v>59.950384615384614</v>
       </c>
       <c r="E107" s="20">
         <f t="shared" si="4"/>
-        <v>5.5703028678638438E-4</v>
+        <v>9.7480300187617261E-4</v>
       </c>
     </row>
     <row r="108" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8592,11 +8592,11 @@
       </c>
       <c r="D108" s="34">
         <f>'OPEX DATA 2'!U219</f>
-        <v>794.67241758241755</v>
+        <v>1390.6767307692307</v>
       </c>
       <c r="E108" s="20">
         <f t="shared" si="4"/>
-        <v>1.2921502724917358E-2</v>
+        <v>2.2612629768605379E-2</v>
       </c>
     </row>
     <row r="109" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8606,11 +8606,11 @@
       </c>
       <c r="D109" s="34">
         <f>'OPEX DATA 2'!U220</f>
-        <v>18.373186813186813</v>
+        <v>32.153076923076924</v>
       </c>
       <c r="E109" s="20">
         <f t="shared" si="4"/>
-        <v>2.9875100509246848E-4</v>
+        <v>5.2281425891181985E-4</v>
       </c>
     </row>
     <row r="110" spans="2:175" x14ac:dyDescent="0.25">
@@ -8635,11 +8635,11 @@
       </c>
       <c r="D111" s="34">
         <f>'OPEX DATA 2'!U222</f>
-        <v>8.797417582417582</v>
+        <v>15.395480769230769</v>
       </c>
       <c r="E111" s="20">
         <f t="shared" si="4"/>
-        <v>1.4304744036451353E-4</v>
+        <v>2.5033302063789866E-4</v>
       </c>
     </row>
     <row r="112" spans="2:175" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -8650,11 +8650,11 @@
       <c r="C112" s="2"/>
       <c r="D112" s="28">
         <f>'OPEX DATA 2'!U223</f>
-        <v>4.0824175824175822E-2</v>
+        <v>7.1442307692307694E-2</v>
       </c>
       <c r="E112" s="18">
         <f t="shared" si="4"/>
-        <v>6.6380773697846864E-7</v>
+        <v>1.1616635397123202E-6</v>
       </c>
       <c r="F112" s="18"/>
       <c r="G112" s="18"/>
@@ -8834,11 +8834,11 @@
       </c>
       <c r="D113" s="34">
         <f>'OPEX DATA 2'!U224</f>
-        <v>3.8060989010989013</v>
+        <v>6.6606730769230769</v>
       </c>
       <c r="E113" s="20">
         <f t="shared" si="4"/>
-        <v>6.1887787009738235E-5</v>
+        <v>1.0830362726704189E-4</v>
       </c>
     </row>
     <row r="114" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8862,11 +8862,11 @@
       </c>
       <c r="D115" s="34">
         <f>'OPEX DATA 2'!U226</f>
-        <v>-0.74967032967032965</v>
+        <v>-1.311923076923077</v>
       </c>
       <c r="E115" s="20">
         <f t="shared" si="4"/>
-        <v>-1.218976145805414E-5</v>
+        <v>-2.1332082551594746E-5</v>
       </c>
     </row>
     <row r="116" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8876,11 +8876,11 @@
       </c>
       <c r="D116" s="34">
         <f>'OPEX DATA 2'!U227</f>
-        <v>118.59192307692308</v>
+        <v>207.53586538461539</v>
       </c>
       <c r="E116" s="20">
         <f t="shared" si="4"/>
-        <v>1.9283239524702941E-3</v>
+        <v>3.3745669168230145E-3</v>
       </c>
     </row>
     <row r="117" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8890,11 +8890,11 @@
       </c>
       <c r="D117" s="34">
         <f>'OPEX DATA 2'!U228</f>
-        <v>24.308406593406595</v>
+        <v>42.539711538461539</v>
       </c>
       <c r="E117" s="20">
         <f t="shared" si="4"/>
-        <v>3.9525864379522921E-4</v>
+        <v>6.9170262664165099E-4</v>
       </c>
     </row>
     <row r="118" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8904,11 +8904,11 @@
       </c>
       <c r="D118" s="34">
         <f>'OPEX DATA 2'!U229</f>
-        <v>0.60989010989010983</v>
+        <v>1.0673076923076923</v>
       </c>
       <c r="E118" s="20">
         <f t="shared" si="4"/>
-        <v>9.9169123559367455E-6</v>
+        <v>1.7354596622889307E-5</v>
       </c>
     </row>
     <row r="119" spans="2:175" x14ac:dyDescent="0.25">
@@ -8919,11 +8919,11 @@
       <c r="C119" s="22"/>
       <c r="D119" s="45">
         <f>'OPEX DATA 2'!U230</f>
-        <v>81.932967032967028</v>
+        <v>143.38269230769231</v>
       </c>
       <c r="E119" s="46">
         <f t="shared" si="4"/>
-        <v>1.3322433663897077E-3</v>
+        <v>2.3314258911819887E-3</v>
       </c>
     </row>
     <row r="120" spans="2:175" x14ac:dyDescent="0.25">
@@ -8948,11 +8948,11 @@
       <c r="C121" s="2"/>
       <c r="D121" s="28">
         <f>'OPEX DATA 2'!U232</f>
-        <v>2.7472527472527473</v>
+        <v>4.8076923076923075</v>
       </c>
       <c r="E121" s="18">
         <f t="shared" si="4"/>
-        <v>4.4670776378093451E-5</v>
+        <v>7.817385866166354E-5</v>
       </c>
       <c r="F121" s="18"/>
       <c r="G121" s="18"/>
@@ -9133,11 +9133,11 @@
       <c r="C122" s="22"/>
       <c r="D122" s="45">
         <f>'OPEX DATA 2'!U233</f>
-        <v>0.50230769230769234</v>
+        <v>0.87903846153846155</v>
       </c>
       <c r="E122" s="46">
         <f t="shared" si="4"/>
-        <v>8.1676047529706064E-6</v>
+        <v>1.4293308317698561E-5</v>
       </c>
     </row>
     <row r="123" spans="2:175" x14ac:dyDescent="0.25">
@@ -9147,11 +9147,11 @@
       </c>
       <c r="D123" s="34">
         <f>'OPEX DATA 2'!U234</f>
-        <v>4.3490659340659343</v>
+        <v>7.6108653846153844</v>
       </c>
       <c r="E123" s="20">
         <f t="shared" si="4"/>
-        <v>7.0716519253104617E-5</v>
+        <v>1.2375390869293309E-4</v>
       </c>
     </row>
     <row r="124" spans="2:175" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -9162,11 +9162,11 @@
       <c r="C124" s="2"/>
       <c r="D124" s="28">
         <f>'OPEX DATA 2'!U235</f>
-        <v>35.93796703296703</v>
+        <v>62.891442307692309</v>
       </c>
       <c r="E124" s="18">
         <f t="shared" si="4"/>
-        <v>5.8435718752791917E-4</v>
+        <v>1.0226250781738588E-3</v>
       </c>
       <c r="F124" s="18"/>
       <c r="G124" s="18"/>
@@ -9346,11 +9346,11 @@
       </c>
       <c r="D125" s="34">
         <f>'OPEX DATA 2'!U236</f>
-        <v>1125.1606043956044</v>
+        <v>1969.0310576923077</v>
       </c>
       <c r="E125" s="20">
         <f t="shared" si="4"/>
-        <v>1.8295294380416331E-2</v>
+        <v>3.2016765165728579E-2</v>
       </c>
     </row>
     <row r="126" spans="2:175" x14ac:dyDescent="0.25">
@@ -9361,11 +9361,11 @@
       <c r="C126" s="22"/>
       <c r="D126" s="45">
         <f>'OPEX DATA 2'!U237</f>
-        <v>81.332197802197811</v>
+        <v>142.33134615384617</v>
       </c>
       <c r="E126" s="46">
         <f t="shared" si="4"/>
-        <v>1.3224747610113465E-3</v>
+        <v>2.3143308317698564E-3</v>
       </c>
     </row>
     <row r="127" spans="2:175" x14ac:dyDescent="0.25">
@@ -9375,11 +9375,11 @@
       </c>
       <c r="D127" s="34">
         <f>'OPEX DATA 2'!U238</f>
-        <v>11.850494505494506</v>
+        <v>20.738365384615385</v>
       </c>
       <c r="E127" s="20">
         <f t="shared" si="4"/>
-        <v>1.9269096756901636E-4</v>
+        <v>3.3720919324577864E-4</v>
       </c>
     </row>
     <row r="128" spans="2:175" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -9589,11 +9589,11 @@
       <c r="C130" s="48"/>
       <c r="D130" s="49">
         <f>SUM(D104:D129)</f>
-        <v>4743.9819230769235</v>
+        <v>8301.9683653846132</v>
       </c>
       <c r="E130" s="50">
         <f t="shared" si="4"/>
-        <v>7.7137917448405258E-2</v>
+        <v>0.13499135553470915</v>
       </c>
       <c r="F130" s="50"/>
       <c r="G130" s="50"/>
@@ -9616,11 +9616,11 @@
       </c>
       <c r="D133" s="34">
         <f>'OPEX DATA 2'!U244</f>
-        <v>20.959285714285709</v>
+        <v>36.678749999999994</v>
       </c>
       <c r="E133" s="20">
         <f t="shared" ref="E133:E141" si="5">D133/D$36</f>
-        <v>3.4080139372822294E-4</v>
+        <v>5.9640243902439019E-4</v>
       </c>
     </row>
     <row r="134" spans="2:7" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -9630,11 +9630,11 @@
       </c>
       <c r="D134" s="34">
         <f>'OPEX DATA 2'!U245</f>
-        <v>15.025109890109889</v>
+        <v>26.293942307692305</v>
       </c>
       <c r="E134" s="20">
         <f t="shared" si="5"/>
-        <v>2.44310729920486E-4</v>
+        <v>4.275437773608505E-4</v>
       </c>
     </row>
     <row r="135" spans="2:7" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -9658,11 +9658,11 @@
       </c>
       <c r="D136" s="34">
         <f>'OPEX DATA 2'!U247</f>
-        <v>144.80395604395605</v>
+        <v>253.40692307692308</v>
       </c>
       <c r="E136" s="20">
         <f t="shared" si="5"/>
-        <v>2.3545358706334317E-3</v>
+        <v>4.1204377736085056E-3</v>
       </c>
     </row>
     <row r="137" spans="2:7" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -9672,11 +9672,11 @@
       </c>
       <c r="D137" s="34">
         <f>'OPEX DATA 2'!U248</f>
-        <v>24.860439560439563</v>
+        <v>43.505769230769232</v>
       </c>
       <c r="E137" s="20">
         <f t="shared" si="5"/>
-        <v>4.0423478960064328E-4</v>
+        <v>7.0741088180112572E-4</v>
       </c>
     </row>
     <row r="138" spans="2:7" x14ac:dyDescent="0.25">
@@ -9687,11 +9687,11 @@
       <c r="C138" s="22"/>
       <c r="D138" s="45">
         <f>'OPEX DATA 2'!U249</f>
-        <v>155.47115384615384</v>
+        <v>272.07451923076923</v>
       </c>
       <c r="E138" s="46">
         <f t="shared" si="5"/>
-        <v>2.5279862414008753E-3</v>
+        <v>4.423975922451532E-3</v>
       </c>
     </row>
     <row r="139" spans="2:7" x14ac:dyDescent="0.25">
@@ -9731,11 +9731,11 @@
       <c r="C141" s="48"/>
       <c r="D141" s="49">
         <f>SUM(D133:D140)</f>
-        <v>361.11994505494505</v>
+        <v>631.95990384615379</v>
       </c>
       <c r="E141" s="50">
         <f t="shared" si="5"/>
-        <v>5.8718690252836598E-3</v>
+        <v>1.0275770794246403E-2</v>
       </c>
       <c r="F141" s="50"/>
       <c r="G141" s="50"/>
@@ -9778,11 +9778,11 @@
       <c r="C145" s="56"/>
       <c r="D145" s="57">
         <f>'OPEX DATA 2'!U256</f>
-        <v>2508.1870329670332</v>
+        <v>4389.3273076923078</v>
       </c>
       <c r="E145" s="58">
         <f t="shared" si="6"/>
-        <v>4.0783528991333876E-2</v>
+        <v>7.1371175734834272E-2</v>
       </c>
     </row>
     <row r="146" spans="2:7" x14ac:dyDescent="0.25">
@@ -9808,11 +9808,11 @@
       <c r="C147" s="56"/>
       <c r="D147" s="57">
         <f>'OPEX DATA 2'!U258</f>
-        <v>126.06516483516484</v>
+        <v>220.61403846153846</v>
       </c>
       <c r="E147" s="58">
         <f t="shared" si="6"/>
-        <v>2.0498400786205665E-3</v>
+        <v>3.5872201375859911E-3</v>
       </c>
     </row>
     <row r="148" spans="2:7" x14ac:dyDescent="0.25">
@@ -9853,11 +9853,11 @@
       <c r="C150" s="56"/>
       <c r="D150" s="57">
         <f>'OPEX DATA 2'!U261</f>
-        <v>831.8067582417583</v>
+        <v>1455.6618269230771</v>
       </c>
       <c r="E150" s="58">
         <f t="shared" si="6"/>
-        <v>1.3525313142142411E-2</v>
+        <v>2.3669297998749221E-2</v>
       </c>
     </row>
     <row r="151" spans="2:7" x14ac:dyDescent="0.25">
@@ -9868,11 +9868,11 @@
       <c r="C151" s="56"/>
       <c r="D151" s="57">
         <f>'OPEX DATA 2'!U262</f>
-        <v>308.97318681318677</v>
+        <v>540.70307692307688</v>
       </c>
       <c r="E151" s="58">
         <f t="shared" si="6"/>
-        <v>5.0239542571249886E-3</v>
+        <v>8.7919199499687292E-3</v>
       </c>
     </row>
     <row r="152" spans="2:7" x14ac:dyDescent="0.25">
@@ -9883,11 +9883,11 @@
       <c r="C152" s="48"/>
       <c r="D152" s="49">
         <f>SUM(D144:D151)</f>
-        <v>3775.0321428571433</v>
+        <v>6606.3062499999996</v>
       </c>
       <c r="E152" s="50">
         <f t="shared" si="6"/>
-        <v>6.1382636469221839E-2</v>
+        <v>0.10741961382113821</v>
       </c>
       <c r="F152" s="50"/>
       <c r="G152" s="50"/>
@@ -9945,11 +9945,11 @@
       <c r="C157" s="56"/>
       <c r="D157" s="57">
         <f>'OPEX DATA 2'!U268</f>
-        <v>-0.18175824175824173</v>
+        <v>-0.31807692307692303</v>
       </c>
       <c r="E157" s="58">
         <f t="shared" si="7"/>
-        <v>-2.9554185651746624E-6</v>
+        <v>-5.1719824890556595E-6</v>
       </c>
     </row>
     <row r="158" spans="2:7" x14ac:dyDescent="0.25">
@@ -10095,11 +10095,11 @@
       <c r="C167" s="56"/>
       <c r="D167" s="57">
         <f>'OPEX DATA 2'!U278</f>
-        <v>-2284.8806593406593</v>
+        <v>-3998.541153846154</v>
       </c>
       <c r="E167" s="58">
         <f t="shared" si="7"/>
-        <v>-3.7152531046189582E-2</v>
+        <v>-6.5016929330831766E-2</v>
       </c>
     </row>
     <row r="168" spans="2:7" x14ac:dyDescent="0.25">
@@ -10170,11 +10170,11 @@
       <c r="C172" s="48"/>
       <c r="D172" s="49">
         <f>SUM(D155:D171)</f>
-        <v>-2285.0624175824178</v>
+        <v>-3998.8592307692311</v>
       </c>
       <c r="E172" s="50">
         <f t="shared" si="7"/>
-        <v>-3.7155486464754757E-2</v>
+        <v>-6.5022101313320826E-2</v>
       </c>
       <c r="F172" s="50"/>
       <c r="G172" s="50"/>
@@ -10217,11 +10217,11 @@
       <c r="C176" s="56"/>
       <c r="D176" s="57">
         <f>'OPEX DATA 2'!U289</f>
-        <v>377.30285714285714</v>
+        <v>660.28</v>
       </c>
       <c r="E176" s="58">
         <f t="shared" si="8"/>
-        <v>6.1350058072009292E-3</v>
+        <v>1.0736260162601626E-2</v>
       </c>
     </row>
     <row r="177" spans="2:5" x14ac:dyDescent="0.25">
@@ -10232,11 +10232,11 @@
       <c r="C177" s="56"/>
       <c r="D177" s="57">
         <f>'OPEX DATA 2'!U290</f>
-        <v>3246.9006043956042</v>
+        <v>5682.0760576923076</v>
       </c>
       <c r="E177" s="58">
         <f t="shared" si="8"/>
-        <v>5.2795131778790312E-2</v>
+        <v>9.2391480612883048E-2</v>
       </c>
     </row>
     <row r="178" spans="2:5" x14ac:dyDescent="0.25">
@@ -10247,11 +10247,11 @@
       <c r="C178" s="56"/>
       <c r="D178" s="57">
         <f>'OPEX DATA 2'!U291</f>
-        <v>0.40659340659340659</v>
+        <v>0.71153846153846156</v>
       </c>
       <c r="E178" s="58">
         <f t="shared" si="8"/>
-        <v>6.6112749039578306E-6</v>
+        <v>1.1569731081926204E-5</v>
       </c>
     </row>
     <row r="179" spans="2:5" x14ac:dyDescent="0.25">
@@ -10262,11 +10262,11 @@
       <c r="C179" s="56"/>
       <c r="D179" s="57">
         <f>'OPEX DATA 2'!U292</f>
-        <v>86.494505494505489</v>
+        <v>151.36538461538461</v>
       </c>
       <c r="E179" s="58">
         <f t="shared" si="8"/>
-        <v>1.4064147234878941E-3</v>
+        <v>2.461225766103815E-3</v>
       </c>
     </row>
     <row r="180" spans="2:5" x14ac:dyDescent="0.25">
@@ -10277,11 +10277,11 @@
       <c r="C180" s="56"/>
       <c r="D180" s="57">
         <f>'OPEX DATA 2'!U293</f>
-        <v>8.3655494505494499</v>
+        <v>14.639711538461539</v>
       </c>
       <c r="E180" s="58">
         <f t="shared" si="8"/>
-        <v>1.3602519431787723E-4</v>
+        <v>2.3804409005628518E-4</v>
       </c>
     </row>
     <row r="181" spans="2:5" x14ac:dyDescent="0.25">
@@ -10292,11 +10292,11 @@
       <c r="C181" s="56"/>
       <c r="D181" s="57">
         <f>'OPEX DATA 2'!U294</f>
-        <v>218.10131868131865</v>
+        <v>381.67730769230764</v>
       </c>
       <c r="E181" s="58">
         <f t="shared" si="8"/>
-        <v>3.546362905387295E-3</v>
+        <v>6.2061350844277666E-3</v>
       </c>
     </row>
     <row r="182" spans="2:5" x14ac:dyDescent="0.25">
@@ -10337,11 +10337,11 @@
       <c r="C184" s="56"/>
       <c r="D184" s="57">
         <f>'OPEX DATA 2'!U297</f>
-        <v>2.6509890109890111</v>
+        <v>4.6392307692307693</v>
       </c>
       <c r="E184" s="58">
         <f t="shared" si="8"/>
-        <v>4.3105512373805061E-5</v>
+        <v>7.5434646654158846E-5</v>
       </c>
     </row>
     <row r="185" spans="2:5" x14ac:dyDescent="0.25">
@@ -10592,11 +10592,11 @@
       <c r="C201" s="48"/>
       <c r="D201" s="49">
         <f>SUM(D175:D200)</f>
-        <v>3940.2224175824176</v>
+        <v>6895.3892307692295</v>
       </c>
       <c r="E201" s="50">
         <f t="shared" si="8"/>
-        <v>6.406865719646207E-2</v>
+        <v>0.11212015009380862</v>
       </c>
       <c r="F201" s="50"/>
       <c r="G201" s="50"/>
@@ -10614,11 +10614,11 @@
       <c r="C203" s="48"/>
       <c r="D203" s="49">
         <f>D43-D50-D101-D130-D141-D152-D172-D201</f>
-        <v>19887.730054945059</v>
+        <v>640.6150961538533</v>
       </c>
       <c r="E203" s="50">
         <f>D203/D36</f>
-        <v>0.32337772447065138</v>
+        <v>1.041650562851794E-2</v>
       </c>
       <c r="F203" s="50"/>
       <c r="G203" s="50"/>
@@ -10644,7 +10644,7 @@
       <c r="C207" s="63"/>
       <c r="D207" s="64">
         <f>E203</f>
-        <v>0.32337772447065138</v>
+        <v>1.041650562851794E-2</v>
       </c>
     </row>
     <row r="208" spans="2:175" s="20" customFormat="1" x14ac:dyDescent="0.25">
@@ -18403,6 +18403,7 @@
     <col min="18" max="18" width="8.25" customWidth="1"/>
     <col min="20" max="20" width="12.75" customWidth="1"/>
     <col min="21" max="21" width="18.375" customWidth="1"/>
+    <col min="23" max="23" width="24.625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.25">
@@ -18578,8 +18579,8 @@
         <v>3118509.06</v>
       </c>
       <c r="U8" s="80">
-        <f>(T8/$V$1)/7</f>
-        <v>17134.665164835165</v>
+        <f>(T8/$V$1)/4</f>
+        <v>29985.664038461538</v>
       </c>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.25">
@@ -18638,7 +18639,7 @@
         <v>0</v>
       </c>
       <c r="U9" s="80">
-        <f t="shared" ref="U9:U72" si="1">(T9/$V$1)/7</f>
+        <f t="shared" ref="U9:U72" si="1">(T9/$V$1)/4</f>
         <v>0</v>
       </c>
       <c r="W9">
@@ -18709,7 +18710,7 @@
       </c>
       <c r="U10" s="80">
         <f t="shared" si="1"/>
-        <v>17134.665164835165</v>
+        <v>29985.664038461538</v>
       </c>
       <c r="W10">
         <f>W9*2</f>
@@ -18773,7 +18774,7 @@
       </c>
       <c r="U11" s="80">
         <f t="shared" si="1"/>
-        <v>2024.687032967033</v>
+        <v>3543.2023076923078</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -18923,7 +18924,7 @@
       </c>
       <c r="U14" s="80">
         <f t="shared" si="1"/>
-        <v>29826.415989010991</v>
+        <v>52196.227980769232</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
@@ -18983,7 +18984,7 @@
       </c>
       <c r="U15" s="80">
         <f t="shared" si="1"/>
-        <v>297.74175824175825</v>
+        <v>521.04807692307691</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
@@ -19043,7 +19044,7 @@
       </c>
       <c r="U16" s="80">
         <f t="shared" si="1"/>
-        <v>6838.2967032967035</v>
+        <v>11967.01923076923</v>
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
@@ -19103,7 +19104,7 @@
       </c>
       <c r="U17" s="80">
         <f t="shared" si="1"/>
-        <v>1401.9230769230769</v>
+        <v>2453.3653846153848</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
@@ -19163,7 +19164,7 @@
       </c>
       <c r="U18" s="80">
         <f t="shared" si="1"/>
-        <v>3094.3406593406594</v>
+        <v>5415.0961538461543</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
@@ -19229,7 +19230,7 @@
       </c>
       <c r="U19" s="80">
         <f t="shared" si="1"/>
-        <v>41458.718186813188</v>
+        <v>72552.756826923083</v>
       </c>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
@@ -19379,7 +19380,7 @@
       </c>
       <c r="U22" s="80">
         <f t="shared" si="1"/>
-        <v>1173.4599999999998</v>
+        <v>2053.5549999999998</v>
       </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
@@ -19439,7 +19440,7 @@
       </c>
       <c r="U23" s="80">
         <f t="shared" si="1"/>
-        <v>-1.1868131868131868</v>
+        <v>-2.0769230769230771</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
@@ -19619,7 +19620,7 @@
       </c>
       <c r="U26" s="80">
         <f t="shared" si="1"/>
-        <v>3147.6684065934064</v>
+        <v>5508.4197115384613</v>
       </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
@@ -19865,7 +19866,7 @@
       </c>
       <c r="U30" s="80">
         <f t="shared" si="1"/>
-        <v>4319.9415934065937</v>
+        <v>7559.8977884615388</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
@@ -20411,7 +20412,7 @@
       </c>
       <c r="U40" s="80">
         <f t="shared" si="1"/>
-        <v>-1.7664835164835164</v>
+        <v>-3.0913461538461537</v>
       </c>
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
@@ -20471,7 +20472,7 @@
       </c>
       <c r="U41" s="80">
         <f t="shared" si="1"/>
-        <v>-66.608791208791203</v>
+        <v>-116.5653846153846</v>
       </c>
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
@@ -20531,7 +20532,7 @@
       </c>
       <c r="U42" s="80">
         <f t="shared" si="1"/>
-        <v>-182.2010989010989</v>
+        <v>-318.85192307692307</v>
       </c>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
@@ -20591,7 +20592,7 @@
       </c>
       <c r="U43" s="80">
         <f t="shared" si="1"/>
-        <v>-710.49450549450546</v>
+        <v>-1243.3653846153845</v>
       </c>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
@@ -20651,7 +20652,7 @@
       </c>
       <c r="U44" s="80">
         <f t="shared" si="1"/>
-        <v>-14.840659340659341</v>
+        <v>-25.971153846153847</v>
       </c>
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
@@ -20774,7 +20775,7 @@
       </c>
       <c r="U46" s="80">
         <f t="shared" si="1"/>
-        <v>-711.1704945054945</v>
+        <v>-1244.5483653846154</v>
       </c>
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
@@ -20834,7 +20835,7 @@
       </c>
       <c r="U47" s="80">
         <f t="shared" si="1"/>
-        <v>-156.07967032967034</v>
+        <v>-273.13942307692309</v>
       </c>
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
@@ -20894,7 +20895,7 @@
       </c>
       <c r="U48" s="80">
         <f t="shared" si="1"/>
-        <v>-127.13186813186813</v>
+        <v>-222.48076923076923</v>
       </c>
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
@@ -20954,7 +20955,7 @@
       </c>
       <c r="U49" s="80">
         <f t="shared" si="1"/>
-        <v>-14.615384615384615</v>
+        <v>-25.576923076923077</v>
       </c>
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
@@ -21017,7 +21018,7 @@
       </c>
       <c r="U50" s="80">
         <f t="shared" si="1"/>
-        <v>-100.13406593406594</v>
+        <v>-175.23461538461541</v>
       </c>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
@@ -21083,7 +21084,7 @@
       </c>
       <c r="U51" s="80">
         <f t="shared" si="1"/>
-        <v>-2085.0430219780219</v>
+        <v>-3648.8252884615381</v>
       </c>
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
@@ -21149,7 +21150,7 @@
       </c>
       <c r="U52" s="80">
         <f t="shared" si="1"/>
-        <v>62852.968956043951</v>
+        <v>109992.69567307692</v>
       </c>
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
@@ -21329,7 +21330,7 @@
       </c>
       <c r="U56" s="80">
         <f t="shared" si="1"/>
-        <v>373.78736263736266</v>
+        <v>654.12788461538469</v>
       </c>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
@@ -21389,7 +21390,7 @@
       </c>
       <c r="U57" s="80">
         <f t="shared" si="1"/>
-        <v>93.62813186813186</v>
+        <v>163.84923076923076</v>
       </c>
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
@@ -21449,7 +21450,7 @@
       </c>
       <c r="U58" s="80">
         <f t="shared" si="1"/>
-        <v>1177.9847252747254</v>
+        <v>2061.4732692307693</v>
       </c>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
@@ -21509,7 +21510,7 @@
       </c>
       <c r="U59" s="80">
         <f t="shared" si="1"/>
-        <v>70.116868131868131</v>
+        <v>122.70451923076924</v>
       </c>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
@@ -21569,7 +21570,7 @@
       </c>
       <c r="U60" s="80">
         <f t="shared" si="1"/>
-        <v>1802.2785714285715</v>
+        <v>3153.9875000000002</v>
       </c>
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
@@ -21629,7 +21630,7 @@
       </c>
       <c r="U61" s="80">
         <f t="shared" si="1"/>
-        <v>309.48340659340658</v>
+        <v>541.59596153846155</v>
       </c>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
@@ -21689,7 +21690,7 @@
       </c>
       <c r="U62" s="80">
         <f t="shared" si="1"/>
-        <v>4.525439560439561</v>
+        <v>7.9195192307692315</v>
       </c>
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
@@ -21749,7 +21750,7 @@
       </c>
       <c r="U63" s="80">
         <f t="shared" si="1"/>
-        <v>149.89934065934068</v>
+        <v>262.3238461538462</v>
       </c>
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
@@ -21875,7 +21876,7 @@
       </c>
       <c r="U65" s="80">
         <f t="shared" si="1"/>
-        <v>3981.7038461538459</v>
+        <v>6967.9817307692301</v>
       </c>
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
@@ -21935,7 +21936,7 @@
       </c>
       <c r="U66" s="80">
         <f t="shared" si="1"/>
-        <v>465.02543956043945</v>
+        <v>813.79451923076908</v>
       </c>
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
@@ -22085,7 +22086,7 @@
       </c>
       <c r="U69" s="80">
         <f t="shared" si="1"/>
-        <v>46.058186813186815</v>
+        <v>80.601826923076928</v>
       </c>
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
@@ -22145,7 +22146,7 @@
       </c>
       <c r="U70" s="80">
         <f t="shared" si="1"/>
-        <v>196.94489010989011</v>
+        <v>344.65355769230769</v>
       </c>
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
@@ -22205,7 +22206,7 @@
       </c>
       <c r="U71" s="80">
         <f t="shared" si="1"/>
-        <v>2739.2541758241759</v>
+        <v>4793.6948076923081</v>
       </c>
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
@@ -22324,8 +22325,8 @@
         <v>526298.73</v>
       </c>
       <c r="U73" s="80">
-        <f t="shared" ref="U73:U136" si="3">(T73/$V$1)/7</f>
-        <v>2891.7512637362638</v>
+        <f t="shared" ref="U73:U136" si="3">(T73/$V$1)/4</f>
+        <v>5060.5647115384618</v>
       </c>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
@@ -22445,7 +22446,7 @@
       </c>
       <c r="U75" s="80">
         <f t="shared" si="3"/>
-        <v>216.86538461538461</v>
+        <v>379.51442307692309</v>
       </c>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
@@ -22511,7 +22512,7 @@
       </c>
       <c r="U76" s="80">
         <f t="shared" si="3"/>
-        <v>6090.8739010989011</v>
+        <v>10659.029326923077</v>
       </c>
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
@@ -22967,7 +22968,7 @@
       </c>
       <c r="U85" s="80">
         <f t="shared" si="3"/>
-        <v>803.83225274725271</v>
+        <v>1406.7064423076922</v>
       </c>
     </row>
     <row r="86" spans="1:21" x14ac:dyDescent="0.25">
@@ -23027,7 +23028,7 @@
       </c>
       <c r="U86" s="80">
         <f t="shared" si="3"/>
-        <v>208.74379120879118</v>
+        <v>365.30163461538456</v>
       </c>
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
@@ -23087,7 +23088,7 @@
       </c>
       <c r="U87" s="80">
         <f t="shared" si="3"/>
-        <v>106.55549450549449</v>
+        <v>186.47211538461536</v>
       </c>
     </row>
     <row r="88" spans="1:21" x14ac:dyDescent="0.25">
@@ -23147,7 +23148,7 @@
       </c>
       <c r="U88" s="80">
         <f t="shared" si="3"/>
-        <v>781.14406593406591</v>
+        <v>1367.0021153846153</v>
       </c>
     </row>
     <row r="89" spans="1:21" x14ac:dyDescent="0.25">
@@ -23207,7 +23208,7 @@
       </c>
       <c r="U89" s="80">
         <f t="shared" si="3"/>
-        <v>6.0676923076923073</v>
+        <v>10.618461538461538</v>
       </c>
     </row>
     <row r="90" spans="1:21" x14ac:dyDescent="0.25">
@@ -23387,7 +23388,7 @@
       </c>
       <c r="U92" s="80">
         <f t="shared" si="3"/>
-        <v>368.4400549450549</v>
+        <v>644.77009615384611</v>
       </c>
     </row>
     <row r="93" spans="1:21" x14ac:dyDescent="0.25">
@@ -23627,7 +23628,7 @@
       </c>
       <c r="U96" s="80">
         <f t="shared" si="3"/>
-        <v>38.46153846153846</v>
+        <v>67.307692307692307</v>
       </c>
     </row>
     <row r="97" spans="1:21" x14ac:dyDescent="0.25">
@@ -23687,7 +23688,7 @@
       </c>
       <c r="U97" s="80">
         <f t="shared" si="3"/>
-        <v>282.50153846153847</v>
+        <v>494.37769230769231</v>
       </c>
     </row>
     <row r="98" spans="1:21" x14ac:dyDescent="0.25">
@@ -23747,7 +23748,7 @@
       </c>
       <c r="U98" s="80">
         <f t="shared" si="3"/>
-        <v>233.49582417582414</v>
+        <v>408.61769230769227</v>
       </c>
     </row>
     <row r="99" spans="1:21" x14ac:dyDescent="0.25">
@@ -24467,7 +24468,7 @@
       </c>
       <c r="U110" s="80">
         <f t="shared" si="3"/>
-        <v>311.44593406593401</v>
+        <v>545.03038461538449</v>
       </c>
     </row>
     <row r="111" spans="1:21" x14ac:dyDescent="0.25">
@@ -24587,10 +24588,10 @@
       </c>
       <c r="U112" s="80">
         <f t="shared" si="3"/>
-        <v>189.75032967032965</v>
-      </c>
-    </row>
-    <row r="113" spans="1:21" x14ac:dyDescent="0.25">
+        <v>332.06307692307689</v>
+      </c>
+    </row>
+    <row r="113" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A113" s="87" t="s">
         <v>141</v>
       </c>
@@ -24650,7 +24651,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A114" s="87" t="s">
         <v>142</v>
       </c>
@@ -24707,10 +24708,10 @@
       </c>
       <c r="U114" s="80">
         <f t="shared" si="3"/>
-        <v>8.497417582417583</v>
-      </c>
-    </row>
-    <row r="115" spans="1:21" x14ac:dyDescent="0.25">
+        <v>14.87048076923077</v>
+      </c>
+    </row>
+    <row r="115" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A115" s="87" t="s">
         <v>143</v>
       </c>
@@ -24770,7 +24771,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A116" s="87" t="s">
         <v>144</v>
       </c>
@@ -24830,7 +24831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A117" s="87" t="s">
         <v>145</v>
       </c>
@@ -24890,7 +24891,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A118" s="87" t="s">
         <v>146</v>
       </c>
@@ -24947,10 +24948,10 @@
       </c>
       <c r="U118" s="80">
         <f t="shared" si="3"/>
-        <v>15.373351648351647</v>
-      </c>
-    </row>
-    <row r="119" spans="1:21" x14ac:dyDescent="0.25">
+        <v>26.903365384615384</v>
+      </c>
+    </row>
+    <row r="119" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A119" s="88" t="s">
         <v>147</v>
       </c>
@@ -25013,10 +25014,10 @@
       </c>
       <c r="U119" s="80">
         <f t="shared" si="3"/>
-        <v>3354.3092857142851</v>
-      </c>
-    </row>
-    <row r="120" spans="1:21" x14ac:dyDescent="0.25">
+        <v>5870.0412499999993</v>
+      </c>
+    </row>
+    <row r="120" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A120" s="81" t="s">
         <v>26</v>
       </c>
@@ -25074,15 +25075,19 @@
         <v>5.9013441202604079E-2</v>
       </c>
       <c r="T120" s="80">
-        <f t="shared" si="2"/>
+        <f>IFERROR(B120+E120+H120+K120+N120+Q120, "NA")</f>
         <v>610484.28999999992</v>
       </c>
       <c r="U120" s="80">
         <f t="shared" si="3"/>
-        <v>3354.3092857142851</v>
-      </c>
-    </row>
-    <row r="121" spans="1:21" x14ac:dyDescent="0.25">
+        <v>5870.0412499999993</v>
+      </c>
+      <c r="W120" s="80">
+        <f>U120+U143+U151</f>
+        <v>19039.900576923079</v>
+      </c>
+    </row>
+    <row r="121" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A121" s="75" t="s">
         <v>148</v>
       </c>
@@ -25112,7 +25117,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A122" s="76" t="s">
         <v>149</v>
       </c>
@@ -25172,7 +25177,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A123" s="76" t="s">
         <v>150</v>
       </c>
@@ -25229,10 +25234,10 @@
       </c>
       <c r="U123" s="80">
         <f t="shared" si="3"/>
-        <v>406.30549450549449</v>
-      </c>
-    </row>
-    <row r="124" spans="1:21" x14ac:dyDescent="0.25">
+        <v>711.03461538461534</v>
+      </c>
+    </row>
+    <row r="124" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A124" s="76" t="s">
         <v>151</v>
       </c>
@@ -25289,10 +25294,10 @@
       </c>
       <c r="U124" s="80">
         <f t="shared" si="3"/>
-        <v>780.64219780219787</v>
-      </c>
-    </row>
-    <row r="125" spans="1:21" ht="31.5" x14ac:dyDescent="0.25">
+        <v>1366.1238461538462</v>
+      </c>
+    </row>
+    <row r="125" spans="1:23" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A125" s="76" t="s">
         <v>152</v>
       </c>
@@ -25352,7 +25357,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A126" s="76" t="s">
         <v>153</v>
       </c>
@@ -25412,7 +25417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A127" s="76" t="s">
         <v>154</v>
       </c>
@@ -25472,7 +25477,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A128" s="76" t="s">
         <v>155</v>
       </c>
@@ -25649,7 +25654,7 @@
       </c>
       <c r="U130" s="80">
         <f t="shared" si="3"/>
-        <v>-44.164835164835161</v>
+        <v>-77.288461538461533</v>
       </c>
     </row>
     <row r="131" spans="1:21" x14ac:dyDescent="0.25">
@@ -26068,7 +26073,7 @@
         <v>0</v>
       </c>
       <c r="U137" s="80">
-        <f t="shared" ref="U137:U200" si="5">(T137/$V$1)/7</f>
+        <f t="shared" ref="U137:U200" si="5">(T137/$V$1)/4</f>
         <v>0</v>
       </c>
     </row>
@@ -26189,7 +26194,7 @@
       </c>
       <c r="U139" s="80">
         <f t="shared" si="5"/>
-        <v>2422.6123076923077</v>
+        <v>4239.5715384615387</v>
       </c>
     </row>
     <row r="140" spans="1:21" x14ac:dyDescent="0.25">
@@ -26309,7 +26314,7 @@
       </c>
       <c r="U141" s="80">
         <f t="shared" si="5"/>
-        <v>1353.3757692307693</v>
+        <v>2368.407596153846</v>
       </c>
     </row>
     <row r="142" spans="1:21" x14ac:dyDescent="0.25">
@@ -26369,7 +26374,7 @@
       </c>
       <c r="U142" s="80">
         <f t="shared" si="5"/>
-        <v>568.76373626373629</v>
+        <v>995.33653846153845</v>
       </c>
     </row>
     <row r="143" spans="1:21" x14ac:dyDescent="0.25">
@@ -26435,7 +26440,7 @@
       </c>
       <c r="U143" s="80">
         <f t="shared" si="5"/>
-        <v>5487.53467032967</v>
+        <v>9603.1856730769232</v>
       </c>
     </row>
     <row r="144" spans="1:21" x14ac:dyDescent="0.25">
@@ -26585,7 +26590,7 @@
       </c>
       <c r="U146" s="80">
         <f t="shared" si="5"/>
-        <v>1169.0604945054945</v>
+        <v>2045.8558653846153</v>
       </c>
     </row>
     <row r="147" spans="1:21" x14ac:dyDescent="0.25">
@@ -26645,7 +26650,7 @@
       </c>
       <c r="U147" s="80">
         <f t="shared" si="5"/>
-        <v>209.66851648351647</v>
+        <v>366.91990384615383</v>
       </c>
     </row>
     <row r="148" spans="1:21" x14ac:dyDescent="0.25">
@@ -26705,7 +26710,7 @@
       </c>
       <c r="U148" s="80">
         <f t="shared" si="5"/>
-        <v>145.23280219780222</v>
+        <v>254.15740384615387</v>
       </c>
     </row>
     <row r="149" spans="1:21" x14ac:dyDescent="0.25">
@@ -26765,7 +26770,7 @@
       </c>
       <c r="U149" s="80">
         <f t="shared" si="5"/>
-        <v>167.74725274725276</v>
+        <v>293.55769230769232</v>
       </c>
     </row>
     <row r="150" spans="1:21" x14ac:dyDescent="0.25">
@@ -26825,7 +26830,7 @@
       </c>
       <c r="U150" s="80">
         <f t="shared" si="5"/>
-        <v>346.39016483516485</v>
+        <v>606.18278846153851</v>
       </c>
     </row>
     <row r="151" spans="1:21" x14ac:dyDescent="0.25">
@@ -26891,7 +26896,7 @@
       </c>
       <c r="U151" s="80">
         <f t="shared" si="5"/>
-        <v>2038.0992307692306</v>
+        <v>3566.6736538461537</v>
       </c>
     </row>
     <row r="152" spans="1:21" x14ac:dyDescent="0.25">
@@ -27011,7 +27016,7 @@
       </c>
       <c r="U153" s="80">
         <f t="shared" si="5"/>
-        <v>452.06032967032968</v>
+        <v>791.10557692307691</v>
       </c>
     </row>
     <row r="154" spans="1:21" x14ac:dyDescent="0.25">
@@ -27071,7 +27076,7 @@
       </c>
       <c r="U154" s="80">
         <f t="shared" si="5"/>
-        <v>9.827637362637363</v>
+        <v>17.198365384615386</v>
       </c>
     </row>
     <row r="155" spans="1:21" x14ac:dyDescent="0.25">
@@ -27131,7 +27136,7 @@
       </c>
       <c r="U155" s="80">
         <f t="shared" si="5"/>
-        <v>0.18516483516483526</v>
+        <v>0.32403846153846172</v>
       </c>
     </row>
     <row r="156" spans="1:21" x14ac:dyDescent="0.25">
@@ -27257,7 +27262,7 @@
       </c>
       <c r="U157" s="80">
         <f t="shared" si="5"/>
-        <v>21879.619505494506</v>
+        <v>38289.334134615383</v>
       </c>
     </row>
     <row r="158" spans="1:21" x14ac:dyDescent="0.25">
@@ -27437,7 +27442,7 @@
       </c>
       <c r="U161" s="80">
         <f t="shared" si="5"/>
-        <v>0.15428571428571428</v>
+        <v>0.26999999999999996</v>
       </c>
     </row>
     <row r="162" spans="1:21" x14ac:dyDescent="0.25">
@@ -27497,7 +27502,7 @@
       </c>
       <c r="U162" s="80">
         <f t="shared" si="5"/>
-        <v>87.150109890109889</v>
+        <v>152.5126923076923</v>
       </c>
     </row>
     <row r="163" spans="1:21" x14ac:dyDescent="0.25">
@@ -27557,7 +27562,7 @@
       </c>
       <c r="U163" s="80">
         <f t="shared" si="5"/>
-        <v>140.36489010989013</v>
+        <v>245.6385576923077</v>
       </c>
     </row>
     <row r="164" spans="1:21" x14ac:dyDescent="0.25">
@@ -27617,7 +27622,7 @@
       </c>
       <c r="U164" s="80">
         <f t="shared" si="5"/>
-        <v>21.98087912087912</v>
+        <v>38.466538461538462</v>
       </c>
     </row>
     <row r="165" spans="1:21" x14ac:dyDescent="0.25">
@@ -27677,7 +27682,7 @@
       </c>
       <c r="U165" s="80">
         <f t="shared" si="5"/>
-        <v>23.528021978021975</v>
+        <v>41.174038461538458</v>
       </c>
     </row>
     <row r="166" spans="1:21" x14ac:dyDescent="0.25">
@@ -27737,7 +27742,7 @@
       </c>
       <c r="U166" s="80">
         <f t="shared" si="5"/>
-        <v>131.82384615384618</v>
+        <v>230.69173076923079</v>
       </c>
     </row>
     <row r="167" spans="1:21" x14ac:dyDescent="0.25">
@@ -27797,7 +27802,7 @@
       </c>
       <c r="U167" s="80">
         <f t="shared" si="5"/>
-        <v>98.866648351648365</v>
+        <v>173.01663461538465</v>
       </c>
     </row>
     <row r="168" spans="1:21" x14ac:dyDescent="0.25">
@@ -27857,7 +27862,7 @@
       </c>
       <c r="U168" s="80">
         <f t="shared" si="5"/>
-        <v>404.94472527472539</v>
+        <v>708.65326923076941</v>
       </c>
     </row>
     <row r="169" spans="1:21" x14ac:dyDescent="0.25">
@@ -27917,7 +27922,7 @@
       </c>
       <c r="U169" s="80">
         <f t="shared" si="5"/>
-        <v>20.565274725274726</v>
+        <v>35.989230769230772</v>
       </c>
     </row>
     <row r="170" spans="1:21" x14ac:dyDescent="0.25">
@@ -27977,7 +27982,7 @@
       </c>
       <c r="U170" s="80">
         <f t="shared" si="5"/>
-        <v>144.35527472527471</v>
+        <v>252.62173076923077</v>
       </c>
     </row>
     <row r="171" spans="1:21" x14ac:dyDescent="0.25">
@@ -28037,7 +28042,7 @@
       </c>
       <c r="U171" s="80">
         <f t="shared" si="5"/>
-        <v>159.63818681318682</v>
+        <v>279.36682692307693</v>
       </c>
     </row>
     <row r="172" spans="1:21" x14ac:dyDescent="0.25">
@@ -28277,7 +28282,7 @@
       </c>
       <c r="U175" s="80">
         <f t="shared" si="5"/>
-        <v>154.4084065934066</v>
+        <v>270.21471153846153</v>
       </c>
     </row>
     <row r="176" spans="1:21" x14ac:dyDescent="0.25">
@@ -28337,7 +28342,7 @@
       </c>
       <c r="U176" s="80">
         <f t="shared" si="5"/>
-        <v>147.91428571428574</v>
+        <v>258.85000000000002</v>
       </c>
     </row>
     <row r="177" spans="1:21" x14ac:dyDescent="0.25">
@@ -28397,7 +28402,7 @@
       </c>
       <c r="U177" s="80">
         <f t="shared" si="5"/>
-        <v>119.39230769230768</v>
+        <v>208.93653846153845</v>
       </c>
     </row>
     <row r="178" spans="1:21" x14ac:dyDescent="0.25">
@@ -28457,7 +28462,7 @@
       </c>
       <c r="U178" s="80">
         <f t="shared" si="5"/>
-        <v>169.7764285714286</v>
+        <v>297.10875000000004</v>
       </c>
     </row>
     <row r="179" spans="1:21" x14ac:dyDescent="0.25">
@@ -28517,7 +28522,7 @@
       </c>
       <c r="U179" s="80">
         <f t="shared" si="5"/>
-        <v>56.898791208791202</v>
+        <v>99.572884615384609</v>
       </c>
     </row>
     <row r="180" spans="1:21" x14ac:dyDescent="0.25">
@@ -28577,7 +28582,7 @@
       </c>
       <c r="U180" s="80">
         <f t="shared" si="5"/>
-        <v>299.24170329670329</v>
+        <v>523.67298076923078</v>
       </c>
     </row>
     <row r="181" spans="1:21" x14ac:dyDescent="0.25">
@@ -28697,7 +28702,7 @@
       </c>
       <c r="U182" s="80">
         <f t="shared" si="5"/>
-        <v>2.1949999999999998</v>
+        <v>3.8412500000000001</v>
       </c>
     </row>
     <row r="183" spans="1:21" x14ac:dyDescent="0.25">
@@ -28757,7 +28762,7 @@
       </c>
       <c r="U183" s="80">
         <f t="shared" si="5"/>
-        <v>83.723791208791212</v>
+        <v>146.51663461538462</v>
       </c>
     </row>
     <row r="184" spans="1:21" x14ac:dyDescent="0.25">
@@ -28817,7 +28822,7 @@
       </c>
       <c r="U184" s="80">
         <f t="shared" si="5"/>
-        <v>29.155659340659337</v>
+        <v>51.022403846153843</v>
       </c>
     </row>
     <row r="185" spans="1:21" x14ac:dyDescent="0.25">
@@ -28997,7 +29002,7 @@
       </c>
       <c r="U187" s="80">
         <f t="shared" si="5"/>
-        <v>11.998406593406594</v>
+        <v>20.997211538461539</v>
       </c>
     </row>
     <row r="188" spans="1:21" x14ac:dyDescent="0.25">
@@ -29057,7 +29062,7 @@
       </c>
       <c r="U188" s="80">
         <f t="shared" si="5"/>
-        <v>102.32258241758242</v>
+        <v>179.06451923076924</v>
       </c>
     </row>
     <row r="189" spans="1:21" x14ac:dyDescent="0.25">
@@ -29117,7 +29122,7 @@
       </c>
       <c r="U189" s="80">
         <f t="shared" si="5"/>
-        <v>170.5397802197802</v>
+        <v>298.44461538461536</v>
       </c>
     </row>
     <row r="190" spans="1:21" x14ac:dyDescent="0.25">
@@ -29177,7 +29182,7 @@
       </c>
       <c r="U190" s="80">
         <f t="shared" si="5"/>
-        <v>6.8321428571428573</v>
+        <v>11.956250000000001</v>
       </c>
     </row>
     <row r="191" spans="1:21" x14ac:dyDescent="0.25">
@@ -29297,7 +29302,7 @@
       </c>
       <c r="U192" s="80">
         <f t="shared" si="5"/>
-        <v>96.996098901098904</v>
+        <v>169.74317307692309</v>
       </c>
     </row>
     <row r="193" spans="1:21" x14ac:dyDescent="0.25">
@@ -29357,7 +29362,7 @@
       </c>
       <c r="U193" s="80">
         <f t="shared" si="5"/>
-        <v>709.21170329670326</v>
+        <v>1241.1204807692307</v>
       </c>
     </row>
     <row r="194" spans="1:21" x14ac:dyDescent="0.25">
@@ -29417,7 +29422,7 @@
       </c>
       <c r="U194" s="80">
         <f t="shared" si="5"/>
-        <v>341.52368131868127</v>
+        <v>597.66644230769225</v>
       </c>
     </row>
     <row r="195" spans="1:21" x14ac:dyDescent="0.25">
@@ -29477,7 +29482,7 @@
       </c>
       <c r="U195" s="80">
         <f t="shared" si="5"/>
-        <v>42.526263736263736</v>
+        <v>74.42096153846154</v>
       </c>
     </row>
     <row r="196" spans="1:21" x14ac:dyDescent="0.25">
@@ -29537,7 +29542,7 @@
       </c>
       <c r="U196" s="80">
         <f t="shared" si="5"/>
-        <v>5139.605549450549</v>
+        <v>8994.3097115384608</v>
       </c>
     </row>
     <row r="197" spans="1:21" x14ac:dyDescent="0.25">
@@ -29597,7 +29602,7 @@
       </c>
       <c r="U197" s="80">
         <f t="shared" si="5"/>
-        <v>16.457582417582415</v>
+        <v>28.800769230769227</v>
       </c>
     </row>
     <row r="198" spans="1:21" x14ac:dyDescent="0.25">
@@ -29836,8 +29841,8 @@
         <v>2810.66</v>
       </c>
       <c r="U201" s="80">
-        <f t="shared" ref="U201:U264" si="7">(T201/$V$1)/7</f>
-        <v>15.443186813186813</v>
+        <f t="shared" ref="U201:U264" si="7">(T201/$V$1)/4</f>
+        <v>27.025576923076922</v>
       </c>
     </row>
     <row r="202" spans="1:21" x14ac:dyDescent="0.25">
@@ -30323,7 +30328,7 @@
       </c>
       <c r="U209" s="80">
         <f t="shared" si="7"/>
-        <v>8949.5354945054951</v>
+        <v>15661.687115384617</v>
       </c>
     </row>
     <row r="210" spans="1:21" x14ac:dyDescent="0.25">
@@ -30449,7 +30454,7 @@
       </c>
       <c r="U211" s="80">
         <f t="shared" si="7"/>
-        <v>8949.5354945054951</v>
+        <v>15661.687115384617</v>
       </c>
     </row>
     <row r="212" spans="1:21" x14ac:dyDescent="0.25">
@@ -30629,7 +30634,7 @@
       </c>
       <c r="U215" s="80">
         <f t="shared" si="7"/>
-        <v>1942.826978021978</v>
+        <v>3399.9472115384615</v>
       </c>
     </row>
     <row r="216" spans="1:21" x14ac:dyDescent="0.25">
@@ -30689,7 +30694,7 @@
       </c>
       <c r="U216" s="80">
         <f t="shared" si="7"/>
-        <v>28.043956043956047</v>
+        <v>49.07692307692308</v>
       </c>
     </row>
     <row r="217" spans="1:21" x14ac:dyDescent="0.25">
@@ -30749,7 +30754,7 @@
       </c>
       <c r="U217" s="80">
         <f t="shared" si="7"/>
-        <v>426.59027472527475</v>
+        <v>746.53298076923079</v>
       </c>
     </row>
     <row r="218" spans="1:21" x14ac:dyDescent="0.25">
@@ -30809,7 +30814,7 @@
       </c>
       <c r="U218" s="80">
         <f t="shared" si="7"/>
-        <v>34.25736263736264</v>
+        <v>59.950384615384614</v>
       </c>
     </row>
     <row r="219" spans="1:21" x14ac:dyDescent="0.25">
@@ -30869,7 +30874,7 @@
       </c>
       <c r="U219" s="80">
         <f t="shared" si="7"/>
-        <v>794.67241758241755</v>
+        <v>1390.6767307692307</v>
       </c>
     </row>
     <row r="220" spans="1:21" x14ac:dyDescent="0.25">
@@ -30929,7 +30934,7 @@
       </c>
       <c r="U220" s="80">
         <f t="shared" si="7"/>
-        <v>18.373186813186813</v>
+        <v>32.153076923076924</v>
       </c>
     </row>
     <row r="221" spans="1:21" x14ac:dyDescent="0.25">
@@ -31049,7 +31054,7 @@
       </c>
       <c r="U222" s="80">
         <f t="shared" si="7"/>
-        <v>8.797417582417582</v>
+        <v>15.395480769230769</v>
       </c>
     </row>
     <row r="223" spans="1:21" x14ac:dyDescent="0.25">
@@ -31109,7 +31114,7 @@
       </c>
       <c r="U223" s="80">
         <f t="shared" si="7"/>
-        <v>4.0824175824175822E-2</v>
+        <v>7.1442307692307694E-2</v>
       </c>
     </row>
     <row r="224" spans="1:21" x14ac:dyDescent="0.25">
@@ -31169,7 +31174,7 @@
       </c>
       <c r="U224" s="80">
         <f t="shared" si="7"/>
-        <v>3.8060989010989013</v>
+        <v>6.6606730769230769</v>
       </c>
     </row>
     <row r="225" spans="1:21" x14ac:dyDescent="0.25">
@@ -31289,7 +31294,7 @@
       </c>
       <c r="U226" s="80">
         <f t="shared" si="7"/>
-        <v>-0.74967032967032965</v>
+        <v>-1.311923076923077</v>
       </c>
     </row>
     <row r="227" spans="1:21" x14ac:dyDescent="0.25">
@@ -31349,7 +31354,7 @@
       </c>
       <c r="U227" s="80">
         <f t="shared" si="7"/>
-        <v>118.59192307692308</v>
+        <v>207.53586538461539</v>
       </c>
     </row>
     <row r="228" spans="1:21" x14ac:dyDescent="0.25">
@@ -31409,7 +31414,7 @@
       </c>
       <c r="U228" s="80">
         <f t="shared" si="7"/>
-        <v>24.308406593406595</v>
+        <v>42.539711538461539</v>
       </c>
     </row>
     <row r="229" spans="1:21" x14ac:dyDescent="0.25">
@@ -31469,7 +31474,7 @@
       </c>
       <c r="U229" s="80">
         <f t="shared" si="7"/>
-        <v>0.60989010989010983</v>
+        <v>1.0673076923076923</v>
       </c>
     </row>
     <row r="230" spans="1:21" x14ac:dyDescent="0.25">
@@ -31529,7 +31534,7 @@
       </c>
       <c r="U230" s="80">
         <f t="shared" si="7"/>
-        <v>81.932967032967028</v>
+        <v>143.38269230769231</v>
       </c>
     </row>
     <row r="231" spans="1:21" x14ac:dyDescent="0.25">
@@ -31649,7 +31654,7 @@
       </c>
       <c r="U232" s="80">
         <f t="shared" si="7"/>
-        <v>2.7472527472527473</v>
+        <v>4.8076923076923075</v>
       </c>
     </row>
     <row r="233" spans="1:21" x14ac:dyDescent="0.25">
@@ -31709,7 +31714,7 @@
       </c>
       <c r="U233" s="80">
         <f t="shared" si="7"/>
-        <v>0.50230769230769234</v>
+        <v>0.87903846153846155</v>
       </c>
     </row>
     <row r="234" spans="1:21" x14ac:dyDescent="0.25">
@@ -31769,7 +31774,7 @@
       </c>
       <c r="U234" s="80">
         <f t="shared" si="7"/>
-        <v>4.3490659340659343</v>
+        <v>7.6108653846153844</v>
       </c>
     </row>
     <row r="235" spans="1:21" x14ac:dyDescent="0.25">
@@ -31829,7 +31834,7 @@
       </c>
       <c r="U235" s="80">
         <f t="shared" si="7"/>
-        <v>35.93796703296703</v>
+        <v>62.891442307692309</v>
       </c>
     </row>
     <row r="236" spans="1:21" x14ac:dyDescent="0.25">
@@ -31889,7 +31894,7 @@
       </c>
       <c r="U236" s="80">
         <f t="shared" si="7"/>
-        <v>1125.1606043956044</v>
+        <v>1969.0310576923077</v>
       </c>
     </row>
     <row r="237" spans="1:21" x14ac:dyDescent="0.25">
@@ -31949,7 +31954,7 @@
       </c>
       <c r="U237" s="80">
         <f t="shared" si="7"/>
-        <v>81.332197802197811</v>
+        <v>142.33134615384617</v>
       </c>
     </row>
     <row r="238" spans="1:21" x14ac:dyDescent="0.25">
@@ -32009,7 +32014,7 @@
       </c>
       <c r="U238" s="80">
         <f t="shared" si="7"/>
-        <v>11.850494505494506</v>
+        <v>20.738365384615385</v>
       </c>
     </row>
     <row r="239" spans="1:21" x14ac:dyDescent="0.25">
@@ -32195,7 +32200,7 @@
       </c>
       <c r="U241" s="80">
         <f t="shared" si="7"/>
-        <v>4743.9819230769235</v>
+        <v>8301.9683653846168</v>
       </c>
     </row>
     <row r="242" spans="1:21" x14ac:dyDescent="0.25">
@@ -32345,7 +32350,7 @@
       </c>
       <c r="U244" s="80">
         <f t="shared" si="7"/>
-        <v>20.959285714285709</v>
+        <v>36.678749999999994</v>
       </c>
     </row>
     <row r="245" spans="1:21" x14ac:dyDescent="0.25">
@@ -32405,7 +32410,7 @@
       </c>
       <c r="U245" s="80">
         <f t="shared" si="7"/>
-        <v>15.025109890109889</v>
+        <v>26.293942307692305</v>
       </c>
     </row>
     <row r="246" spans="1:21" x14ac:dyDescent="0.25">
@@ -32525,7 +32530,7 @@
       </c>
       <c r="U247" s="80">
         <f t="shared" si="7"/>
-        <v>144.80395604395605</v>
+        <v>253.40692307692308</v>
       </c>
     </row>
     <row r="248" spans="1:21" x14ac:dyDescent="0.25">
@@ -32585,7 +32590,7 @@
       </c>
       <c r="U248" s="80">
         <f t="shared" si="7"/>
-        <v>24.860439560439563</v>
+        <v>43.505769230769232</v>
       </c>
     </row>
     <row r="249" spans="1:21" x14ac:dyDescent="0.25">
@@ -32645,7 +32650,7 @@
       </c>
       <c r="U249" s="80">
         <f t="shared" si="7"/>
-        <v>155.47115384615384</v>
+        <v>272.07451923076923</v>
       </c>
     </row>
     <row r="250" spans="1:21" x14ac:dyDescent="0.25">
@@ -32831,7 +32836,7 @@
       </c>
       <c r="U252" s="80">
         <f t="shared" si="7"/>
-        <v>361.11994505494511</v>
+        <v>631.95990384615391</v>
       </c>
     </row>
     <row r="253" spans="1:21" x14ac:dyDescent="0.25">
@@ -33041,7 +33046,7 @@
       </c>
       <c r="U256" s="80">
         <f t="shared" si="7"/>
-        <v>2508.1870329670332</v>
+        <v>4389.3273076923078</v>
       </c>
     </row>
     <row r="257" spans="1:21" x14ac:dyDescent="0.25">
@@ -33161,7 +33166,7 @@
       </c>
       <c r="U258" s="80">
         <f t="shared" si="7"/>
-        <v>126.06516483516484</v>
+        <v>220.61403846153846</v>
       </c>
     </row>
     <row r="259" spans="1:21" x14ac:dyDescent="0.25">
@@ -33341,7 +33346,7 @@
       </c>
       <c r="U261" s="80">
         <f t="shared" si="7"/>
-        <v>831.8067582417583</v>
+        <v>1455.6618269230771</v>
       </c>
     </row>
     <row r="262" spans="1:21" x14ac:dyDescent="0.25">
@@ -33401,7 +33406,7 @@
       </c>
       <c r="U262" s="80">
         <f t="shared" si="7"/>
-        <v>308.97318681318677</v>
+        <v>540.70307692307688</v>
       </c>
     </row>
     <row r="263" spans="1:21" x14ac:dyDescent="0.25">
@@ -33467,7 +33472,7 @@
       </c>
       <c r="U263" s="80">
         <f t="shared" si="7"/>
-        <v>3775.0321428571428</v>
+        <v>6606.3062499999996</v>
       </c>
     </row>
     <row r="264" spans="1:21" x14ac:dyDescent="0.25">
@@ -33556,7 +33561,7 @@
         <v>0</v>
       </c>
       <c r="U265" s="80">
-        <f t="shared" ref="U265:U327" si="9">(T265/$V$1)/7</f>
+        <f t="shared" ref="U265:U327" si="9">(T265/$V$1)/4</f>
         <v>0</v>
       </c>
     </row>
@@ -33737,7 +33742,7 @@
       </c>
       <c r="U268" s="80">
         <f t="shared" si="9"/>
-        <v>-0.18175824175824173</v>
+        <v>-0.31807692307692303</v>
       </c>
     </row>
     <row r="269" spans="1:21" x14ac:dyDescent="0.25">
@@ -34337,7 +34342,7 @@
       </c>
       <c r="U278" s="80">
         <f t="shared" si="9"/>
-        <v>-2284.8806593406593</v>
+        <v>-3998.541153846154</v>
       </c>
     </row>
     <row r="279" spans="1:21" x14ac:dyDescent="0.25">
@@ -34643,7 +34648,7 @@
       </c>
       <c r="U283" s="80">
         <f t="shared" si="9"/>
-        <v>-2285.0624175824173</v>
+        <v>-3998.8592307692306</v>
       </c>
     </row>
     <row r="284" spans="1:21" x14ac:dyDescent="0.25">
@@ -34709,7 +34714,7 @@
       </c>
       <c r="U284" s="80">
         <f t="shared" si="9"/>
-        <v>6595.0715934065938</v>
+        <v>11541.375288461539</v>
       </c>
     </row>
     <row r="285" spans="1:21" x14ac:dyDescent="0.25">
@@ -34949,7 +34954,7 @@
       </c>
       <c r="U289" s="80">
         <f t="shared" si="9"/>
-        <v>377.30285714285714</v>
+        <v>660.28</v>
       </c>
     </row>
     <row r="290" spans="1:21" x14ac:dyDescent="0.25">
@@ -35008,8 +35013,8 @@
         <v>590935.91</v>
       </c>
       <c r="U290" s="80">
-        <f>(T290/$V$1)/7</f>
-        <v>3246.9006043956042</v>
+        <f t="shared" si="9"/>
+        <v>5682.0760576923076</v>
       </c>
     </row>
     <row r="291" spans="1:21" x14ac:dyDescent="0.25">
@@ -35069,7 +35074,7 @@
       </c>
       <c r="U291" s="80">
         <f t="shared" si="9"/>
-        <v>0.40659340659340659</v>
+        <v>0.71153846153846156</v>
       </c>
     </row>
     <row r="292" spans="1:21" x14ac:dyDescent="0.25">
@@ -35129,7 +35134,7 @@
       </c>
       <c r="U292" s="80">
         <f t="shared" si="9"/>
-        <v>86.494505494505489</v>
+        <v>151.36538461538461</v>
       </c>
     </row>
     <row r="293" spans="1:21" x14ac:dyDescent="0.25">
@@ -35189,7 +35194,7 @@
       </c>
       <c r="U293" s="80">
         <f t="shared" si="9"/>
-        <v>8.3655494505494499</v>
+        <v>14.639711538461539</v>
       </c>
     </row>
     <row r="294" spans="1:21" x14ac:dyDescent="0.25">
@@ -35249,7 +35254,7 @@
       </c>
       <c r="U294" s="80">
         <f t="shared" si="9"/>
-        <v>218.10131868131865</v>
+        <v>381.67730769230764</v>
       </c>
     </row>
     <row r="295" spans="1:21" x14ac:dyDescent="0.25">
@@ -35429,7 +35434,7 @@
       </c>
       <c r="U297" s="80">
         <f t="shared" si="9"/>
-        <v>2.6509890109890111</v>
+        <v>4.6392307692307693</v>
       </c>
     </row>
     <row r="298" spans="1:21" x14ac:dyDescent="0.25">
@@ -36455,7 +36460,7 @@
       </c>
       <c r="U314" s="80">
         <f t="shared" si="9"/>
-        <v>3940.2224175824181</v>
+        <v>6895.3892307692313</v>
       </c>
     </row>
     <row r="315" spans="1:21" x14ac:dyDescent="0.25">
@@ -36725,7 +36730,7 @@
       </c>
       <c r="U319" s="80">
         <f t="shared" si="9"/>
-        <v>0.93406593406593408</v>
+        <v>1.6346153846153846</v>
       </c>
     </row>
     <row r="320" spans="1:21" x14ac:dyDescent="0.25">
@@ -37031,7 +37036,7 @@
       </c>
       <c r="U324" s="80">
         <f t="shared" si="9"/>
-        <v>0.93406593406593408</v>
+        <v>1.6346153846153846</v>
       </c>
     </row>
     <row r="325" spans="1:21" x14ac:dyDescent="0.25">
@@ -37097,7 +37102,7 @@
       </c>
       <c r="U325" s="80">
         <f t="shared" si="9"/>
-        <v>3941.1564835164841</v>
+        <v>6897.0238461538474</v>
       </c>
     </row>
     <row r="326" spans="1:21" x14ac:dyDescent="0.25">
@@ -37163,7 +37168,7 @@
       </c>
       <c r="U326" s="80">
         <f t="shared" si="9"/>
-        <v>21487.58587912087</v>
+        <v>37603.275288461526</v>
       </c>
     </row>
     <row r="327" spans="1:21" x14ac:dyDescent="0.25">
@@ -37205,7 +37210,7 @@
       </c>
       <c r="U327" s="80">
         <f t="shared" si="9"/>
-        <v>62852.968956043951</v>
+        <v>109992.69567307692</v>
       </c>
     </row>
     <row r="330" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Flash v5.8: MILA occupancy/other tweak from latest EBITDA workbook
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/excel/ebidta-calculation-mila-lounge.xlsx
+++ b/data/excel/ebidta-calculation-mila-lounge.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MatthiasLavenant\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1489FA02-5096-4E88-B8B1-3E6B83A97E1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{101F0B2A-8655-4919-99C5-76B8DE05C21D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="855" windowWidth="29040" windowHeight="15720" xr2:uid="{3C90C578-B115-41AD-8F85-41FE68FE49FA}"/>
   </bookViews>
@@ -9882,12 +9882,11 @@
       </c>
       <c r="C152" s="48"/>
       <c r="D152" s="49">
-        <f>SUM(D144:D151)</f>
-        <v>6606.3062499999996</v>
+        <f>E152*D10</f>
+        <v>3690</v>
       </c>
       <c r="E152" s="50">
-        <f t="shared" si="6"/>
-        <v>0.10741961382113821</v>
+        <v>0.06</v>
       </c>
       <c r="F152" s="50"/>
       <c r="G152" s="50"/>
@@ -10094,12 +10093,11 @@
       </c>
       <c r="C167" s="56"/>
       <c r="D167" s="57">
-        <f>'OPEX DATA 2'!U278</f>
-        <v>-3998.541153846154</v>
+        <f>E167*D10</f>
+        <v>-2029.5</v>
       </c>
       <c r="E167" s="58">
-        <f t="shared" si="7"/>
-        <v>-6.5016929330831766E-2</v>
+        <v>-3.3000000000000002E-2</v>
       </c>
     </row>
     <row r="168" spans="2:7" x14ac:dyDescent="0.25">
@@ -10170,11 +10168,11 @@
       <c r="C172" s="48"/>
       <c r="D172" s="49">
         <f>SUM(D155:D171)</f>
-        <v>-3998.8592307692311</v>
+        <v>-2029.8180769230769</v>
       </c>
       <c r="E172" s="50">
         <f t="shared" si="7"/>
-        <v>-6.5022101313320826E-2</v>
+        <v>-3.3005171982489055E-2</v>
       </c>
       <c r="F172" s="50"/>
       <c r="G172" s="50"/>
@@ -10614,11 +10612,11 @@
       <c r="C203" s="48"/>
       <c r="D203" s="49">
         <f>D43-D50-D101-D130-D141-D152-D172-D201</f>
-        <v>640.6150961538533</v>
+        <v>1587.880192307699</v>
       </c>
       <c r="E203" s="50">
         <f>D203/D36</f>
-        <v>1.041650562851794E-2</v>
+        <v>2.5819190118824373E-2</v>
       </c>
       <c r="F203" s="50"/>
       <c r="G203" s="50"/>
@@ -10644,7 +10642,7 @@
       <c r="C207" s="63"/>
       <c r="D207" s="64">
         <f>E203</f>
-        <v>1.041650562851794E-2</v>
+        <v>2.5819190118824373E-2</v>
       </c>
     </row>
     <row r="208" spans="2:175" s="20" customFormat="1" x14ac:dyDescent="0.25">
@@ -35253,7 +35251,7 @@
         <v>39694.439999999995</v>
       </c>
       <c r="U294" s="80">
-        <f t="shared" si="9"/>
+        <f>(T294/$V$1)/4</f>
         <v>381.67730769230764</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Flash v5.9: MILA EBITDA fixed daily OPEX + occupancy/service charge pct
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/excel/ebidta-calculation-mila-lounge.xlsx
+++ b/data/excel/ebidta-calculation-mila-lounge.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MatthiasLavenant\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{101F0B2A-8655-4919-99C5-76B8DE05C21D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9206479A-0069-4734-A499-938135B83D28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="855" windowWidth="29040" windowHeight="15720" xr2:uid="{3C90C578-B115-41AD-8F85-41FE68FE49FA}"/>
   </bookViews>
@@ -6241,7 +6241,7 @@
         <v>11</v>
       </c>
       <c r="D5" s="11">
-        <v>4000</v>
+        <v>15000</v>
       </c>
       <c r="E5" s="12"/>
       <c r="F5" s="13"/>
@@ -6422,7 +6422,7 @@
       <c r="C6" s="2"/>
       <c r="D6" s="14">
         <f>IFERROR(D5/D8,"")</f>
-        <v>0.14285714285714285</v>
+        <v>0.3</v>
       </c>
       <c r="E6" s="15"/>
       <c r="F6" s="16"/>
@@ -6781,7 +6781,7 @@
       </c>
       <c r="D8" s="19">
         <f>D15+D16</f>
-        <v>28000</v>
+        <v>50000</v>
       </c>
       <c r="E8" s="19"/>
       <c r="T8" t="str">
@@ -6813,7 +6813,7 @@
       </c>
       <c r="C10" s="22"/>
       <c r="D10" s="23">
-        <v>61500</v>
+        <v>67500</v>
       </c>
       <c r="E10" s="23"/>
       <c r="W10">
@@ -6887,7 +6887,7 @@
       </c>
       <c r="D16" s="34">
         <f>IFERROR(D5*E16,0)</f>
-        <v>8000</v>
+        <v>30000</v>
       </c>
       <c r="E16" s="35">
         <f>VLOOKUP(D$2,'[1]Overview 2026'!$B$7:$AC$52,$C16,FALSE)</f>
@@ -6924,7 +6924,7 @@
       </c>
       <c r="D20" s="39">
         <f>D16/D19</f>
-        <v>285.71428571428572</v>
+        <v>1071.4285714285713</v>
       </c>
       <c r="E20" s="39"/>
     </row>
@@ -7121,7 +7121,7 @@
       </c>
       <c r="D33" s="34">
         <f>D$36*E33</f>
-        <v>38130</v>
+        <v>41850</v>
       </c>
       <c r="E33" s="20">
         <v>0.62</v>
@@ -7133,7 +7133,7 @@
       </c>
       <c r="D34" s="34">
         <f t="shared" ref="D34" si="0">D$36*E34</f>
-        <v>20910</v>
+        <v>22950</v>
       </c>
       <c r="E34" s="20">
         <f>E36-E33-E35</f>
@@ -7146,7 +7146,7 @@
       </c>
       <c r="D35" s="34">
         <f>D$36*E35</f>
-        <v>2460</v>
+        <v>2700</v>
       </c>
       <c r="E35" s="20">
         <v>0.04</v>
@@ -7159,7 +7159,7 @@
       <c r="C36" s="22"/>
       <c r="D36" s="45">
         <f>D10</f>
-        <v>61500</v>
+        <v>67500</v>
       </c>
       <c r="E36" s="46">
         <v>1</v>
@@ -7174,7 +7174,7 @@
       </c>
       <c r="D38" s="34">
         <f>E38*D33</f>
-        <v>5719.5</v>
+        <v>6277.5</v>
       </c>
       <c r="E38" s="20">
         <v>0.15</v>
@@ -7186,7 +7186,7 @@
       </c>
       <c r="D39" s="34">
         <f t="shared" ref="D39:D40" si="1">E39*D34</f>
-        <v>5541.1500000000005</v>
+        <v>6081.75</v>
       </c>
       <c r="E39" s="20">
         <v>0.26500000000000001</v>
@@ -7198,7 +7198,7 @@
       </c>
       <c r="D40" s="34">
         <f t="shared" si="1"/>
-        <v>688.80000000000007</v>
+        <v>756.00000000000011</v>
       </c>
       <c r="E40" s="20">
         <v>0.28000000000000003</v>
@@ -7211,7 +7211,7 @@
       <c r="C41" s="22"/>
       <c r="D41" s="45">
         <f>SUM(D38:D40)</f>
-        <v>11949.45</v>
+        <v>13115.25</v>
       </c>
       <c r="E41" s="46">
         <f>D41/D36</f>
@@ -7228,11 +7228,11 @@
       <c r="C43" s="22"/>
       <c r="D43" s="45">
         <f>D36-D41</f>
-        <v>49550.55</v>
+        <v>54384.75</v>
       </c>
       <c r="E43" s="46">
         <f>D43/D36</f>
-        <v>0.80570000000000008</v>
+        <v>0.80569999999999997</v>
       </c>
     </row>
     <row r="45" spans="2:175" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -7422,7 +7422,7 @@
       </c>
       <c r="E46" s="20">
         <f>D46/D$36</f>
-        <v>0.12363114915572233</v>
+        <v>0.11264171367521368</v>
       </c>
     </row>
     <row r="47" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7435,7 +7435,7 @@
       </c>
       <c r="E47" s="20">
         <f t="shared" ref="E47:E50" si="2">D47/D$36</f>
-        <v>4.0506072545340839E-2</v>
+        <v>3.6905532763532763E-2</v>
       </c>
     </row>
     <row r="48" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7448,7 +7448,7 @@
       </c>
       <c r="E48" s="20">
         <f t="shared" si="2"/>
-        <v>8.6770345528455292E-2</v>
+        <v>7.9057425925925934E-2</v>
       </c>
     </row>
     <row r="49" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7461,7 +7461,7 @@
       </c>
       <c r="E49" s="20">
         <f t="shared" si="2"/>
-        <v>7.1137847091932452E-2</v>
+        <v>6.4814482905982906E-2</v>
       </c>
     </row>
     <row r="50" spans="2:175" x14ac:dyDescent="0.25">
@@ -7475,7 +7475,7 @@
       </c>
       <c r="E50" s="46">
         <f t="shared" si="2"/>
-        <v>0.3220454143214509</v>
+        <v>0.29341915527065526</v>
       </c>
     </row>
     <row r="52" spans="2:175" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -7668,7 +7668,7 @@
       </c>
       <c r="E53" s="20">
         <f t="shared" ref="E53:E101" si="3">D53/D$36</f>
-        <v>4.3902439024390241E-6</v>
+        <v>3.9999999999999998E-6</v>
       </c>
     </row>
     <row r="54" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7682,7 +7682,7 @@
       </c>
       <c r="E54" s="20">
         <f t="shared" si="3"/>
-        <v>2.4798811757348344E-3</v>
+        <v>2.2594472934472933E-3</v>
       </c>
     </row>
     <row r="55" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7696,7 +7696,7 @@
       </c>
       <c r="E55" s="20">
         <f t="shared" si="3"/>
-        <v>3.9941228893058166E-3</v>
+        <v>3.6390897435897439E-3</v>
       </c>
     </row>
     <row r="56" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7710,7 +7710,7 @@
       </c>
       <c r="E56" s="20">
         <f t="shared" si="3"/>
-        <v>6.2547217010631647E-4</v>
+        <v>5.6987464387464387E-4</v>
       </c>
     </row>
     <row r="57" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7724,7 +7724,7 @@
       </c>
       <c r="E57" s="20">
         <f t="shared" si="3"/>
-        <v>6.6949656035021881E-4</v>
+        <v>6.0998575498575497E-4</v>
       </c>
     </row>
     <row r="58" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7738,7 +7738,7 @@
       </c>
       <c r="E58" s="20">
         <f t="shared" si="3"/>
-        <v>3.7510850531582243E-3</v>
+        <v>3.4176552706552711E-3</v>
       </c>
     </row>
     <row r="59" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7752,7 +7752,7 @@
       </c>
       <c r="E59" s="20">
         <f t="shared" si="3"/>
-        <v>2.8132786116322707E-3</v>
+        <v>2.5632094017094022E-3</v>
       </c>
     </row>
     <row r="60" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7766,7 +7766,7 @@
       </c>
       <c r="E60" s="20">
         <f t="shared" si="3"/>
-        <v>1.152281738586617E-2</v>
+        <v>1.0498566951566955E-2</v>
       </c>
     </row>
     <row r="61" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="E61" s="20">
         <f t="shared" si="3"/>
-        <v>5.8519074421513448E-4</v>
+        <v>5.3317378917378921E-4</v>
       </c>
     </row>
     <row r="62" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7794,7 +7794,7 @@
       </c>
       <c r="E62" s="20">
         <f t="shared" si="3"/>
-        <v>4.1076704190118824E-3</v>
+        <v>3.7425441595441596E-3</v>
       </c>
     </row>
     <row r="63" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7808,7 +7808,7 @@
       </c>
       <c r="E63" s="20">
         <f t="shared" si="3"/>
-        <v>4.5425500312695436E-3</v>
+        <v>4.1387678062678067E-3</v>
       </c>
     </row>
     <row r="64" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="E67" s="20">
         <f t="shared" si="3"/>
-        <v>4.3937351469668538E-3</v>
+        <v>4.0031809116809116E-3</v>
       </c>
     </row>
     <row r="68" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7878,7 +7878,7 @@
       </c>
       <c r="E68" s="20">
         <f t="shared" si="3"/>
-        <v>4.2089430894308947E-3</v>
+        <v>3.8348148148148152E-3</v>
       </c>
     </row>
     <row r="69" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7892,7 +7892,7 @@
       </c>
       <c r="E69" s="20">
         <f t="shared" si="3"/>
-        <v>3.3973420888055031E-3</v>
+        <v>3.0953561253561253E-3</v>
       </c>
     </row>
     <row r="70" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7906,7 +7906,7 @@
       </c>
       <c r="E70" s="20">
         <f t="shared" si="3"/>
-        <v>4.8310365853658542E-3</v>
+        <v>4.4016111111111113E-3</v>
       </c>
     </row>
     <row r="71" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7920,7 +7920,7 @@
       </c>
       <c r="E71" s="20">
         <f t="shared" si="3"/>
-        <v>1.6190712945590993E-3</v>
+        <v>1.4751538461538461E-3</v>
       </c>
     </row>
     <row r="72" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7934,7 +7934,7 @@
       </c>
       <c r="E72" s="20">
         <f t="shared" si="3"/>
-        <v>8.5150078173858671E-3</v>
+        <v>7.7581182336182337E-3</v>
       </c>
     </row>
     <row r="73" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7962,7 +7962,7 @@
       </c>
       <c r="E74" s="20">
         <f t="shared" si="3"/>
-        <v>6.2459349593495936E-5</v>
+        <v>5.6907407407407407E-5</v>
       </c>
     </row>
     <row r="75" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7976,7 +7976,7 @@
       </c>
       <c r="E75" s="20">
         <f t="shared" si="3"/>
-        <v>2.382384302689181E-3</v>
+        <v>2.1706168091168094E-3</v>
       </c>
     </row>
     <row r="76" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7990,7 +7990,7 @@
       </c>
       <c r="E76" s="20">
         <f t="shared" si="3"/>
-        <v>8.2963258286429011E-4</v>
+        <v>7.5588746438746436E-4</v>
       </c>
     </row>
     <row r="77" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8032,7 +8032,7 @@
       </c>
       <c r="E79" s="20">
         <f t="shared" si="3"/>
-        <v>3.414180737961226E-4</v>
+        <v>3.1106980056980058E-4</v>
       </c>
     </row>
     <row r="80" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8046,7 +8046,7 @@
       </c>
       <c r="E80" s="20">
         <f t="shared" si="3"/>
-        <v>2.9116181988742963E-3</v>
+        <v>2.6528076923076926E-3</v>
       </c>
     </row>
     <row r="81" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8060,7 +8060,7 @@
       </c>
       <c r="E81" s="20">
         <f t="shared" si="3"/>
-        <v>4.8527579737335834E-3</v>
+        <v>4.4214017094017094E-3</v>
       </c>
     </row>
     <row r="82" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8074,7 +8074,7 @@
       </c>
       <c r="E82" s="20">
         <f t="shared" si="3"/>
-        <v>1.9441056910569107E-4</v>
+        <v>1.7712962962962965E-4</v>
       </c>
     </row>
     <row r="83" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8102,7 +8102,7 @@
       </c>
       <c r="E84" s="20">
         <f t="shared" si="3"/>
-        <v>2.7600515947467166E-3</v>
+        <v>2.5147136752136754E-3</v>
       </c>
     </row>
     <row r="85" spans="2:175" x14ac:dyDescent="0.25">
@@ -8117,7 +8117,7 @@
       </c>
       <c r="E85" s="46">
         <f t="shared" si="3"/>
-        <v>2.0180820825515946E-2</v>
+        <v>1.8386970085470085E-2</v>
       </c>
     </row>
     <row r="86" spans="2:175" x14ac:dyDescent="0.25">
@@ -8131,7 +8131,7 @@
       </c>
       <c r="E86" s="20">
         <f t="shared" si="3"/>
-        <v>9.7181535334584113E-3</v>
+        <v>8.8543176638176627E-3</v>
       </c>
     </row>
     <row r="87" spans="2:175" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -8146,7 +8146,7 @@
       </c>
       <c r="E87" s="18">
         <f t="shared" si="3"/>
-        <v>1.2100969355847405E-3</v>
+        <v>1.1025327635327635E-3</v>
       </c>
       <c r="F87" s="18"/>
       <c r="G87" s="18"/>
@@ -8326,11 +8326,11 @@
       </c>
       <c r="D88" s="34">
         <f>D5</f>
-        <v>4000</v>
+        <v>15000</v>
       </c>
       <c r="E88" s="20">
         <f t="shared" si="3"/>
-        <v>6.5040650406504072E-2</v>
+        <v>0.22222222222222221</v>
       </c>
     </row>
     <row r="89" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8344,7 +8344,7 @@
       </c>
       <c r="E89" s="20">
         <f t="shared" si="3"/>
-        <v>4.6830519074421504E-4</v>
+        <v>4.2667806267806261E-4</v>
       </c>
     </row>
     <row r="90" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8400,7 +8400,7 @@
       </c>
       <c r="E93" s="20">
         <f t="shared" si="3"/>
-        <v>4.3944027517198246E-4</v>
+        <v>4.0037891737891736E-4</v>
       </c>
     </row>
     <row r="94" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8509,11 +8509,11 @@
       <c r="C101" s="48"/>
       <c r="D101" s="49">
         <f>SUM(D53:D100)</f>
-        <v>10667.377403846154</v>
+        <v>21667.377403846152</v>
       </c>
       <c r="E101" s="50">
         <f t="shared" si="3"/>
-        <v>0.17345329111944965</v>
+        <v>0.32099818376068373</v>
       </c>
       <c r="F101" s="50"/>
       <c r="G101" s="50"/>
@@ -8540,7 +8540,7 @@
       </c>
       <c r="E104" s="20">
         <f t="shared" ref="E104:E130" si="4">D104/D$36</f>
-        <v>5.528369449656035E-2</v>
+        <v>5.0369588319088318E-2</v>
       </c>
     </row>
     <row r="105" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8554,7 +8554,7 @@
       </c>
       <c r="E105" s="20">
         <f t="shared" si="4"/>
-        <v>7.979987492182615E-4</v>
+        <v>7.2706552706552712E-4</v>
       </c>
     </row>
     <row r="106" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8568,7 +8568,7 @@
       </c>
       <c r="E106" s="20">
         <f t="shared" si="4"/>
-        <v>1.2138747654784241E-2</v>
+        <v>1.1059747863247864E-2</v>
       </c>
     </row>
     <row r="107" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8582,7 +8582,7 @@
       </c>
       <c r="E107" s="20">
         <f t="shared" si="4"/>
-        <v>9.7480300187617261E-4</v>
+        <v>8.8815384615384613E-4</v>
       </c>
     </row>
     <row r="108" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8596,7 +8596,7 @@
       </c>
       <c r="E108" s="20">
         <f t="shared" si="4"/>
-        <v>2.2612629768605379E-2</v>
+        <v>2.0602618233618232E-2</v>
       </c>
     </row>
     <row r="109" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8610,7 +8610,7 @@
       </c>
       <c r="E109" s="20">
         <f t="shared" si="4"/>
-        <v>5.2281425891181985E-4</v>
+        <v>4.7634188034188037E-4</v>
       </c>
     </row>
     <row r="110" spans="2:175" x14ac:dyDescent="0.25">
@@ -8639,7 +8639,7 @@
       </c>
       <c r="E111" s="20">
         <f t="shared" si="4"/>
-        <v>2.5033302063789866E-4</v>
+        <v>2.2808119658119657E-4</v>
       </c>
     </row>
     <row r="112" spans="2:175" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -8654,7 +8654,7 @@
       </c>
       <c r="E112" s="18">
         <f t="shared" si="4"/>
-        <v>1.1616635397123202E-6</v>
+        <v>1.0584045584045585E-6</v>
       </c>
       <c r="F112" s="18"/>
       <c r="G112" s="18"/>
@@ -8838,7 +8838,7 @@
       </c>
       <c r="E113" s="20">
         <f t="shared" si="4"/>
-        <v>1.0830362726704189E-4</v>
+        <v>9.8676638176638178E-5</v>
       </c>
     </row>
     <row r="114" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8866,7 +8866,7 @@
       </c>
       <c r="E115" s="20">
         <f t="shared" si="4"/>
-        <v>-2.1332082551594746E-5</v>
+        <v>-1.9435897435897435E-5</v>
       </c>
     </row>
     <row r="116" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8880,7 +8880,7 @@
       </c>
       <c r="E116" s="20">
         <f t="shared" si="4"/>
-        <v>3.3745669168230145E-3</v>
+        <v>3.0746054131054134E-3</v>
       </c>
     </row>
     <row r="117" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8894,7 +8894,7 @@
       </c>
       <c r="E117" s="20">
         <f t="shared" si="4"/>
-        <v>6.9170262664165099E-4</v>
+        <v>6.3021794871794868E-4</v>
       </c>
     </row>
     <row r="118" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8908,7 +8908,7 @@
       </c>
       <c r="E118" s="20">
         <f t="shared" si="4"/>
-        <v>1.7354596622889307E-5</v>
+        <v>1.5811965811965812E-5</v>
       </c>
     </row>
     <row r="119" spans="2:175" x14ac:dyDescent="0.25">
@@ -8923,7 +8923,7 @@
       </c>
       <c r="E119" s="46">
         <f t="shared" si="4"/>
-        <v>2.3314258911819887E-3</v>
+        <v>2.1241880341880343E-3</v>
       </c>
     </row>
     <row r="120" spans="2:175" x14ac:dyDescent="0.25">
@@ -8952,7 +8952,7 @@
       </c>
       <c r="E121" s="18">
         <f t="shared" si="4"/>
-        <v>7.817385866166354E-5</v>
+        <v>7.122507122507122E-5</v>
       </c>
       <c r="F121" s="18"/>
       <c r="G121" s="18"/>
@@ -9137,7 +9137,7 @@
       </c>
       <c r="E122" s="46">
         <f t="shared" si="4"/>
-        <v>1.4293308317698561E-5</v>
+        <v>1.3022792022792023E-5</v>
       </c>
     </row>
     <row r="123" spans="2:175" x14ac:dyDescent="0.25">
@@ -9151,7 +9151,7 @@
       </c>
       <c r="E123" s="20">
         <f t="shared" si="4"/>
-        <v>1.2375390869293309E-4</v>
+        <v>1.1275356125356125E-4</v>
       </c>
     </row>
     <row r="124" spans="2:175" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -9166,7 +9166,7 @@
       </c>
       <c r="E124" s="18">
         <f t="shared" si="4"/>
-        <v>1.0226250781738588E-3</v>
+        <v>9.317250712250712E-4</v>
       </c>
       <c r="F124" s="18"/>
       <c r="G124" s="18"/>
@@ -9350,7 +9350,7 @@
       </c>
       <c r="E125" s="20">
         <f t="shared" si="4"/>
-        <v>3.2016765165728579E-2</v>
+        <v>2.9170830484330484E-2</v>
       </c>
     </row>
     <row r="126" spans="2:175" x14ac:dyDescent="0.25">
@@ -9365,7 +9365,7 @@
       </c>
       <c r="E126" s="46">
         <f t="shared" si="4"/>
-        <v>2.3143308317698564E-3</v>
+        <v>2.1086125356125358E-3</v>
       </c>
     </row>
     <row r="127" spans="2:175" x14ac:dyDescent="0.25">
@@ -9379,7 +9379,7 @@
       </c>
       <c r="E127" s="20">
         <f t="shared" si="4"/>
-        <v>3.3720919324577864E-4</v>
+        <v>3.0723504273504271E-4</v>
       </c>
     </row>
     <row r="128" spans="2:175" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -9593,7 +9593,7 @@
       </c>
       <c r="E130" s="50">
         <f t="shared" si="4"/>
-        <v>0.13499135553470915</v>
+        <v>0.1229921239316239</v>
       </c>
       <c r="F130" s="50"/>
       <c r="G130" s="50"/>
@@ -9620,7 +9620,7 @@
       </c>
       <c r="E133" s="20">
         <f t="shared" ref="E133:E141" si="5">D133/D$36</f>
-        <v>5.9640243902439019E-4</v>
+        <v>5.4338888888888883E-4</v>
       </c>
     </row>
     <row r="134" spans="2:7" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -9634,7 +9634,7 @@
       </c>
       <c r="E134" s="20">
         <f t="shared" si="5"/>
-        <v>4.275437773608505E-4</v>
+        <v>3.8953988603988599E-4</v>
       </c>
     </row>
     <row r="135" spans="2:7" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -9662,7 +9662,7 @@
       </c>
       <c r="E136" s="20">
         <f t="shared" si="5"/>
-        <v>4.1204377736085056E-3</v>
+        <v>3.7541766381766384E-3</v>
       </c>
     </row>
     <row r="137" spans="2:7" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -9676,7 +9676,7 @@
       </c>
       <c r="E137" s="20">
         <f t="shared" si="5"/>
-        <v>7.0741088180112572E-4</v>
+        <v>6.445299145299146E-4</v>
       </c>
     </row>
     <row r="138" spans="2:7" x14ac:dyDescent="0.25">
@@ -9691,7 +9691,7 @@
       </c>
       <c r="E138" s="46">
         <f t="shared" si="5"/>
-        <v>4.423975922451532E-3</v>
+        <v>4.0307336182336178E-3</v>
       </c>
     </row>
     <row r="139" spans="2:7" x14ac:dyDescent="0.25">
@@ -9735,7 +9735,7 @@
       </c>
       <c r="E141" s="50">
         <f t="shared" si="5"/>
-        <v>1.0275770794246403E-2</v>
+        <v>9.3623689458689451E-3</v>
       </c>
       <c r="F141" s="50"/>
       <c r="G141" s="50"/>
@@ -9782,7 +9782,7 @@
       </c>
       <c r="E145" s="58">
         <f t="shared" si="6"/>
-        <v>7.1371175734834272E-2</v>
+        <v>6.5027071225071231E-2</v>
       </c>
     </row>
     <row r="146" spans="2:7" x14ac:dyDescent="0.25">
@@ -9812,7 +9812,7 @@
       </c>
       <c r="E147" s="58">
         <f t="shared" si="6"/>
-        <v>3.5872201375859911E-3</v>
+        <v>3.2683561253561253E-3</v>
       </c>
     </row>
     <row r="148" spans="2:7" x14ac:dyDescent="0.25">
@@ -9857,7 +9857,7 @@
       </c>
       <c r="E150" s="58">
         <f t="shared" si="6"/>
-        <v>2.3669297998749221E-2</v>
+        <v>2.1565360398860402E-2</v>
       </c>
     </row>
     <row r="151" spans="2:7" x14ac:dyDescent="0.25">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="E151" s="58">
         <f t="shared" si="6"/>
-        <v>8.7919199499687292E-3</v>
+        <v>8.0104159544159542E-3</v>
       </c>
     </row>
     <row r="152" spans="2:7" x14ac:dyDescent="0.25">
@@ -9883,7 +9883,7 @@
       <c r="C152" s="48"/>
       <c r="D152" s="49">
         <f>E152*D10</f>
-        <v>3690</v>
+        <v>4050</v>
       </c>
       <c r="E152" s="50">
         <v>0.06</v>
@@ -9948,7 +9948,7 @@
       </c>
       <c r="E157" s="58">
         <f t="shared" si="7"/>
-        <v>-5.1719824890556595E-6</v>
+        <v>-4.7122507122507113E-6</v>
       </c>
     </row>
     <row r="158" spans="2:7" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
       <c r="C167" s="56"/>
       <c r="D167" s="57">
         <f>E167*D10</f>
-        <v>-2029.5</v>
+        <v>-2227.5</v>
       </c>
       <c r="E167" s="58">
         <v>-3.3000000000000002E-2</v>
@@ -10168,11 +10168,11 @@
       <c r="C172" s="48"/>
       <c r="D172" s="49">
         <f>SUM(D155:D171)</f>
-        <v>-2029.8180769230769</v>
+        <v>-2227.8180769230771</v>
       </c>
       <c r="E172" s="50">
         <f t="shared" si="7"/>
-        <v>-3.3005171982489055E-2</v>
+        <v>-3.3004712250712255E-2</v>
       </c>
       <c r="F172" s="50"/>
       <c r="G172" s="50"/>
@@ -10219,7 +10219,7 @@
       </c>
       <c r="E176" s="58">
         <f t="shared" si="8"/>
-        <v>1.0736260162601626E-2</v>
+        <v>9.7819259259259248E-3</v>
       </c>
     </row>
     <row r="177" spans="2:5" x14ac:dyDescent="0.25">
@@ -10234,7 +10234,7 @@
       </c>
       <c r="E177" s="58">
         <f t="shared" si="8"/>
-        <v>9.2391480612883048E-2</v>
+        <v>8.4178904558404558E-2</v>
       </c>
     </row>
     <row r="178" spans="2:5" x14ac:dyDescent="0.25">
@@ -10249,7 +10249,7 @@
       </c>
       <c r="E178" s="58">
         <f t="shared" si="8"/>
-        <v>1.1569731081926204E-5</v>
+        <v>1.0541310541310541E-5</v>
       </c>
     </row>
     <row r="179" spans="2:5" x14ac:dyDescent="0.25">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="E179" s="58">
         <f t="shared" si="8"/>
-        <v>2.461225766103815E-3</v>
+        <v>2.2424501424501424E-3</v>
       </c>
     </row>
     <row r="180" spans="2:5" x14ac:dyDescent="0.25">
@@ -10279,7 +10279,7 @@
       </c>
       <c r="E180" s="58">
         <f t="shared" si="8"/>
-        <v>2.3804409005628518E-4</v>
+        <v>2.168846153846154E-4</v>
       </c>
     </row>
     <row r="181" spans="2:5" x14ac:dyDescent="0.25">
@@ -10294,7 +10294,7 @@
       </c>
       <c r="E181" s="58">
         <f t="shared" si="8"/>
-        <v>6.2061350844277666E-3</v>
+        <v>5.6544786324786321E-3</v>
       </c>
     </row>
     <row r="182" spans="2:5" x14ac:dyDescent="0.25">
@@ -10339,7 +10339,7 @@
       </c>
       <c r="E184" s="58">
         <f t="shared" si="8"/>
-        <v>7.5434646654158846E-5</v>
+        <v>6.8729344729344732E-5</v>
       </c>
     </row>
     <row r="185" spans="2:5" x14ac:dyDescent="0.25">
@@ -10594,7 +10594,7 @@
       </c>
       <c r="E201" s="50">
         <f t="shared" si="8"/>
-        <v>0.11212015009380862</v>
+        <v>0.10215391452991451</v>
       </c>
       <c r="F201" s="50"/>
       <c r="G201" s="50"/>
@@ -10612,11 +10612,11 @@
       <c r="C203" s="48"/>
       <c r="D203" s="49">
         <f>D43-D50-D101-D130-D141-D152-D172-D201</f>
-        <v>1587.880192307699</v>
+        <v>-4739.9198076922985</v>
       </c>
       <c r="E203" s="50">
         <f>D203/D36</f>
-        <v>2.5819190118824373E-2</v>
+        <v>-7.0221034188034048E-2</v>
       </c>
       <c r="F203" s="50"/>
       <c r="G203" s="50"/>
@@ -10642,7 +10642,7 @@
       <c r="C207" s="63"/>
       <c r="D207" s="64">
         <f>E203</f>
-        <v>2.5819190118824373E-2</v>
+        <v>-7.0221034188034048E-2</v>
       </c>
     </row>
     <row r="208" spans="2:175" s="20" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Flash v5.14: MILA OPEX refresh, CC fees % in G&A, week compare grid
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/excel/ebidta-calculation-mila-lounge.xlsx
+++ b/data/excel/ebidta-calculation-mila-lounge.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MatthiasLavenant\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9206479A-0069-4734-A499-938135B83D28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA0A10D2-8EB8-4B68-B921-D8A3C17DB4D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="855" windowWidth="29040" windowHeight="15720" xr2:uid="{3C90C578-B115-41AD-8F85-41FE68FE49FA}"/>
   </bookViews>
@@ -5579,6 +5579,55 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="12">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="3">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{0D1FC6E1-D2B9-4DAA-84B1-687CE5E9F7F4}">
+  <we:reference id="WA200009404" version="1.0.0.8" store="Omex" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="WA200009404" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;2d62813f-d039-4fcf-bf65-91c64db4909c&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+  <we:extLst>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
+      <we:containsCustomFunctions/>
+    </a:ext>
+  </we:extLst>
+</we:webextension>
+</file>
+
+<file path=xl/webextensions/webextension2.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{D09D00BA-4115-4719-8340-4946343EAEF0}">
+  <we:reference id="WA200010725" version="1.0.0.1" store="Omex" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200010725" version="1.0.0.1" store="WA200010725" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;0274738e-1f28-498a-8004-0266299e1695&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+  <we:extLst>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
+      <we:containsCustomFunctions/>
+    </a:ext>
+  </we:extLst>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B26BDD18-EC06-4B8C-8F68-C4E97E1A8EA4}">
   <sheetPr>
@@ -6813,7 +6862,7 @@
       </c>
       <c r="C10" s="22"/>
       <c r="D10" s="23">
-        <v>67500</v>
+        <v>61000</v>
       </c>
       <c r="E10" s="23"/>
       <c r="W10">
@@ -7121,7 +7170,7 @@
       </c>
       <c r="D33" s="34">
         <f>D$36*E33</f>
-        <v>41850</v>
+        <v>37820</v>
       </c>
       <c r="E33" s="20">
         <v>0.62</v>
@@ -7133,7 +7182,7 @@
       </c>
       <c r="D34" s="34">
         <f t="shared" ref="D34" si="0">D$36*E34</f>
-        <v>22950</v>
+        <v>20740</v>
       </c>
       <c r="E34" s="20">
         <f>E36-E33-E35</f>
@@ -7146,7 +7195,7 @@
       </c>
       <c r="D35" s="34">
         <f>D$36*E35</f>
-        <v>2700</v>
+        <v>2440</v>
       </c>
       <c r="E35" s="20">
         <v>0.04</v>
@@ -7159,7 +7208,7 @@
       <c r="C36" s="22"/>
       <c r="D36" s="45">
         <f>D10</f>
-        <v>67500</v>
+        <v>61000</v>
       </c>
       <c r="E36" s="46">
         <v>1</v>
@@ -7174,7 +7223,7 @@
       </c>
       <c r="D38" s="34">
         <f>E38*D33</f>
-        <v>6277.5</v>
+        <v>5673</v>
       </c>
       <c r="E38" s="20">
         <v>0.15</v>
@@ -7186,7 +7235,7 @@
       </c>
       <c r="D39" s="34">
         <f t="shared" ref="D39:D40" si="1">E39*D34</f>
-        <v>6081.75</v>
+        <v>5496.1</v>
       </c>
       <c r="E39" s="20">
         <v>0.26500000000000001</v>
@@ -7198,7 +7247,7 @@
       </c>
       <c r="D40" s="34">
         <f t="shared" si="1"/>
-        <v>756.00000000000011</v>
+        <v>683.2</v>
       </c>
       <c r="E40" s="20">
         <v>0.28000000000000003</v>
@@ -7211,11 +7260,11 @@
       <c r="C41" s="22"/>
       <c r="D41" s="45">
         <f>SUM(D38:D40)</f>
-        <v>13115.25</v>
+        <v>11852.300000000001</v>
       </c>
       <c r="E41" s="46">
         <f>D41/D36</f>
-        <v>0.1943</v>
+        <v>0.19430000000000003</v>
       </c>
     </row>
     <row r="42" spans="2:175" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
@@ -7228,7 +7277,7 @@
       <c r="C43" s="22"/>
       <c r="D43" s="45">
         <f>D36-D41</f>
-        <v>54384.75</v>
+        <v>49147.7</v>
       </c>
       <c r="E43" s="46">
         <f>D43/D36</f>
@@ -7417,12 +7466,12 @@
         <v>22</v>
       </c>
       <c r="D46" s="34">
-        <f>'OPEX DATA 2'!U139+'OPEX DATA 2'!U141+'OPEX DATA 2'!U142</f>
-        <v>7603.3156730769233</v>
+        <f>'OPEX DATA 2'!U143</f>
+        <v>5487.53467032967</v>
       </c>
       <c r="E46" s="20">
         <f>D46/D$36</f>
-        <v>0.11264171367521368</v>
+        <v>8.9959584759502789E-2</v>
       </c>
     </row>
     <row r="47" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7430,25 +7479,22 @@
         <v>23</v>
       </c>
       <c r="D47" s="34">
-        <f>'OPEX DATA 2'!U123+'OPEX DATA 2'!U97+'OPEX DATA 2'!U98+'OPEX DATA 2'!U110+'OPEX DATA 2'!U112</f>
-        <v>2491.1234615384615</v>
+        <f>'OPEX DATA 2'!U119</f>
+        <v>3354.3092857142851</v>
       </c>
       <c r="E47" s="20">
         <f t="shared" ref="E47:E50" si="2">D47/D$36</f>
-        <v>3.6905532763532763E-2</v>
+        <v>5.4988676814988278E-2</v>
       </c>
     </row>
     <row r="48" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B48" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D48" s="34">
-        <f>'OPEX DATA 2'!U85+'OPEX DATA 2'!U86+'OPEX DATA 2'!U87+'OPEX DATA 2'!U88+'OPEX DATA 2'!U92+'OPEX DATA 2'!U124</f>
-        <v>5336.3762500000003</v>
-      </c>
+      <c r="D48" s="34"/>
       <c r="E48" s="20">
         <f t="shared" si="2"/>
-        <v>7.9057425925925934E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7456,12 +7502,12 @@
         <v>25</v>
       </c>
       <c r="D49" s="34">
-        <f>'OPEX DATA 2'!U151+'OPEX DATA 2'!U153+'OPEX DATA 2'!U154</f>
-        <v>4374.9775961538462</v>
+        <f>'OPEX DATA 2'!U151</f>
+        <v>2038.0992307692306</v>
       </c>
       <c r="E49" s="20">
         <f t="shared" si="2"/>
-        <v>6.4814482905982906E-2</v>
+        <v>3.3411462799495584E-2</v>
       </c>
     </row>
     <row r="50" spans="2:175" x14ac:dyDescent="0.25">
@@ -7471,11 +7517,11 @@
       <c r="C50" s="22"/>
       <c r="D50" s="45">
         <f>SUM(D46:D49)</f>
-        <v>19805.792980769231</v>
+        <v>10879.943186813185</v>
       </c>
       <c r="E50" s="46">
         <f t="shared" si="2"/>
-        <v>0.29341915527065526</v>
+        <v>0.17835972437398664</v>
       </c>
     </row>
     <row r="52" spans="2:175" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -7664,11 +7710,11 @@
       </c>
       <c r="D53" s="34">
         <f>'OPEX DATA 2'!U161</f>
-        <v>0.26999999999999996</v>
+        <v>0.15428571428571428</v>
       </c>
       <c r="E53" s="20">
         <f t="shared" ref="E53:E101" si="3">D53/D$36</f>
-        <v>3.9999999999999998E-6</v>
+        <v>2.5292740046838404E-6</v>
       </c>
     </row>
     <row r="54" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7678,11 +7724,11 @@
       </c>
       <c r="D54" s="34">
         <f>'OPEX DATA 2'!U162</f>
-        <v>152.5126923076923</v>
+        <v>87.150109890109889</v>
       </c>
       <c r="E54" s="20">
         <f t="shared" si="3"/>
-        <v>2.2594472934472933E-3</v>
+        <v>1.4286903260673752E-3</v>
       </c>
     </row>
     <row r="55" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7692,11 +7738,11 @@
       </c>
       <c r="D55" s="34">
         <f>'OPEX DATA 2'!U163</f>
-        <v>245.6385576923077</v>
+        <v>140.36489010989013</v>
       </c>
       <c r="E55" s="20">
         <f t="shared" si="3"/>
-        <v>3.6390897435897439E-3</v>
+        <v>2.3010637722932809E-3</v>
       </c>
     </row>
     <row r="56" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7706,11 +7752,11 @@
       </c>
       <c r="D56" s="34">
         <f>'OPEX DATA 2'!U164</f>
-        <v>38.466538461538462</v>
+        <v>21.98087912087912</v>
       </c>
       <c r="E56" s="20">
         <f t="shared" si="3"/>
-        <v>5.6987464387464387E-4</v>
+        <v>3.6034228067014949E-4</v>
       </c>
     </row>
     <row r="57" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7720,11 +7766,11 @@
       </c>
       <c r="D57" s="34">
         <f>'OPEX DATA 2'!U165</f>
-        <v>41.174038461538458</v>
+        <v>23.528021978021975</v>
       </c>
       <c r="E57" s="20">
         <f t="shared" si="3"/>
-        <v>6.0998575498575497E-4</v>
+        <v>3.8570527832822908E-4</v>
       </c>
     </row>
     <row r="58" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7734,11 +7780,11 @@
       </c>
       <c r="D58" s="34">
         <f>'OPEX DATA 2'!U166</f>
-        <v>230.69173076923079</v>
+        <v>131.82384615384618</v>
       </c>
       <c r="E58" s="20">
         <f t="shared" si="3"/>
-        <v>3.4176552706552711E-3</v>
+        <v>2.1610466582597733E-3</v>
       </c>
     </row>
     <row r="59" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7748,11 +7794,11 @@
       </c>
       <c r="D59" s="34">
         <f>'OPEX DATA 2'!U167</f>
-        <v>173.01663461538465</v>
+        <v>98.866648351648365</v>
       </c>
       <c r="E59" s="20">
         <f t="shared" si="3"/>
-        <v>2.5632094017094022E-3</v>
+        <v>1.6207647270762026E-3</v>
       </c>
     </row>
     <row r="60" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7762,11 +7808,11 @@
       </c>
       <c r="D60" s="34">
         <f>'OPEX DATA 2'!U168</f>
-        <v>708.65326923076941</v>
+        <v>404.94472527472539</v>
       </c>
       <c r="E60" s="20">
         <f t="shared" si="3"/>
-        <v>1.0498566951566955E-2</v>
+        <v>6.6384381192577929E-3</v>
       </c>
     </row>
     <row r="61" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7776,11 +7822,11 @@
       </c>
       <c r="D61" s="34">
         <f>'OPEX DATA 2'!U169</f>
-        <v>35.989230769230772</v>
+        <v>20.565274725274726</v>
       </c>
       <c r="E61" s="20">
         <f t="shared" si="3"/>
-        <v>5.3317378917378921E-4</v>
+        <v>3.3713565123401188E-4</v>
       </c>
     </row>
     <row r="62" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7790,11 +7836,11 @@
       </c>
       <c r="D62" s="34">
         <f>'OPEX DATA 2'!U170</f>
-        <v>252.62173076923077</v>
+        <v>144.35527472527471</v>
       </c>
       <c r="E62" s="20">
         <f t="shared" si="3"/>
-        <v>3.7425441595441596E-3</v>
+        <v>2.3664799135290934E-3</v>
       </c>
     </row>
     <row r="63" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7804,11 +7850,11 @@
       </c>
       <c r="D63" s="34">
         <f>'OPEX DATA 2'!U171</f>
-        <v>279.36682692307693</v>
+        <v>159.63818681318682</v>
       </c>
       <c r="E63" s="20">
         <f t="shared" si="3"/>
-        <v>4.1387678062678067E-3</v>
+        <v>2.6170194559538822E-3</v>
       </c>
     </row>
     <row r="64" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7860,11 +7906,11 @@
       </c>
       <c r="D67" s="34">
         <f>'OPEX DATA 2'!U175</f>
-        <v>270.21471153846153</v>
+        <v>154.4084065934066</v>
       </c>
       <c r="E67" s="20">
         <f t="shared" si="3"/>
-        <v>4.0031809116809116E-3</v>
+        <v>2.5312853539902719E-3</v>
       </c>
     </row>
     <row r="68" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7874,11 +7920,11 @@
       </c>
       <c r="D68" s="34">
         <f>'OPEX DATA 2'!U176</f>
-        <v>258.85000000000002</v>
+        <v>147.91428571428574</v>
       </c>
       <c r="E68" s="20">
         <f t="shared" si="3"/>
-        <v>3.8348148148148152E-3</v>
+        <v>2.4248243559718973E-3</v>
       </c>
     </row>
     <row r="69" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7888,11 +7934,11 @@
       </c>
       <c r="D69" s="34">
         <f>'OPEX DATA 2'!U177</f>
-        <v>208.93653846153845</v>
+        <v>119.39230769230768</v>
       </c>
       <c r="E69" s="20">
         <f t="shared" si="3"/>
-        <v>3.0953561253561253E-3</v>
+        <v>1.9572509457755358E-3</v>
       </c>
     </row>
     <row r="70" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7902,11 +7948,11 @@
       </c>
       <c r="D70" s="34">
         <f>'OPEX DATA 2'!U178</f>
-        <v>297.10875000000004</v>
+        <v>169.7764285714286</v>
       </c>
       <c r="E70" s="20">
         <f t="shared" si="3"/>
-        <v>4.4016111111111113E-3</v>
+        <v>2.783220140515223E-3</v>
       </c>
     </row>
     <row r="71" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7916,11 +7962,11 @@
       </c>
       <c r="D71" s="34">
         <f>'OPEX DATA 2'!U179</f>
-        <v>99.572884615384609</v>
+        <v>56.898791208791202</v>
       </c>
       <c r="E71" s="20">
         <f t="shared" si="3"/>
-        <v>1.4751538461538461E-3</v>
+        <v>9.3276706899657704E-4</v>
       </c>
     </row>
     <row r="72" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7930,11 +7976,11 @@
       </c>
       <c r="D72" s="34">
         <f>'OPEX DATA 2'!U180</f>
-        <v>523.67298076923078</v>
+        <v>299.24170329670329</v>
       </c>
       <c r="E72" s="20">
         <f t="shared" si="3"/>
-        <v>7.7581182336182337E-3</v>
+        <v>4.9056016933885782E-3</v>
       </c>
     </row>
     <row r="73" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7958,11 +8004,11 @@
       </c>
       <c r="D74" s="34">
         <f>'OPEX DATA 2'!U182</f>
-        <v>3.8412500000000001</v>
+        <v>2.1949999999999998</v>
       </c>
       <c r="E74" s="20">
         <f t="shared" si="3"/>
-        <v>5.6907407407407407E-5</v>
+        <v>3.598360655737705E-5</v>
       </c>
     </row>
     <row r="75" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7972,11 +8018,11 @@
       </c>
       <c r="D75" s="34">
         <f>'OPEX DATA 2'!U183</f>
-        <v>146.51663461538462</v>
+        <v>83.723791208791212</v>
       </c>
       <c r="E75" s="20">
         <f t="shared" si="3"/>
-        <v>2.1706168091168094E-3</v>
+        <v>1.3725211673572329E-3</v>
       </c>
     </row>
     <row r="76" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7986,11 +8032,11 @@
       </c>
       <c r="D76" s="34">
         <f>'OPEX DATA 2'!U184</f>
-        <v>51.022403846153843</v>
+        <v>29.155659340659337</v>
       </c>
       <c r="E76" s="20">
         <f t="shared" si="3"/>
-        <v>7.5588746438746436E-4</v>
+        <v>4.7796162853539897E-4</v>
       </c>
     </row>
     <row r="77" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8028,11 +8074,11 @@
       </c>
       <c r="D79" s="34">
         <f>'OPEX DATA 2'!U187</f>
-        <v>20.997211538461539</v>
+        <v>11.998406593406594</v>
       </c>
       <c r="E79" s="20">
         <f t="shared" si="3"/>
-        <v>3.1106980056980058E-4</v>
+        <v>1.966951900558458E-4</v>
       </c>
     </row>
     <row r="80" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8042,11 +8088,11 @@
       </c>
       <c r="D80" s="34">
         <f>'OPEX DATA 2'!U188</f>
-        <v>179.06451923076924</v>
+        <v>102.32258241758242</v>
       </c>
       <c r="E80" s="20">
         <f t="shared" si="3"/>
-        <v>2.6528076923076926E-3</v>
+        <v>1.6774193838947939E-3</v>
       </c>
     </row>
     <row r="81" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8056,11 +8102,11 @@
       </c>
       <c r="D81" s="34">
         <f>'OPEX DATA 2'!U189</f>
-        <v>298.44461538461536</v>
+        <v>170.5397802197802</v>
       </c>
       <c r="E81" s="20">
         <f t="shared" si="3"/>
-        <v>4.4214017094017094E-3</v>
+        <v>2.7957341019636097E-3</v>
       </c>
     </row>
     <row r="82" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8070,11 +8116,11 @@
       </c>
       <c r="D82" s="34">
         <f>'OPEX DATA 2'!U190</f>
-        <v>11.956250000000001</v>
+        <v>6.8321428571428573</v>
       </c>
       <c r="E82" s="20">
         <f t="shared" si="3"/>
-        <v>1.7712962962962965E-4</v>
+        <v>1.1200234192037471E-4</v>
       </c>
     </row>
     <row r="83" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8098,11 +8144,11 @@
       </c>
       <c r="D84" s="34">
         <f>'OPEX DATA 2'!U192</f>
-        <v>169.74317307692309</v>
+        <v>96.996098901098904</v>
       </c>
       <c r="E84" s="20">
         <f t="shared" si="3"/>
-        <v>2.5147136752136754E-3</v>
+        <v>1.5900999819852279E-3</v>
       </c>
     </row>
     <row r="85" spans="2:175" x14ac:dyDescent="0.25">
@@ -8113,11 +8159,11 @@
       <c r="C85" s="22"/>
       <c r="D85" s="45">
         <f>'OPEX DATA 2'!U193</f>
-        <v>1241.1204807692307</v>
+        <v>709.21170329670326</v>
       </c>
       <c r="E85" s="46">
         <f t="shared" si="3"/>
-        <v>1.8386970085470085E-2</v>
+        <v>1.1626421365519725E-2</v>
       </c>
     </row>
     <row r="86" spans="2:175" x14ac:dyDescent="0.25">
@@ -8127,11 +8173,11 @@
       </c>
       <c r="D86" s="34">
         <f>'OPEX DATA 2'!U194</f>
-        <v>597.66644230769225</v>
+        <v>341.52368131868127</v>
       </c>
       <c r="E86" s="20">
         <f t="shared" si="3"/>
-        <v>8.8543176638176627E-3</v>
+        <v>5.5987488740767422E-3</v>
       </c>
     </row>
     <row r="87" spans="2:175" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -8142,11 +8188,11 @@
       <c r="C87" s="2"/>
       <c r="D87" s="28">
         <f>'OPEX DATA 2'!U195</f>
-        <v>74.42096153846154</v>
+        <v>42.526263736263736</v>
       </c>
       <c r="E87" s="18">
         <f t="shared" si="3"/>
-        <v>1.1025327635327635E-3</v>
+        <v>6.9715186452891376E-4</v>
       </c>
       <c r="F87" s="18"/>
       <c r="G87" s="18"/>
@@ -8330,7 +8376,7 @@
       </c>
       <c r="E88" s="20">
         <f t="shared" si="3"/>
-        <v>0.22222222222222221</v>
+        <v>0.24590163934426229</v>
       </c>
     </row>
     <row r="89" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8340,11 +8386,11 @@
       </c>
       <c r="D89" s="34">
         <f>'OPEX DATA 2'!U197</f>
-        <v>28.800769230769227</v>
+        <v>16.457582417582415</v>
       </c>
       <c r="E89" s="20">
         <f t="shared" si="3"/>
-        <v>4.2667806267806261E-4</v>
+        <v>2.6979643307512154E-4</v>
       </c>
     </row>
     <row r="90" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8396,11 +8442,11 @@
       </c>
       <c r="D93" s="34">
         <f>'OPEX DATA 2'!U201</f>
-        <v>27.025576923076922</v>
+        <v>15.443186813186813</v>
       </c>
       <c r="E93" s="20">
         <f t="shared" si="3"/>
-        <v>4.0037891737891736E-4</v>
+        <v>2.5316699693748876E-4</v>
       </c>
     </row>
     <row r="94" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8509,11 +8555,11 @@
       <c r="C101" s="48"/>
       <c r="D101" s="49">
         <f>SUM(D53:D100)</f>
-        <v>21667.377403846152</v>
+        <v>18809.929945054944</v>
       </c>
       <c r="E101" s="50">
         <f t="shared" si="3"/>
-        <v>0.32099818376068373</v>
+        <v>0.30835950729598272</v>
       </c>
       <c r="F101" s="50"/>
       <c r="G101" s="50"/>
@@ -8535,12 +8581,11 @@
         <v>7010 - Credit Card Fees</v>
       </c>
       <c r="D104" s="34">
-        <f>'OPEX DATA 2'!U215</f>
-        <v>3399.9472115384615</v>
+        <f>E104*D36</f>
+        <v>2013</v>
       </c>
       <c r="E104" s="20">
-        <f t="shared" ref="E104:E130" si="4">D104/D$36</f>
-        <v>5.0369588319088318E-2</v>
+        <v>3.3000000000000002E-2</v>
       </c>
     </row>
     <row r="105" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8550,11 +8595,11 @@
       </c>
       <c r="D105" s="34">
         <f>'OPEX DATA 2'!U216</f>
-        <v>49.07692307692308</v>
+        <v>28.043956043956047</v>
       </c>
       <c r="E105" s="20">
-        <f t="shared" si="4"/>
-        <v>7.2706552706552712E-4</v>
+        <f t="shared" ref="E104:E130" si="4">D105/D$36</f>
+        <v>4.597369843271483E-4</v>
       </c>
     </row>
     <row r="106" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8564,11 +8609,11 @@
       </c>
       <c r="D106" s="34">
         <f>'OPEX DATA 2'!U217</f>
-        <v>746.53298076923079</v>
+        <v>426.59027472527475</v>
       </c>
       <c r="E106" s="20">
         <f t="shared" si="4"/>
-        <v>1.1059747863247864E-2</v>
+        <v>6.9932831922176189E-3</v>
       </c>
     </row>
     <row r="107" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8578,11 +8623,11 @@
       </c>
       <c r="D107" s="34">
         <f>'OPEX DATA 2'!U218</f>
-        <v>59.950384615384614</v>
+        <v>34.25736263736264</v>
       </c>
       <c r="E107" s="20">
         <f t="shared" si="4"/>
-        <v>8.8815384615384613E-4</v>
+        <v>5.615961088092236E-4</v>
       </c>
     </row>
     <row r="108" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8592,11 +8637,11 @@
       </c>
       <c r="D108" s="34">
         <f>'OPEX DATA 2'!U219</f>
-        <v>1390.6767307692307</v>
+        <v>794.67241758241755</v>
       </c>
       <c r="E108" s="20">
         <f t="shared" si="4"/>
-        <v>2.0602618233618232E-2</v>
+        <v>1.3027416681678975E-2</v>
       </c>
     </row>
     <row r="109" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8606,11 +8651,11 @@
       </c>
       <c r="D109" s="34">
         <f>'OPEX DATA 2'!U220</f>
-        <v>32.153076923076924</v>
+        <v>18.373186813186813</v>
       </c>
       <c r="E109" s="20">
         <f t="shared" si="4"/>
-        <v>4.7634188034188037E-4</v>
+        <v>3.0119978382273462E-4</v>
       </c>
     </row>
     <row r="110" spans="2:175" x14ac:dyDescent="0.25">
@@ -8635,11 +8680,11 @@
       </c>
       <c r="D111" s="34">
         <f>'OPEX DATA 2'!U222</f>
-        <v>15.395480769230769</v>
+        <v>8.797417582417582</v>
       </c>
       <c r="E111" s="20">
         <f t="shared" si="4"/>
-        <v>2.2808119658119657E-4</v>
+        <v>1.4421996036750135E-4</v>
       </c>
     </row>
     <row r="112" spans="2:175" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -8650,11 +8695,11 @@
       <c r="C112" s="2"/>
       <c r="D112" s="28">
         <f>'OPEX DATA 2'!U223</f>
-        <v>7.1442307692307694E-2</v>
+        <v>4.0824175824175822E-2</v>
       </c>
       <c r="E112" s="18">
         <f t="shared" si="4"/>
-        <v>1.0584045584045585E-6</v>
+        <v>6.6924878400288237E-7</v>
       </c>
       <c r="F112" s="18"/>
       <c r="G112" s="18"/>
@@ -8834,11 +8879,11 @@
       </c>
       <c r="D113" s="34">
         <f>'OPEX DATA 2'!U224</f>
-        <v>6.6606730769230769</v>
+        <v>3.8060989010989013</v>
       </c>
       <c r="E113" s="20">
         <f t="shared" si="4"/>
-        <v>9.8676638176638178E-5</v>
+        <v>6.2395063952441001E-5</v>
       </c>
     </row>
     <row r="114" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8862,11 +8907,11 @@
       </c>
       <c r="D115" s="34">
         <f>'OPEX DATA 2'!U226</f>
-        <v>-1.311923076923077</v>
+        <v>-0.74967032967032965</v>
       </c>
       <c r="E115" s="20">
         <f t="shared" si="4"/>
-        <v>-1.9435897435897435E-5</v>
+        <v>-1.2289677535579174E-5</v>
       </c>
     </row>
     <row r="116" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8876,11 +8921,11 @@
       </c>
       <c r="D116" s="34">
         <f>'OPEX DATA 2'!U227</f>
-        <v>207.53586538461539</v>
+        <v>118.59192307692308</v>
       </c>
       <c r="E116" s="20">
         <f t="shared" si="4"/>
-        <v>3.0746054131054134E-3</v>
+        <v>1.9441298865069357E-3</v>
       </c>
     </row>
     <row r="117" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8890,11 +8935,11 @@
       </c>
       <c r="D117" s="34">
         <f>'OPEX DATA 2'!U228</f>
-        <v>42.539711538461539</v>
+        <v>24.308406593406595</v>
       </c>
       <c r="E117" s="20">
         <f t="shared" si="4"/>
-        <v>6.3021794871794868E-4</v>
+        <v>3.9849846874437042E-4</v>
       </c>
     </row>
     <row r="118" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -8904,11 +8949,11 @@
       </c>
       <c r="D118" s="34">
         <f>'OPEX DATA 2'!U229</f>
-        <v>1.0673076923076923</v>
+        <v>0.60989010989010983</v>
       </c>
       <c r="E118" s="20">
         <f t="shared" si="4"/>
-        <v>1.5811965811965812E-5</v>
+        <v>9.9981985227886857E-6</v>
       </c>
     </row>
     <row r="119" spans="2:175" x14ac:dyDescent="0.25">
@@ -8919,11 +8964,11 @@
       <c r="C119" s="22"/>
       <c r="D119" s="45">
         <f>'OPEX DATA 2'!U230</f>
-        <v>143.38269230769231</v>
+        <v>81.932967032967028</v>
       </c>
       <c r="E119" s="46">
         <f t="shared" si="4"/>
-        <v>2.1241880341880343E-3</v>
+        <v>1.3431633939830661E-3</v>
       </c>
     </row>
     <row r="120" spans="2:175" x14ac:dyDescent="0.25">
@@ -8948,11 +8993,11 @@
       <c r="C121" s="2"/>
       <c r="D121" s="28">
         <f>'OPEX DATA 2'!U232</f>
-        <v>4.8076923076923075</v>
+        <v>2.7472527472527473</v>
       </c>
       <c r="E121" s="18">
         <f t="shared" si="4"/>
-        <v>7.122507122507122E-5</v>
+        <v>4.5036930282831922E-5</v>
       </c>
       <c r="F121" s="18"/>
       <c r="G121" s="18"/>
@@ -9133,11 +9178,11 @@
       <c r="C122" s="22"/>
       <c r="D122" s="45">
         <f>'OPEX DATA 2'!U233</f>
-        <v>0.87903846153846155</v>
+        <v>0.50230769230769234</v>
       </c>
       <c r="E122" s="46">
         <f t="shared" si="4"/>
-        <v>1.3022792022792023E-5</v>
+        <v>8.2345523329129891E-6</v>
       </c>
     </row>
     <row r="123" spans="2:175" x14ac:dyDescent="0.25">
@@ -9147,11 +9192,11 @@
       </c>
       <c r="D123" s="34">
         <f>'OPEX DATA 2'!U234</f>
-        <v>7.6108653846153844</v>
+        <v>4.3490659340659343</v>
       </c>
       <c r="E123" s="20">
         <f t="shared" si="4"/>
-        <v>1.1275356125356125E-4</v>
+        <v>7.1296162853539901E-5</v>
       </c>
     </row>
     <row r="124" spans="2:175" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -9162,11 +9207,11 @@
       <c r="C124" s="2"/>
       <c r="D124" s="28">
         <f>'OPEX DATA 2'!U235</f>
-        <v>62.891442307692309</v>
+        <v>35.93796703296703</v>
       </c>
       <c r="E124" s="18">
         <f t="shared" si="4"/>
-        <v>9.317250712250712E-4</v>
+        <v>5.8914700054044317E-4</v>
       </c>
       <c r="F124" s="18"/>
       <c r="G124" s="18"/>
@@ -9346,11 +9391,11 @@
       </c>
       <c r="D125" s="34">
         <f>'OPEX DATA 2'!U236</f>
-        <v>1969.0310576923077</v>
+        <v>1125.1606043956044</v>
       </c>
       <c r="E125" s="20">
         <f t="shared" si="4"/>
-        <v>2.9170830484330484E-2</v>
+        <v>1.8445255809764007E-2</v>
       </c>
     </row>
     <row r="126" spans="2:175" x14ac:dyDescent="0.25">
@@ -9361,11 +9406,11 @@
       <c r="C126" s="22"/>
       <c r="D126" s="45">
         <f>'OPEX DATA 2'!U237</f>
-        <v>142.33134615384617</v>
+        <v>81.332197802197811</v>
       </c>
       <c r="E126" s="46">
         <f t="shared" si="4"/>
-        <v>2.1086125356125358E-3</v>
+        <v>1.3333147180688166E-3</v>
       </c>
     </row>
     <row r="127" spans="2:175" x14ac:dyDescent="0.25">
@@ -9375,11 +9420,11 @@
       </c>
       <c r="D127" s="34">
         <f>'OPEX DATA 2'!U238</f>
-        <v>20.738365384615385</v>
+        <v>11.850494505494506</v>
       </c>
       <c r="E127" s="20">
         <f t="shared" si="4"/>
-        <v>3.0723504273504271E-4</v>
+        <v>1.9427040172941815E-4</v>
       </c>
     </row>
     <row r="128" spans="2:175" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -9589,11 +9634,11 @@
       <c r="C130" s="48"/>
       <c r="D130" s="49">
         <f>SUM(D104:D129)</f>
-        <v>8301.9683653846132</v>
+        <v>4814.1549450549455</v>
       </c>
       <c r="E130" s="50">
         <f t="shared" si="4"/>
-        <v>0.1229921239316239</v>
+        <v>7.8920572869753208E-2</v>
       </c>
       <c r="F130" s="50"/>
       <c r="G130" s="50"/>
@@ -9616,11 +9661,11 @@
       </c>
       <c r="D133" s="34">
         <f>'OPEX DATA 2'!U244</f>
-        <v>36.678749999999994</v>
+        <v>20.959285714285709</v>
       </c>
       <c r="E133" s="20">
         <f t="shared" ref="E133:E141" si="5">D133/D$36</f>
-        <v>5.4338888888888883E-4</v>
+        <v>3.4359484777517554E-4</v>
       </c>
     </row>
     <row r="134" spans="2:7" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -9630,11 +9675,11 @@
       </c>
       <c r="D134" s="34">
         <f>'OPEX DATA 2'!U245</f>
-        <v>26.293942307692305</v>
+        <v>15.025109890109889</v>
       </c>
       <c r="E134" s="20">
         <f t="shared" si="5"/>
-        <v>3.8953988603988599E-4</v>
+        <v>2.4631327688704737E-4</v>
       </c>
     </row>
     <row r="135" spans="2:7" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -9658,11 +9703,11 @@
       </c>
       <c r="D136" s="34">
         <f>'OPEX DATA 2'!U247</f>
-        <v>253.40692307692308</v>
+        <v>144.80395604395605</v>
       </c>
       <c r="E136" s="20">
         <f t="shared" si="5"/>
-        <v>3.7541766381766384E-3</v>
+        <v>2.3738353449828859E-3</v>
       </c>
     </row>
     <row r="137" spans="2:7" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -9672,11 +9717,11 @@
       </c>
       <c r="D137" s="34">
         <f>'OPEX DATA 2'!U248</f>
-        <v>43.505769230769232</v>
+        <v>24.860439560439563</v>
       </c>
       <c r="E137" s="20">
         <f t="shared" si="5"/>
-        <v>6.445299145299146E-4</v>
+        <v>4.0754818951540265E-4</v>
       </c>
     </row>
     <row r="138" spans="2:7" x14ac:dyDescent="0.25">
@@ -9687,11 +9732,11 @@
       <c r="C138" s="22"/>
       <c r="D138" s="45">
         <f>'OPEX DATA 2'!U249</f>
-        <v>272.07451923076923</v>
+        <v>155.47115384615384</v>
       </c>
       <c r="E138" s="46">
         <f t="shared" si="5"/>
-        <v>4.0307336182336178E-3</v>
+        <v>2.5487074401008827E-3</v>
       </c>
     </row>
     <row r="139" spans="2:7" x14ac:dyDescent="0.25">
@@ -9731,11 +9776,11 @@
       <c r="C141" s="48"/>
       <c r="D141" s="49">
         <f>SUM(D133:D140)</f>
-        <v>631.95990384615379</v>
+        <v>361.11994505494505</v>
       </c>
       <c r="E141" s="50">
         <f t="shared" si="5"/>
-        <v>9.3623689458689451E-3</v>
+        <v>5.9199990992613938E-3</v>
       </c>
       <c r="F141" s="50"/>
       <c r="G141" s="50"/>
@@ -9778,11 +9823,11 @@
       <c r="C145" s="56"/>
       <c r="D145" s="57">
         <f>'OPEX DATA 2'!U256</f>
-        <v>4389.3273076923078</v>
+        <v>2508.1870329670332</v>
       </c>
       <c r="E145" s="58">
         <f t="shared" si="6"/>
-        <v>6.5027071225071231E-2</v>
+        <v>4.1117820212574319E-2</v>
       </c>
     </row>
     <row r="146" spans="2:7" x14ac:dyDescent="0.25">
@@ -9808,11 +9853,11 @@
       <c r="C147" s="56"/>
       <c r="D147" s="57">
         <f>'OPEX DATA 2'!U258</f>
-        <v>220.61403846153846</v>
+        <v>126.06516483516484</v>
       </c>
       <c r="E147" s="58">
         <f t="shared" si="6"/>
-        <v>3.2683561253561253E-3</v>
+        <v>2.0666420464781122E-3</v>
       </c>
     </row>
     <row r="148" spans="2:7" x14ac:dyDescent="0.25">
@@ -9853,11 +9898,11 @@
       <c r="C150" s="56"/>
       <c r="D150" s="57">
         <f>'OPEX DATA 2'!U261</f>
-        <v>1455.6618269230771</v>
+        <v>831.8067582417583</v>
       </c>
       <c r="E150" s="58">
         <f t="shared" si="6"/>
-        <v>2.1565360398860402E-2</v>
+        <v>1.3636176364618989E-2</v>
       </c>
     </row>
     <row r="151" spans="2:7" x14ac:dyDescent="0.25">
@@ -9868,11 +9913,11 @@
       <c r="C151" s="56"/>
       <c r="D151" s="57">
         <f>'OPEX DATA 2'!U262</f>
-        <v>540.70307692307688</v>
+        <v>308.97318681318677</v>
       </c>
       <c r="E151" s="58">
         <f t="shared" si="6"/>
-        <v>8.0104159544159542E-3</v>
+        <v>5.0651342100522419E-3</v>
       </c>
     </row>
     <row r="152" spans="2:7" x14ac:dyDescent="0.25">
@@ -9883,7 +9928,7 @@
       <c r="C152" s="48"/>
       <c r="D152" s="49">
         <f>E152*D10</f>
-        <v>4050</v>
+        <v>3660</v>
       </c>
       <c r="E152" s="50">
         <v>0.06</v>
@@ -9944,11 +9989,11 @@
       <c r="C157" s="56"/>
       <c r="D157" s="57">
         <f>'OPEX DATA 2'!U268</f>
-        <v>-0.31807692307692303</v>
+        <v>-0.18175824175824173</v>
       </c>
       <c r="E157" s="58">
         <f t="shared" si="7"/>
-        <v>-4.7122507122507113E-6</v>
+        <v>-2.9796433075121596E-6</v>
       </c>
     </row>
     <row r="158" spans="2:7" x14ac:dyDescent="0.25">
@@ -10094,7 +10139,7 @@
       <c r="C167" s="56"/>
       <c r="D167" s="57">
         <f>E167*D10</f>
-        <v>-2227.5</v>
+        <v>-2013</v>
       </c>
       <c r="E167" s="58">
         <v>-3.3000000000000002E-2</v>
@@ -10168,11 +10213,11 @@
       <c r="C172" s="48"/>
       <c r="D172" s="49">
         <f>SUM(D155:D171)</f>
-        <v>-2227.8180769230771</v>
+        <v>-2013.1817582417582</v>
       </c>
       <c r="E172" s="50">
         <f t="shared" si="7"/>
-        <v>-3.3004712250712255E-2</v>
+        <v>-3.3002979643307513E-2</v>
       </c>
       <c r="F172" s="50"/>
       <c r="G172" s="50"/>
@@ -10215,11 +10260,11 @@
       <c r="C176" s="56"/>
       <c r="D176" s="57">
         <f>'OPEX DATA 2'!U289</f>
-        <v>660.28</v>
+        <v>377.30285714285714</v>
       </c>
       <c r="E176" s="58">
         <f t="shared" si="8"/>
-        <v>9.7819259259259248E-3</v>
+        <v>6.1852927400468383E-3</v>
       </c>
     </row>
     <row r="177" spans="2:5" x14ac:dyDescent="0.25">
@@ -10230,11 +10275,11 @@
       <c r="C177" s="56"/>
       <c r="D177" s="57">
         <f>'OPEX DATA 2'!U290</f>
-        <v>5682.0760576923076</v>
+        <v>3246.9006043956042</v>
       </c>
       <c r="E177" s="58">
         <f t="shared" si="8"/>
-        <v>8.4178904558404558E-2</v>
+        <v>5.3227878760583679E-2</v>
       </c>
     </row>
     <row r="178" spans="2:5" x14ac:dyDescent="0.25">
@@ -10245,11 +10290,11 @@
       <c r="C178" s="56"/>
       <c r="D178" s="57">
         <f>'OPEX DATA 2'!U291</f>
-        <v>0.71153846153846156</v>
+        <v>0.40659340659340659</v>
       </c>
       <c r="E178" s="58">
         <f t="shared" si="8"/>
-        <v>1.0541310541310541E-5</v>
+        <v>6.6654656818591246E-6</v>
       </c>
     </row>
     <row r="179" spans="2:5" x14ac:dyDescent="0.25">
@@ -10260,11 +10305,11 @@
       <c r="C179" s="56"/>
       <c r="D179" s="57">
         <f>'OPEX DATA 2'!U292</f>
-        <v>151.36538461538461</v>
+        <v>86.494505494505489</v>
       </c>
       <c r="E179" s="58">
         <f t="shared" si="8"/>
-        <v>2.2424501424501424E-3</v>
+        <v>1.4179427130246803E-3</v>
       </c>
     </row>
     <row r="180" spans="2:5" x14ac:dyDescent="0.25">
@@ -10275,11 +10320,11 @@
       <c r="C180" s="56"/>
       <c r="D180" s="57">
         <f>'OPEX DATA 2'!U293</f>
-        <v>14.639711538461539</v>
+        <v>8.3655494505494499</v>
       </c>
       <c r="E180" s="58">
         <f t="shared" si="8"/>
-        <v>2.168846153846154E-4</v>
+        <v>1.3714015492704017E-4</v>
       </c>
     </row>
     <row r="181" spans="2:5" x14ac:dyDescent="0.25">
@@ -10290,11 +10335,11 @@
       <c r="C181" s="56"/>
       <c r="D181" s="57">
         <f>'OPEX DATA 2'!U294</f>
-        <v>381.67730769230764</v>
+        <v>218.10131868131865</v>
       </c>
       <c r="E181" s="58">
         <f t="shared" si="8"/>
-        <v>5.6544786324786321E-3</v>
+        <v>3.5754314537921089E-3</v>
       </c>
     </row>
     <row r="182" spans="2:5" x14ac:dyDescent="0.25">
@@ -10335,11 +10380,11 @@
       <c r="C184" s="56"/>
       <c r="D184" s="57">
         <f>'OPEX DATA 2'!U297</f>
-        <v>4.6392307692307693</v>
+        <v>2.6509890109890111</v>
       </c>
       <c r="E184" s="58">
         <f t="shared" si="8"/>
-        <v>6.8729344729344732E-5</v>
+        <v>4.345883624572149E-5</v>
       </c>
     </row>
     <row r="185" spans="2:5" x14ac:dyDescent="0.25">
@@ -10590,11 +10635,11 @@
       <c r="C201" s="48"/>
       <c r="D201" s="49">
         <f>SUM(D175:D200)</f>
-        <v>6895.3892307692295</v>
+        <v>3940.2224175824176</v>
       </c>
       <c r="E201" s="50">
         <f t="shared" si="8"/>
-        <v>0.10215391452991451</v>
+        <v>6.4593810124301931E-2</v>
       </c>
       <c r="F201" s="50"/>
       <c r="G201" s="50"/>
@@ -10612,11 +10657,11 @@
       <c r="C203" s="48"/>
       <c r="D203" s="49">
         <f>D43-D50-D101-D130-D141-D152-D172-D201</f>
-        <v>-4739.9198076922985</v>
+        <v>8695.511318681316</v>
       </c>
       <c r="E203" s="50">
         <f>D203/D36</f>
-        <v>-7.0221034188034048E-2</v>
+        <v>0.14254936588002157</v>
       </c>
       <c r="F203" s="50"/>
       <c r="G203" s="50"/>
@@ -10642,7 +10687,7 @@
       <c r="C207" s="63"/>
       <c r="D207" s="64">
         <f>E203</f>
-        <v>-7.0221034188034048E-2</v>
+        <v>0.14254936588002157</v>
       </c>
     </row>
     <row r="208" spans="2:175" s="20" customFormat="1" x14ac:dyDescent="0.25">
@@ -18577,8 +18622,8 @@
         <v>3118509.06</v>
       </c>
       <c r="U8" s="80">
-        <f>(T8/$V$1)/4</f>
-        <v>29985.664038461538</v>
+        <f>(T8/$V$1)/7</f>
+        <v>17134.665164835165</v>
       </c>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.25">
@@ -18637,7 +18682,7 @@
         <v>0</v>
       </c>
       <c r="U9" s="80">
-        <f t="shared" ref="U9:U72" si="1">(T9/$V$1)/4</f>
+        <f t="shared" ref="U9:U72" si="1">(T9/$V$1)/7</f>
         <v>0</v>
       </c>
       <c r="W9">
@@ -18708,7 +18753,7 @@
       </c>
       <c r="U10" s="80">
         <f t="shared" si="1"/>
-        <v>29985.664038461538</v>
+        <v>17134.665164835165</v>
       </c>
       <c r="W10">
         <f>W9*2</f>
@@ -18772,7 +18817,7 @@
       </c>
       <c r="U11" s="80">
         <f t="shared" si="1"/>
-        <v>3543.2023076923078</v>
+        <v>2024.687032967033</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -18922,7 +18967,7 @@
       </c>
       <c r="U14" s="80">
         <f t="shared" si="1"/>
-        <v>52196.227980769232</v>
+        <v>29826.415989010991</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
@@ -18982,7 +19027,7 @@
       </c>
       <c r="U15" s="80">
         <f t="shared" si="1"/>
-        <v>521.04807692307691</v>
+        <v>297.74175824175825</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
@@ -19042,7 +19087,7 @@
       </c>
       <c r="U16" s="80">
         <f t="shared" si="1"/>
-        <v>11967.01923076923</v>
+        <v>6838.2967032967035</v>
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
@@ -19102,7 +19147,7 @@
       </c>
       <c r="U17" s="80">
         <f t="shared" si="1"/>
-        <v>2453.3653846153848</v>
+        <v>1401.9230769230769</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
@@ -19162,7 +19207,7 @@
       </c>
       <c r="U18" s="80">
         <f t="shared" si="1"/>
-        <v>5415.0961538461543</v>
+        <v>3094.3406593406594</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
@@ -19228,7 +19273,7 @@
       </c>
       <c r="U19" s="80">
         <f t="shared" si="1"/>
-        <v>72552.756826923083</v>
+        <v>41458.718186813188</v>
       </c>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
@@ -19378,7 +19423,7 @@
       </c>
       <c r="U22" s="80">
         <f t="shared" si="1"/>
-        <v>2053.5549999999998</v>
+        <v>1173.4599999999998</v>
       </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
@@ -19438,7 +19483,7 @@
       </c>
       <c r="U23" s="80">
         <f t="shared" si="1"/>
-        <v>-2.0769230769230771</v>
+        <v>-1.1868131868131868</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
@@ -19618,7 +19663,7 @@
       </c>
       <c r="U26" s="80">
         <f t="shared" si="1"/>
-        <v>5508.4197115384613</v>
+        <v>3147.6684065934064</v>
       </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
@@ -19864,7 +19909,7 @@
       </c>
       <c r="U30" s="80">
         <f t="shared" si="1"/>
-        <v>7559.8977884615388</v>
+        <v>4319.9415934065937</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
@@ -20410,7 +20455,7 @@
       </c>
       <c r="U40" s="80">
         <f t="shared" si="1"/>
-        <v>-3.0913461538461537</v>
+        <v>-1.7664835164835164</v>
       </c>
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
@@ -20470,7 +20515,7 @@
       </c>
       <c r="U41" s="80">
         <f t="shared" si="1"/>
-        <v>-116.5653846153846</v>
+        <v>-66.608791208791203</v>
       </c>
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
@@ -20530,7 +20575,7 @@
       </c>
       <c r="U42" s="80">
         <f t="shared" si="1"/>
-        <v>-318.85192307692307</v>
+        <v>-182.2010989010989</v>
       </c>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
@@ -20590,7 +20635,7 @@
       </c>
       <c r="U43" s="80">
         <f t="shared" si="1"/>
-        <v>-1243.3653846153845</v>
+        <v>-710.49450549450546</v>
       </c>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
@@ -20650,7 +20695,7 @@
       </c>
       <c r="U44" s="80">
         <f t="shared" si="1"/>
-        <v>-25.971153846153847</v>
+        <v>-14.840659340659341</v>
       </c>
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
@@ -20773,7 +20818,7 @@
       </c>
       <c r="U46" s="80">
         <f t="shared" si="1"/>
-        <v>-1244.5483653846154</v>
+        <v>-711.1704945054945</v>
       </c>
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
@@ -20833,7 +20878,7 @@
       </c>
       <c r="U47" s="80">
         <f t="shared" si="1"/>
-        <v>-273.13942307692309</v>
+        <v>-156.07967032967034</v>
       </c>
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
@@ -20893,7 +20938,7 @@
       </c>
       <c r="U48" s="80">
         <f t="shared" si="1"/>
-        <v>-222.48076923076923</v>
+        <v>-127.13186813186813</v>
       </c>
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
@@ -20953,7 +20998,7 @@
       </c>
       <c r="U49" s="80">
         <f t="shared" si="1"/>
-        <v>-25.576923076923077</v>
+        <v>-14.615384615384615</v>
       </c>
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
@@ -21016,7 +21061,7 @@
       </c>
       <c r="U50" s="80">
         <f t="shared" si="1"/>
-        <v>-175.23461538461541</v>
+        <v>-100.13406593406594</v>
       </c>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
@@ -21082,7 +21127,7 @@
       </c>
       <c r="U51" s="80">
         <f t="shared" si="1"/>
-        <v>-3648.8252884615381</v>
+        <v>-2085.0430219780219</v>
       </c>
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
@@ -21148,7 +21193,7 @@
       </c>
       <c r="U52" s="80">
         <f t="shared" si="1"/>
-        <v>109992.69567307692</v>
+        <v>62852.968956043951</v>
       </c>
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
@@ -21328,7 +21373,7 @@
       </c>
       <c r="U56" s="80">
         <f t="shared" si="1"/>
-        <v>654.12788461538469</v>
+        <v>373.78736263736266</v>
       </c>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
@@ -21388,7 +21433,7 @@
       </c>
       <c r="U57" s="80">
         <f t="shared" si="1"/>
-        <v>163.84923076923076</v>
+        <v>93.62813186813186</v>
       </c>
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
@@ -21448,7 +21493,7 @@
       </c>
       <c r="U58" s="80">
         <f t="shared" si="1"/>
-        <v>2061.4732692307693</v>
+        <v>1177.9847252747254</v>
       </c>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
@@ -21508,7 +21553,7 @@
       </c>
       <c r="U59" s="80">
         <f t="shared" si="1"/>
-        <v>122.70451923076924</v>
+        <v>70.116868131868131</v>
       </c>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
@@ -21568,7 +21613,7 @@
       </c>
       <c r="U60" s="80">
         <f t="shared" si="1"/>
-        <v>3153.9875000000002</v>
+        <v>1802.2785714285715</v>
       </c>
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
@@ -21628,7 +21673,7 @@
       </c>
       <c r="U61" s="80">
         <f t="shared" si="1"/>
-        <v>541.59596153846155</v>
+        <v>309.48340659340658</v>
       </c>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
@@ -21688,7 +21733,7 @@
       </c>
       <c r="U62" s="80">
         <f t="shared" si="1"/>
-        <v>7.9195192307692315</v>
+        <v>4.525439560439561</v>
       </c>
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
@@ -21748,7 +21793,7 @@
       </c>
       <c r="U63" s="80">
         <f t="shared" si="1"/>
-        <v>262.3238461538462</v>
+        <v>149.89934065934068</v>
       </c>
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
@@ -21874,7 +21919,7 @@
       </c>
       <c r="U65" s="80">
         <f t="shared" si="1"/>
-        <v>6967.9817307692301</v>
+        <v>3981.7038461538459</v>
       </c>
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
@@ -21934,7 +21979,7 @@
       </c>
       <c r="U66" s="80">
         <f t="shared" si="1"/>
-        <v>813.79451923076908</v>
+        <v>465.02543956043945</v>
       </c>
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
@@ -22084,7 +22129,7 @@
       </c>
       <c r="U69" s="80">
         <f t="shared" si="1"/>
-        <v>80.601826923076928</v>
+        <v>46.058186813186815</v>
       </c>
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
@@ -22144,7 +22189,7 @@
       </c>
       <c r="U70" s="80">
         <f t="shared" si="1"/>
-        <v>344.65355769230769</v>
+        <v>196.94489010989011</v>
       </c>
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
@@ -22204,7 +22249,7 @@
       </c>
       <c r="U71" s="80">
         <f t="shared" si="1"/>
-        <v>4793.6948076923081</v>
+        <v>2739.2541758241759</v>
       </c>
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
@@ -22323,8 +22368,8 @@
         <v>526298.73</v>
       </c>
       <c r="U73" s="80">
-        <f t="shared" ref="U73:U136" si="3">(T73/$V$1)/4</f>
-        <v>5060.5647115384618</v>
+        <f t="shared" ref="U73:U136" si="3">(T73/$V$1)/7</f>
+        <v>2891.7512637362638</v>
       </c>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
@@ -22444,7 +22489,7 @@
       </c>
       <c r="U75" s="80">
         <f t="shared" si="3"/>
-        <v>379.51442307692309</v>
+        <v>216.86538461538461</v>
       </c>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
@@ -22510,7 +22555,7 @@
       </c>
       <c r="U76" s="80">
         <f t="shared" si="3"/>
-        <v>10659.029326923077</v>
+        <v>6090.8739010989011</v>
       </c>
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
@@ -22966,7 +23011,7 @@
       </c>
       <c r="U85" s="80">
         <f t="shared" si="3"/>
-        <v>1406.7064423076922</v>
+        <v>803.83225274725271</v>
       </c>
     </row>
     <row r="86" spans="1:21" x14ac:dyDescent="0.25">
@@ -23026,7 +23071,7 @@
       </c>
       <c r="U86" s="80">
         <f t="shared" si="3"/>
-        <v>365.30163461538456</v>
+        <v>208.74379120879118</v>
       </c>
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
@@ -23086,7 +23131,7 @@
       </c>
       <c r="U87" s="80">
         <f t="shared" si="3"/>
-        <v>186.47211538461536</v>
+        <v>106.55549450549449</v>
       </c>
     </row>
     <row r="88" spans="1:21" x14ac:dyDescent="0.25">
@@ -23146,7 +23191,7 @@
       </c>
       <c r="U88" s="80">
         <f t="shared" si="3"/>
-        <v>1367.0021153846153</v>
+        <v>781.14406593406591</v>
       </c>
     </row>
     <row r="89" spans="1:21" x14ac:dyDescent="0.25">
@@ -23206,7 +23251,7 @@
       </c>
       <c r="U89" s="80">
         <f t="shared" si="3"/>
-        <v>10.618461538461538</v>
+        <v>6.0676923076923073</v>
       </c>
     </row>
     <row r="90" spans="1:21" x14ac:dyDescent="0.25">
@@ -23386,7 +23431,7 @@
       </c>
       <c r="U92" s="80">
         <f t="shared" si="3"/>
-        <v>644.77009615384611</v>
+        <v>368.4400549450549</v>
       </c>
     </row>
     <row r="93" spans="1:21" x14ac:dyDescent="0.25">
@@ -23626,7 +23671,7 @@
       </c>
       <c r="U96" s="80">
         <f t="shared" si="3"/>
-        <v>67.307692307692307</v>
+        <v>38.46153846153846</v>
       </c>
     </row>
     <row r="97" spans="1:21" x14ac:dyDescent="0.25">
@@ -23686,7 +23731,7 @@
       </c>
       <c r="U97" s="80">
         <f t="shared" si="3"/>
-        <v>494.37769230769231</v>
+        <v>282.50153846153847</v>
       </c>
     </row>
     <row r="98" spans="1:21" x14ac:dyDescent="0.25">
@@ -23746,7 +23791,7 @@
       </c>
       <c r="U98" s="80">
         <f t="shared" si="3"/>
-        <v>408.61769230769227</v>
+        <v>233.49582417582414</v>
       </c>
     </row>
     <row r="99" spans="1:21" x14ac:dyDescent="0.25">
@@ -24466,7 +24511,7 @@
       </c>
       <c r="U110" s="80">
         <f t="shared" si="3"/>
-        <v>545.03038461538449</v>
+        <v>311.44593406593401</v>
       </c>
     </row>
     <row r="111" spans="1:21" x14ac:dyDescent="0.25">
@@ -24586,7 +24631,7 @@
       </c>
       <c r="U112" s="80">
         <f t="shared" si="3"/>
-        <v>332.06307692307689</v>
+        <v>189.75032967032965</v>
       </c>
     </row>
     <row r="113" spans="1:23" x14ac:dyDescent="0.25">
@@ -24706,7 +24751,7 @@
       </c>
       <c r="U114" s="80">
         <f t="shared" si="3"/>
-        <v>14.87048076923077</v>
+        <v>8.497417582417583</v>
       </c>
     </row>
     <row r="115" spans="1:23" x14ac:dyDescent="0.25">
@@ -24946,7 +24991,7 @@
       </c>
       <c r="U118" s="80">
         <f t="shared" si="3"/>
-        <v>26.903365384615384</v>
+        <v>15.373351648351647</v>
       </c>
     </row>
     <row r="119" spans="1:23" x14ac:dyDescent="0.25">
@@ -25012,7 +25057,7 @@
       </c>
       <c r="U119" s="80">
         <f t="shared" si="3"/>
-        <v>5870.0412499999993</v>
+        <v>3354.3092857142851</v>
       </c>
     </row>
     <row r="120" spans="1:23" x14ac:dyDescent="0.25">
@@ -25078,11 +25123,11 @@
       </c>
       <c r="U120" s="80">
         <f t="shared" si="3"/>
-        <v>5870.0412499999993</v>
+        <v>3354.3092857142851</v>
       </c>
       <c r="W120" s="80">
         <f>U120+U143+U151</f>
-        <v>19039.900576923079</v>
+        <v>10879.943186813185</v>
       </c>
     </row>
     <row r="121" spans="1:23" x14ac:dyDescent="0.25">
@@ -25232,7 +25277,7 @@
       </c>
       <c r="U123" s="80">
         <f t="shared" si="3"/>
-        <v>711.03461538461534</v>
+        <v>406.30549450549449</v>
       </c>
     </row>
     <row r="124" spans="1:23" x14ac:dyDescent="0.25">
@@ -25292,7 +25337,7 @@
       </c>
       <c r="U124" s="80">
         <f t="shared" si="3"/>
-        <v>1366.1238461538462</v>
+        <v>780.64219780219787</v>
       </c>
     </row>
     <row r="125" spans="1:23" ht="31.5" x14ac:dyDescent="0.25">
@@ -25652,7 +25697,7 @@
       </c>
       <c r="U130" s="80">
         <f t="shared" si="3"/>
-        <v>-77.288461538461533</v>
+        <v>-44.164835164835161</v>
       </c>
     </row>
     <row r="131" spans="1:21" x14ac:dyDescent="0.25">
@@ -26071,7 +26116,7 @@
         <v>0</v>
       </c>
       <c r="U137" s="80">
-        <f t="shared" ref="U137:U200" si="5">(T137/$V$1)/4</f>
+        <f t="shared" ref="U137:U200" si="5">(T137/$V$1)/7</f>
         <v>0</v>
       </c>
     </row>
@@ -26192,7 +26237,7 @@
       </c>
       <c r="U139" s="80">
         <f t="shared" si="5"/>
-        <v>4239.5715384615387</v>
+        <v>2422.6123076923077</v>
       </c>
     </row>
     <row r="140" spans="1:21" x14ac:dyDescent="0.25">
@@ -26312,7 +26357,7 @@
       </c>
       <c r="U141" s="80">
         <f t="shared" si="5"/>
-        <v>2368.407596153846</v>
+        <v>1353.3757692307693</v>
       </c>
     </row>
     <row r="142" spans="1:21" x14ac:dyDescent="0.25">
@@ -26372,7 +26417,7 @@
       </c>
       <c r="U142" s="80">
         <f t="shared" si="5"/>
-        <v>995.33653846153845</v>
+        <v>568.76373626373629</v>
       </c>
     </row>
     <row r="143" spans="1:21" x14ac:dyDescent="0.25">
@@ -26438,7 +26483,7 @@
       </c>
       <c r="U143" s="80">
         <f t="shared" si="5"/>
-        <v>9603.1856730769232</v>
+        <v>5487.53467032967</v>
       </c>
     </row>
     <row r="144" spans="1:21" x14ac:dyDescent="0.25">
@@ -26588,7 +26633,7 @@
       </c>
       <c r="U146" s="80">
         <f t="shared" si="5"/>
-        <v>2045.8558653846153</v>
+        <v>1169.0604945054945</v>
       </c>
     </row>
     <row r="147" spans="1:21" x14ac:dyDescent="0.25">
@@ -26648,7 +26693,7 @@
       </c>
       <c r="U147" s="80">
         <f t="shared" si="5"/>
-        <v>366.91990384615383</v>
+        <v>209.66851648351647</v>
       </c>
     </row>
     <row r="148" spans="1:21" x14ac:dyDescent="0.25">
@@ -26708,7 +26753,7 @@
       </c>
       <c r="U148" s="80">
         <f t="shared" si="5"/>
-        <v>254.15740384615387</v>
+        <v>145.23280219780222</v>
       </c>
     </row>
     <row r="149" spans="1:21" x14ac:dyDescent="0.25">
@@ -26768,7 +26813,7 @@
       </c>
       <c r="U149" s="80">
         <f t="shared" si="5"/>
-        <v>293.55769230769232</v>
+        <v>167.74725274725276</v>
       </c>
     </row>
     <row r="150" spans="1:21" x14ac:dyDescent="0.25">
@@ -26828,7 +26873,7 @@
       </c>
       <c r="U150" s="80">
         <f t="shared" si="5"/>
-        <v>606.18278846153851</v>
+        <v>346.39016483516485</v>
       </c>
     </row>
     <row r="151" spans="1:21" x14ac:dyDescent="0.25">
@@ -26894,7 +26939,7 @@
       </c>
       <c r="U151" s="80">
         <f t="shared" si="5"/>
-        <v>3566.6736538461537</v>
+        <v>2038.0992307692306</v>
       </c>
     </row>
     <row r="152" spans="1:21" x14ac:dyDescent="0.25">
@@ -27014,7 +27059,7 @@
       </c>
       <c r="U153" s="80">
         <f t="shared" si="5"/>
-        <v>791.10557692307691</v>
+        <v>452.06032967032968</v>
       </c>
     </row>
     <row r="154" spans="1:21" x14ac:dyDescent="0.25">
@@ -27074,7 +27119,7 @@
       </c>
       <c r="U154" s="80">
         <f t="shared" si="5"/>
-        <v>17.198365384615386</v>
+        <v>9.827637362637363</v>
       </c>
     </row>
     <row r="155" spans="1:21" x14ac:dyDescent="0.25">
@@ -27134,7 +27179,7 @@
       </c>
       <c r="U155" s="80">
         <f t="shared" si="5"/>
-        <v>0.32403846153846172</v>
+        <v>0.18516483516483526</v>
       </c>
     </row>
     <row r="156" spans="1:21" x14ac:dyDescent="0.25">
@@ -27260,7 +27305,7 @@
       </c>
       <c r="U157" s="80">
         <f t="shared" si="5"/>
-        <v>38289.334134615383</v>
+        <v>21879.619505494506</v>
       </c>
     </row>
     <row r="158" spans="1:21" x14ac:dyDescent="0.25">
@@ -27440,7 +27485,7 @@
       </c>
       <c r="U161" s="80">
         <f t="shared" si="5"/>
-        <v>0.26999999999999996</v>
+        <v>0.15428571428571428</v>
       </c>
     </row>
     <row r="162" spans="1:21" x14ac:dyDescent="0.25">
@@ -27500,7 +27545,7 @@
       </c>
       <c r="U162" s="80">
         <f t="shared" si="5"/>
-        <v>152.5126923076923</v>
+        <v>87.150109890109889</v>
       </c>
     </row>
     <row r="163" spans="1:21" x14ac:dyDescent="0.25">
@@ -27560,7 +27605,7 @@
       </c>
       <c r="U163" s="80">
         <f t="shared" si="5"/>
-        <v>245.6385576923077</v>
+        <v>140.36489010989013</v>
       </c>
     </row>
     <row r="164" spans="1:21" x14ac:dyDescent="0.25">
@@ -27620,7 +27665,7 @@
       </c>
       <c r="U164" s="80">
         <f t="shared" si="5"/>
-        <v>38.466538461538462</v>
+        <v>21.98087912087912</v>
       </c>
     </row>
     <row r="165" spans="1:21" x14ac:dyDescent="0.25">
@@ -27680,7 +27725,7 @@
       </c>
       <c r="U165" s="80">
         <f t="shared" si="5"/>
-        <v>41.174038461538458</v>
+        <v>23.528021978021975</v>
       </c>
     </row>
     <row r="166" spans="1:21" x14ac:dyDescent="0.25">
@@ -27740,7 +27785,7 @@
       </c>
       <c r="U166" s="80">
         <f t="shared" si="5"/>
-        <v>230.69173076923079</v>
+        <v>131.82384615384618</v>
       </c>
     </row>
     <row r="167" spans="1:21" x14ac:dyDescent="0.25">
@@ -27800,7 +27845,7 @@
       </c>
       <c r="U167" s="80">
         <f t="shared" si="5"/>
-        <v>173.01663461538465</v>
+        <v>98.866648351648365</v>
       </c>
     </row>
     <row r="168" spans="1:21" x14ac:dyDescent="0.25">
@@ -27860,7 +27905,7 @@
       </c>
       <c r="U168" s="80">
         <f t="shared" si="5"/>
-        <v>708.65326923076941</v>
+        <v>404.94472527472539</v>
       </c>
     </row>
     <row r="169" spans="1:21" x14ac:dyDescent="0.25">
@@ -27920,7 +27965,7 @@
       </c>
       <c r="U169" s="80">
         <f t="shared" si="5"/>
-        <v>35.989230769230772</v>
+        <v>20.565274725274726</v>
       </c>
     </row>
     <row r="170" spans="1:21" x14ac:dyDescent="0.25">
@@ -27980,7 +28025,7 @@
       </c>
       <c r="U170" s="80">
         <f t="shared" si="5"/>
-        <v>252.62173076923077</v>
+        <v>144.35527472527471</v>
       </c>
     </row>
     <row r="171" spans="1:21" x14ac:dyDescent="0.25">
@@ -28040,7 +28085,7 @@
       </c>
       <c r="U171" s="80">
         <f t="shared" si="5"/>
-        <v>279.36682692307693</v>
+        <v>159.63818681318682</v>
       </c>
     </row>
     <row r="172" spans="1:21" x14ac:dyDescent="0.25">
@@ -28280,7 +28325,7 @@
       </c>
       <c r="U175" s="80">
         <f t="shared" si="5"/>
-        <v>270.21471153846153</v>
+        <v>154.4084065934066</v>
       </c>
     </row>
     <row r="176" spans="1:21" x14ac:dyDescent="0.25">
@@ -28340,7 +28385,7 @@
       </c>
       <c r="U176" s="80">
         <f t="shared" si="5"/>
-        <v>258.85000000000002</v>
+        <v>147.91428571428574</v>
       </c>
     </row>
     <row r="177" spans="1:21" x14ac:dyDescent="0.25">
@@ -28400,7 +28445,7 @@
       </c>
       <c r="U177" s="80">
         <f t="shared" si="5"/>
-        <v>208.93653846153845</v>
+        <v>119.39230769230768</v>
       </c>
     </row>
     <row r="178" spans="1:21" x14ac:dyDescent="0.25">
@@ -28460,7 +28505,7 @@
       </c>
       <c r="U178" s="80">
         <f t="shared" si="5"/>
-        <v>297.10875000000004</v>
+        <v>169.7764285714286</v>
       </c>
     </row>
     <row r="179" spans="1:21" x14ac:dyDescent="0.25">
@@ -28520,7 +28565,7 @@
       </c>
       <c r="U179" s="80">
         <f t="shared" si="5"/>
-        <v>99.572884615384609</v>
+        <v>56.898791208791202</v>
       </c>
     </row>
     <row r="180" spans="1:21" x14ac:dyDescent="0.25">
@@ -28580,7 +28625,7 @@
       </c>
       <c r="U180" s="80">
         <f t="shared" si="5"/>
-        <v>523.67298076923078</v>
+        <v>299.24170329670329</v>
       </c>
     </row>
     <row r="181" spans="1:21" x14ac:dyDescent="0.25">
@@ -28700,7 +28745,7 @@
       </c>
       <c r="U182" s="80">
         <f t="shared" si="5"/>
-        <v>3.8412500000000001</v>
+        <v>2.1949999999999998</v>
       </c>
     </row>
     <row r="183" spans="1:21" x14ac:dyDescent="0.25">
@@ -28760,7 +28805,7 @@
       </c>
       <c r="U183" s="80">
         <f t="shared" si="5"/>
-        <v>146.51663461538462</v>
+        <v>83.723791208791212</v>
       </c>
     </row>
     <row r="184" spans="1:21" x14ac:dyDescent="0.25">
@@ -28820,7 +28865,7 @@
       </c>
       <c r="U184" s="80">
         <f t="shared" si="5"/>
-        <v>51.022403846153843</v>
+        <v>29.155659340659337</v>
       </c>
     </row>
     <row r="185" spans="1:21" x14ac:dyDescent="0.25">
@@ -29000,7 +29045,7 @@
       </c>
       <c r="U187" s="80">
         <f t="shared" si="5"/>
-        <v>20.997211538461539</v>
+        <v>11.998406593406594</v>
       </c>
     </row>
     <row r="188" spans="1:21" x14ac:dyDescent="0.25">
@@ -29060,7 +29105,7 @@
       </c>
       <c r="U188" s="80">
         <f t="shared" si="5"/>
-        <v>179.06451923076924</v>
+        <v>102.32258241758242</v>
       </c>
     </row>
     <row r="189" spans="1:21" x14ac:dyDescent="0.25">
@@ -29120,7 +29165,7 @@
       </c>
       <c r="U189" s="80">
         <f t="shared" si="5"/>
-        <v>298.44461538461536</v>
+        <v>170.5397802197802</v>
       </c>
     </row>
     <row r="190" spans="1:21" x14ac:dyDescent="0.25">
@@ -29180,7 +29225,7 @@
       </c>
       <c r="U190" s="80">
         <f t="shared" si="5"/>
-        <v>11.956250000000001</v>
+        <v>6.8321428571428573</v>
       </c>
     </row>
     <row r="191" spans="1:21" x14ac:dyDescent="0.25">
@@ -29300,7 +29345,7 @@
       </c>
       <c r="U192" s="80">
         <f t="shared" si="5"/>
-        <v>169.74317307692309</v>
+        <v>96.996098901098904</v>
       </c>
     </row>
     <row r="193" spans="1:21" x14ac:dyDescent="0.25">
@@ -29360,7 +29405,7 @@
       </c>
       <c r="U193" s="80">
         <f t="shared" si="5"/>
-        <v>1241.1204807692307</v>
+        <v>709.21170329670326</v>
       </c>
     </row>
     <row r="194" spans="1:21" x14ac:dyDescent="0.25">
@@ -29420,7 +29465,7 @@
       </c>
       <c r="U194" s="80">
         <f t="shared" si="5"/>
-        <v>597.66644230769225</v>
+        <v>341.52368131868127</v>
       </c>
     </row>
     <row r="195" spans="1:21" x14ac:dyDescent="0.25">
@@ -29480,7 +29525,7 @@
       </c>
       <c r="U195" s="80">
         <f t="shared" si="5"/>
-        <v>74.42096153846154</v>
+        <v>42.526263736263736</v>
       </c>
     </row>
     <row r="196" spans="1:21" x14ac:dyDescent="0.25">
@@ -29540,7 +29585,7 @@
       </c>
       <c r="U196" s="80">
         <f t="shared" si="5"/>
-        <v>8994.3097115384608</v>
+        <v>5139.605549450549</v>
       </c>
     </row>
     <row r="197" spans="1:21" x14ac:dyDescent="0.25">
@@ -29600,7 +29645,7 @@
       </c>
       <c r="U197" s="80">
         <f t="shared" si="5"/>
-        <v>28.800769230769227</v>
+        <v>16.457582417582415</v>
       </c>
     </row>
     <row r="198" spans="1:21" x14ac:dyDescent="0.25">
@@ -29839,8 +29884,8 @@
         <v>2810.66</v>
       </c>
       <c r="U201" s="80">
-        <f t="shared" ref="U201:U264" si="7">(T201/$V$1)/4</f>
-        <v>27.025576923076922</v>
+        <f t="shared" ref="U201:U264" si="7">(T201/$V$1)/7</f>
+        <v>15.443186813186813</v>
       </c>
     </row>
     <row r="202" spans="1:21" x14ac:dyDescent="0.25">
@@ -30326,7 +30371,7 @@
       </c>
       <c r="U209" s="80">
         <f t="shared" si="7"/>
-        <v>15661.687115384617</v>
+        <v>8949.5354945054951</v>
       </c>
     </row>
     <row r="210" spans="1:21" x14ac:dyDescent="0.25">
@@ -30452,7 +30497,7 @@
       </c>
       <c r="U211" s="80">
         <f t="shared" si="7"/>
-        <v>15661.687115384617</v>
+        <v>8949.5354945054951</v>
       </c>
     </row>
     <row r="212" spans="1:21" x14ac:dyDescent="0.25">
@@ -30632,7 +30677,7 @@
       </c>
       <c r="U215" s="80">
         <f t="shared" si="7"/>
-        <v>3399.9472115384615</v>
+        <v>1942.826978021978</v>
       </c>
     </row>
     <row r="216" spans="1:21" x14ac:dyDescent="0.25">
@@ -30692,7 +30737,7 @@
       </c>
       <c r="U216" s="80">
         <f t="shared" si="7"/>
-        <v>49.07692307692308</v>
+        <v>28.043956043956047</v>
       </c>
     </row>
     <row r="217" spans="1:21" x14ac:dyDescent="0.25">
@@ -30752,7 +30797,7 @@
       </c>
       <c r="U217" s="80">
         <f t="shared" si="7"/>
-        <v>746.53298076923079</v>
+        <v>426.59027472527475</v>
       </c>
     </row>
     <row r="218" spans="1:21" x14ac:dyDescent="0.25">
@@ -30812,7 +30857,7 @@
       </c>
       <c r="U218" s="80">
         <f t="shared" si="7"/>
-        <v>59.950384615384614</v>
+        <v>34.25736263736264</v>
       </c>
     </row>
     <row r="219" spans="1:21" x14ac:dyDescent="0.25">
@@ -30872,7 +30917,7 @@
       </c>
       <c r="U219" s="80">
         <f t="shared" si="7"/>
-        <v>1390.6767307692307</v>
+        <v>794.67241758241755</v>
       </c>
     </row>
     <row r="220" spans="1:21" x14ac:dyDescent="0.25">
@@ -30932,7 +30977,7 @@
       </c>
       <c r="U220" s="80">
         <f t="shared" si="7"/>
-        <v>32.153076923076924</v>
+        <v>18.373186813186813</v>
       </c>
     </row>
     <row r="221" spans="1:21" x14ac:dyDescent="0.25">
@@ -31052,7 +31097,7 @@
       </c>
       <c r="U222" s="80">
         <f t="shared" si="7"/>
-        <v>15.395480769230769</v>
+        <v>8.797417582417582</v>
       </c>
     </row>
     <row r="223" spans="1:21" x14ac:dyDescent="0.25">
@@ -31112,7 +31157,7 @@
       </c>
       <c r="U223" s="80">
         <f t="shared" si="7"/>
-        <v>7.1442307692307694E-2</v>
+        <v>4.0824175824175822E-2</v>
       </c>
     </row>
     <row r="224" spans="1:21" x14ac:dyDescent="0.25">
@@ -31172,7 +31217,7 @@
       </c>
       <c r="U224" s="80">
         <f t="shared" si="7"/>
-        <v>6.6606730769230769</v>
+        <v>3.8060989010989013</v>
       </c>
     </row>
     <row r="225" spans="1:21" x14ac:dyDescent="0.25">
@@ -31292,7 +31337,7 @@
       </c>
       <c r="U226" s="80">
         <f t="shared" si="7"/>
-        <v>-1.311923076923077</v>
+        <v>-0.74967032967032965</v>
       </c>
     </row>
     <row r="227" spans="1:21" x14ac:dyDescent="0.25">
@@ -31352,7 +31397,7 @@
       </c>
       <c r="U227" s="80">
         <f t="shared" si="7"/>
-        <v>207.53586538461539</v>
+        <v>118.59192307692308</v>
       </c>
     </row>
     <row r="228" spans="1:21" x14ac:dyDescent="0.25">
@@ -31412,7 +31457,7 @@
       </c>
       <c r="U228" s="80">
         <f t="shared" si="7"/>
-        <v>42.539711538461539</v>
+        <v>24.308406593406595</v>
       </c>
     </row>
     <row r="229" spans="1:21" x14ac:dyDescent="0.25">
@@ -31472,7 +31517,7 @@
       </c>
       <c r="U229" s="80">
         <f t="shared" si="7"/>
-        <v>1.0673076923076923</v>
+        <v>0.60989010989010983</v>
       </c>
     </row>
     <row r="230" spans="1:21" x14ac:dyDescent="0.25">
@@ -31532,7 +31577,7 @@
       </c>
       <c r="U230" s="80">
         <f t="shared" si="7"/>
-        <v>143.38269230769231</v>
+        <v>81.932967032967028</v>
       </c>
     </row>
     <row r="231" spans="1:21" x14ac:dyDescent="0.25">
@@ -31652,7 +31697,7 @@
       </c>
       <c r="U232" s="80">
         <f t="shared" si="7"/>
-        <v>4.8076923076923075</v>
+        <v>2.7472527472527473</v>
       </c>
     </row>
     <row r="233" spans="1:21" x14ac:dyDescent="0.25">
@@ -31712,7 +31757,7 @@
       </c>
       <c r="U233" s="80">
         <f t="shared" si="7"/>
-        <v>0.87903846153846155</v>
+        <v>0.50230769230769234</v>
       </c>
     </row>
     <row r="234" spans="1:21" x14ac:dyDescent="0.25">
@@ -31772,7 +31817,7 @@
       </c>
       <c r="U234" s="80">
         <f t="shared" si="7"/>
-        <v>7.6108653846153844</v>
+        <v>4.3490659340659343</v>
       </c>
     </row>
     <row r="235" spans="1:21" x14ac:dyDescent="0.25">
@@ -31832,7 +31877,7 @@
       </c>
       <c r="U235" s="80">
         <f t="shared" si="7"/>
-        <v>62.891442307692309</v>
+        <v>35.93796703296703</v>
       </c>
     </row>
     <row r="236" spans="1:21" x14ac:dyDescent="0.25">
@@ -31892,7 +31937,7 @@
       </c>
       <c r="U236" s="80">
         <f t="shared" si="7"/>
-        <v>1969.0310576923077</v>
+        <v>1125.1606043956044</v>
       </c>
     </row>
     <row r="237" spans="1:21" x14ac:dyDescent="0.25">
@@ -31952,7 +31997,7 @@
       </c>
       <c r="U237" s="80">
         <f t="shared" si="7"/>
-        <v>142.33134615384617</v>
+        <v>81.332197802197811</v>
       </c>
     </row>
     <row r="238" spans="1:21" x14ac:dyDescent="0.25">
@@ -32012,7 +32057,7 @@
       </c>
       <c r="U238" s="80">
         <f t="shared" si="7"/>
-        <v>20.738365384615385</v>
+        <v>11.850494505494506</v>
       </c>
     </row>
     <row r="239" spans="1:21" x14ac:dyDescent="0.25">
@@ -32198,7 +32243,7 @@
       </c>
       <c r="U241" s="80">
         <f t="shared" si="7"/>
-        <v>8301.9683653846168</v>
+        <v>4743.9819230769235</v>
       </c>
     </row>
     <row r="242" spans="1:21" x14ac:dyDescent="0.25">
@@ -32348,7 +32393,7 @@
       </c>
       <c r="U244" s="80">
         <f t="shared" si="7"/>
-        <v>36.678749999999994</v>
+        <v>20.959285714285709</v>
       </c>
     </row>
     <row r="245" spans="1:21" x14ac:dyDescent="0.25">
@@ -32408,7 +32453,7 @@
       </c>
       <c r="U245" s="80">
         <f t="shared" si="7"/>
-        <v>26.293942307692305</v>
+        <v>15.025109890109889</v>
       </c>
     </row>
     <row r="246" spans="1:21" x14ac:dyDescent="0.25">
@@ -32528,7 +32573,7 @@
       </c>
       <c r="U247" s="80">
         <f t="shared" si="7"/>
-        <v>253.40692307692308</v>
+        <v>144.80395604395605</v>
       </c>
     </row>
     <row r="248" spans="1:21" x14ac:dyDescent="0.25">
@@ -32588,7 +32633,7 @@
       </c>
       <c r="U248" s="80">
         <f t="shared" si="7"/>
-        <v>43.505769230769232</v>
+        <v>24.860439560439563</v>
       </c>
     </row>
     <row r="249" spans="1:21" x14ac:dyDescent="0.25">
@@ -32648,7 +32693,7 @@
       </c>
       <c r="U249" s="80">
         <f t="shared" si="7"/>
-        <v>272.07451923076923</v>
+        <v>155.47115384615384</v>
       </c>
     </row>
     <row r="250" spans="1:21" x14ac:dyDescent="0.25">
@@ -32834,7 +32879,7 @@
       </c>
       <c r="U252" s="80">
         <f t="shared" si="7"/>
-        <v>631.95990384615391</v>
+        <v>361.11994505494511</v>
       </c>
     </row>
     <row r="253" spans="1:21" x14ac:dyDescent="0.25">
@@ -33044,7 +33089,7 @@
       </c>
       <c r="U256" s="80">
         <f t="shared" si="7"/>
-        <v>4389.3273076923078</v>
+        <v>2508.1870329670332</v>
       </c>
     </row>
     <row r="257" spans="1:21" x14ac:dyDescent="0.25">
@@ -33164,7 +33209,7 @@
       </c>
       <c r="U258" s="80">
         <f t="shared" si="7"/>
-        <v>220.61403846153846</v>
+        <v>126.06516483516484</v>
       </c>
     </row>
     <row r="259" spans="1:21" x14ac:dyDescent="0.25">
@@ -33344,7 +33389,7 @@
       </c>
       <c r="U261" s="80">
         <f t="shared" si="7"/>
-        <v>1455.6618269230771</v>
+        <v>831.8067582417583</v>
       </c>
     </row>
     <row r="262" spans="1:21" x14ac:dyDescent="0.25">
@@ -33404,7 +33449,7 @@
       </c>
       <c r="U262" s="80">
         <f t="shared" si="7"/>
-        <v>540.70307692307688</v>
+        <v>308.97318681318677</v>
       </c>
     </row>
     <row r="263" spans="1:21" x14ac:dyDescent="0.25">
@@ -33470,7 +33515,7 @@
       </c>
       <c r="U263" s="80">
         <f t="shared" si="7"/>
-        <v>6606.3062499999996</v>
+        <v>3775.0321428571428</v>
       </c>
     </row>
     <row r="264" spans="1:21" x14ac:dyDescent="0.25">
@@ -33559,7 +33604,7 @@
         <v>0</v>
       </c>
       <c r="U265" s="80">
-        <f t="shared" ref="U265:U327" si="9">(T265/$V$1)/4</f>
+        <f t="shared" ref="U265:U327" si="9">(T265/$V$1)/7</f>
         <v>0</v>
       </c>
     </row>
@@ -33740,7 +33785,7 @@
       </c>
       <c r="U268" s="80">
         <f t="shared" si="9"/>
-        <v>-0.31807692307692303</v>
+        <v>-0.18175824175824173</v>
       </c>
     </row>
     <row r="269" spans="1:21" x14ac:dyDescent="0.25">
@@ -34340,7 +34385,7 @@
       </c>
       <c r="U278" s="80">
         <f t="shared" si="9"/>
-        <v>-3998.541153846154</v>
+        <v>-2284.8806593406593</v>
       </c>
     </row>
     <row r="279" spans="1:21" x14ac:dyDescent="0.25">
@@ -34646,7 +34691,7 @@
       </c>
       <c r="U283" s="80">
         <f t="shared" si="9"/>
-        <v>-3998.8592307692306</v>
+        <v>-2285.0624175824173</v>
       </c>
     </row>
     <row r="284" spans="1:21" x14ac:dyDescent="0.25">
@@ -34712,7 +34757,7 @@
       </c>
       <c r="U284" s="80">
         <f t="shared" si="9"/>
-        <v>11541.375288461539</v>
+        <v>6595.0715934065938</v>
       </c>
     </row>
     <row r="285" spans="1:21" x14ac:dyDescent="0.25">
@@ -34952,7 +34997,7 @@
       </c>
       <c r="U289" s="80">
         <f t="shared" si="9"/>
-        <v>660.28</v>
+        <v>377.30285714285714</v>
       </c>
     </row>
     <row r="290" spans="1:21" x14ac:dyDescent="0.25">
@@ -35012,7 +35057,7 @@
       </c>
       <c r="U290" s="80">
         <f t="shared" si="9"/>
-        <v>5682.0760576923076</v>
+        <v>3246.9006043956042</v>
       </c>
     </row>
     <row r="291" spans="1:21" x14ac:dyDescent="0.25">
@@ -35072,7 +35117,7 @@
       </c>
       <c r="U291" s="80">
         <f t="shared" si="9"/>
-        <v>0.71153846153846156</v>
+        <v>0.40659340659340659</v>
       </c>
     </row>
     <row r="292" spans="1:21" x14ac:dyDescent="0.25">
@@ -35132,7 +35177,7 @@
       </c>
       <c r="U292" s="80">
         <f t="shared" si="9"/>
-        <v>151.36538461538461</v>
+        <v>86.494505494505489</v>
       </c>
     </row>
     <row r="293" spans="1:21" x14ac:dyDescent="0.25">
@@ -35192,7 +35237,7 @@
       </c>
       <c r="U293" s="80">
         <f t="shared" si="9"/>
-        <v>14.639711538461539</v>
+        <v>8.3655494505494499</v>
       </c>
     </row>
     <row r="294" spans="1:21" x14ac:dyDescent="0.25">
@@ -35251,8 +35296,8 @@
         <v>39694.439999999995</v>
       </c>
       <c r="U294" s="80">
-        <f>(T294/$V$1)/4</f>
-        <v>381.67730769230764</v>
+        <f t="shared" si="9"/>
+        <v>218.10131868131865</v>
       </c>
     </row>
     <row r="295" spans="1:21" x14ac:dyDescent="0.25">
@@ -35432,7 +35477,7 @@
       </c>
       <c r="U297" s="80">
         <f t="shared" si="9"/>
-        <v>4.6392307692307693</v>
+        <v>2.6509890109890111</v>
       </c>
     </row>
     <row r="298" spans="1:21" x14ac:dyDescent="0.25">
@@ -36458,7 +36503,7 @@
       </c>
       <c r="U314" s="80">
         <f t="shared" si="9"/>
-        <v>6895.3892307692313</v>
+        <v>3940.2224175824181</v>
       </c>
     </row>
     <row r="315" spans="1:21" x14ac:dyDescent="0.25">
@@ -36728,7 +36773,7 @@
       </c>
       <c r="U319" s="80">
         <f t="shared" si="9"/>
-        <v>1.6346153846153846</v>
+        <v>0.93406593406593408</v>
       </c>
     </row>
     <row r="320" spans="1:21" x14ac:dyDescent="0.25">
@@ -37034,7 +37079,7 @@
       </c>
       <c r="U324" s="80">
         <f t="shared" si="9"/>
-        <v>1.6346153846153846</v>
+        <v>0.93406593406593408</v>
       </c>
     </row>
     <row r="325" spans="1:21" x14ac:dyDescent="0.25">
@@ -37100,7 +37145,7 @@
       </c>
       <c r="U325" s="80">
         <f t="shared" si="9"/>
-        <v>6897.0238461538474</v>
+        <v>3941.1564835164841</v>
       </c>
     </row>
     <row r="326" spans="1:21" x14ac:dyDescent="0.25">
@@ -37166,7 +37211,7 @@
       </c>
       <c r="U326" s="80">
         <f t="shared" si="9"/>
-        <v>37603.275288461526</v>
+        <v>21487.58587912087</v>
       </c>
     </row>
     <row r="327" spans="1:21" x14ac:dyDescent="0.25">
@@ -37208,7 +37253,7 @@
       </c>
       <c r="U327" s="80">
         <f t="shared" si="9"/>
-        <v>109992.69567307692</v>
+        <v>62852.968956043951</v>
       </c>
     </row>
     <row r="330" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Flash v5.15: refresh CN BC, CN Lounge, MILA OPEX from updated workbooks
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/excel/ebidta-calculation-mila-lounge.xlsx
+++ b/data/excel/ebidta-calculation-mila-lounge.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MatthiasLavenant\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA0A10D2-8EB8-4B68-B921-D8A3C17DB4D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCB63A3A-2F48-416E-BF33-9E2889CFAE5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="855" windowWidth="29040" windowHeight="15720" xr2:uid="{3C90C578-B115-41AD-8F85-41FE68FE49FA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{3C90C578-B115-41AD-8F85-41FE68FE49FA}"/>
   </bookViews>
   <sheets>
     <sheet name="EBIDTA 2" sheetId="1" r:id="rId1"/>
@@ -5579,55 +5579,6 @@
 </a:theme>
 </file>
 
-<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
-<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="350" row="12">
-    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </wetp:taskpane>
-  <wetp:taskpane dockstate="right" visibility="0" width="350" row="3">
-    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
-  </wetp:taskpane>
-</wetp:taskpanes>
-</file>
-
-<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
-<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{0D1FC6E1-D2B9-4DAA-84B1-687CE5E9F7F4}">
-  <we:reference id="WA200009404" version="1.0.0.8" store="Omex" storeType="OMEX"/>
-  <we:alternateReferences>
-    <we:reference id="WA200009404" version="1.0.0.8" store="WA200009404" storeType="OMEX"/>
-  </we:alternateReferences>
-  <we:properties>
-    <we:property name="claude.fileId" value="&quot;2d62813f-d039-4fcf-bf65-91c64db4909c&quot;"/>
-  </we:properties>
-  <we:bindings/>
-  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-  <we:extLst>
-    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
-      <we:containsCustomFunctions/>
-    </a:ext>
-  </we:extLst>
-</we:webextension>
-</file>
-
-<file path=xl/webextensions/webextension2.xml><?xml version="1.0" encoding="utf-8"?>
-<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{D09D00BA-4115-4719-8340-4946343EAEF0}">
-  <we:reference id="WA200010725" version="1.0.0.1" store="Omex" storeType="OMEX"/>
-  <we:alternateReferences>
-    <we:reference id="WA200010725" version="1.0.0.1" store="WA200010725" storeType="OMEX"/>
-  </we:alternateReferences>
-  <we:properties>
-    <we:property name="claude.fileId" value="&quot;0274738e-1f28-498a-8004-0266299e1695&quot;"/>
-  </we:properties>
-  <we:bindings/>
-  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-  <we:extLst>
-    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
-      <we:containsCustomFunctions/>
-    </a:ext>
-  </we:extLst>
-</we:webextension>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B26BDD18-EC06-4B8C-8F68-C4E97E1A8EA4}">
   <sheetPr>
@@ -7467,11 +7418,11 @@
       </c>
       <c r="D46" s="34">
         <f>'OPEX DATA 2'!U143</f>
-        <v>5487.53467032967</v>
+        <v>9603.1856730769232</v>
       </c>
       <c r="E46" s="20">
         <f>D46/D$36</f>
-        <v>8.9959584759502789E-2</v>
+        <v>0.1574292733291299</v>
       </c>
     </row>
     <row r="47" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7480,11 +7431,11 @@
       </c>
       <c r="D47" s="34">
         <f>'OPEX DATA 2'!U119</f>
-        <v>3354.3092857142851</v>
+        <v>5870.0412499999993</v>
       </c>
       <c r="E47" s="20">
         <f t="shared" ref="E47:E50" si="2">D47/D$36</f>
-        <v>5.4988676814988278E-2</v>
+        <v>9.6230184426229493E-2</v>
       </c>
     </row>
     <row r="48" spans="2:175" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7503,11 +7454,11 @@
       </c>
       <c r="D49" s="34">
         <f>'OPEX DATA 2'!U151</f>
-        <v>2038.0992307692306</v>
+        <v>3566.6736538461537</v>
       </c>
       <c r="E49" s="20">
         <f t="shared" si="2"/>
-        <v>3.3411462799495584E-2</v>
+        <v>5.8470059899117272E-2</v>
       </c>
     </row>
     <row r="50" spans="2:175" x14ac:dyDescent="0.25">
@@ -7517,11 +7468,11 @@
       <c r="C50" s="22"/>
       <c r="D50" s="45">
         <f>SUM(D46:D49)</f>
-        <v>10879.943186813185</v>
+        <v>19039.900576923079</v>
       </c>
       <c r="E50" s="46">
         <f t="shared" si="2"/>
-        <v>0.17835972437398664</v>
+        <v>0.31212951765447672</v>
       </c>
     </row>
     <row r="52" spans="2:175" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -10657,11 +10608,11 @@
       <c r="C203" s="48"/>
       <c r="D203" s="49">
         <f>D43-D50-D101-D130-D141-D152-D172-D201</f>
-        <v>8695.511318681316</v>
+        <v>535.55392857142397</v>
       </c>
       <c r="E203" s="50">
         <f>D203/D36</f>
-        <v>0.14254936588002157</v>
+        <v>8.7795725995315401E-3</v>
       </c>
       <c r="F203" s="50"/>
       <c r="G203" s="50"/>
@@ -10687,7 +10638,7 @@
       <c r="C207" s="63"/>
       <c r="D207" s="64">
         <f>E203</f>
-        <v>0.14254936588002157</v>
+        <v>8.7795725995315401E-3</v>
       </c>
     </row>
     <row r="208" spans="2:175" s="20" customFormat="1" x14ac:dyDescent="0.25">
@@ -23010,8 +22961,8 @@
         <v>146297.47</v>
       </c>
       <c r="U85" s="80">
-        <f t="shared" si="3"/>
-        <v>803.83225274725271</v>
+        <f>(T85/$V$1)/4</f>
+        <v>1406.7064423076922</v>
       </c>
     </row>
     <row r="86" spans="1:21" x14ac:dyDescent="0.25">
@@ -23070,8 +23021,8 @@
         <v>37991.369999999995</v>
       </c>
       <c r="U86" s="80">
-        <f t="shared" si="3"/>
-        <v>208.74379120879118</v>
+        <f t="shared" ref="U86:U149" si="4">(T86/$V$1)/4</f>
+        <v>365.30163461538456</v>
       </c>
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
@@ -23130,8 +23081,8 @@
         <v>19393.099999999999</v>
       </c>
       <c r="U87" s="80">
-        <f t="shared" si="3"/>
-        <v>106.55549450549449</v>
+        <f t="shared" si="4"/>
+        <v>186.47211538461536</v>
       </c>
     </row>
     <row r="88" spans="1:21" x14ac:dyDescent="0.25">
@@ -23190,8 +23141,8 @@
         <v>142168.22</v>
       </c>
       <c r="U88" s="80">
-        <f t="shared" si="3"/>
-        <v>781.14406593406591</v>
+        <f t="shared" si="4"/>
+        <v>1367.0021153846153</v>
       </c>
     </row>
     <row r="89" spans="1:21" x14ac:dyDescent="0.25">
@@ -23250,8 +23201,8 @@
         <v>1104.32</v>
       </c>
       <c r="U89" s="80">
-        <f t="shared" si="3"/>
-        <v>6.0676923076923073</v>
+        <f t="shared" si="4"/>
+        <v>10.618461538461538</v>
       </c>
     </row>
     <row r="90" spans="1:21" x14ac:dyDescent="0.25">
@@ -23310,7 +23261,7 @@
         <v>0</v>
       </c>
       <c r="U90" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -23370,7 +23321,7 @@
         <v>0</v>
       </c>
       <c r="U91" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -23430,8 +23381,8 @@
         <v>67056.09</v>
       </c>
       <c r="U92" s="80">
-        <f t="shared" si="3"/>
-        <v>368.4400549450549</v>
+        <f t="shared" si="4"/>
+        <v>644.77009615384611</v>
       </c>
     </row>
     <row r="93" spans="1:21" x14ac:dyDescent="0.25">
@@ -23490,7 +23441,7 @@
         <v>0</v>
       </c>
       <c r="U93" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -23550,7 +23501,7 @@
         <v>0</v>
       </c>
       <c r="U94" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -23610,7 +23561,7 @@
         <v>0</v>
       </c>
       <c r="U95" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -23670,8 +23621,8 @@
         <v>7000</v>
       </c>
       <c r="U96" s="80">
-        <f t="shared" si="3"/>
-        <v>38.46153846153846</v>
+        <f t="shared" si="4"/>
+        <v>67.307692307692307</v>
       </c>
     </row>
     <row r="97" spans="1:21" x14ac:dyDescent="0.25">
@@ -23730,8 +23681,8 @@
         <v>51415.28</v>
       </c>
       <c r="U97" s="80">
-        <f t="shared" si="3"/>
-        <v>282.50153846153847</v>
+        <f t="shared" si="4"/>
+        <v>494.37769230769231</v>
       </c>
     </row>
     <row r="98" spans="1:21" x14ac:dyDescent="0.25">
@@ -23790,8 +23741,8 @@
         <v>42496.24</v>
       </c>
       <c r="U98" s="80">
-        <f t="shared" si="3"/>
-        <v>233.49582417582414</v>
+        <f t="shared" si="4"/>
+        <v>408.61769230769227</v>
       </c>
     </row>
     <row r="99" spans="1:21" x14ac:dyDescent="0.25">
@@ -23850,7 +23801,7 @@
         <v>0</v>
       </c>
       <c r="U99" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -23910,7 +23861,7 @@
         <v>0</v>
       </c>
       <c r="U100" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -23970,7 +23921,7 @@
         <v>0</v>
       </c>
       <c r="U101" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -24030,7 +23981,7 @@
         <v>0</v>
       </c>
       <c r="U102" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -24090,7 +24041,7 @@
         <v>0</v>
       </c>
       <c r="U103" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -24150,7 +24101,7 @@
         <v>0</v>
       </c>
       <c r="U104" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -24210,7 +24161,7 @@
         <v>0</v>
       </c>
       <c r="U105" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -24270,7 +24221,7 @@
         <v>0</v>
       </c>
       <c r="U106" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -24330,7 +24281,7 @@
         <v>0</v>
       </c>
       <c r="U107" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -24390,7 +24341,7 @@
         <v>0</v>
       </c>
       <c r="U108" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -24450,7 +24401,7 @@
         <v>0</v>
       </c>
       <c r="U109" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -24510,8 +24461,8 @@
         <v>56683.159999999989</v>
       </c>
       <c r="U110" s="80">
-        <f t="shared" si="3"/>
-        <v>311.44593406593401</v>
+        <f t="shared" si="4"/>
+        <v>545.03038461538449</v>
       </c>
     </row>
     <row r="111" spans="1:21" x14ac:dyDescent="0.25">
@@ -24570,7 +24521,7 @@
         <v>0</v>
       </c>
       <c r="U111" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -24630,8 +24581,8 @@
         <v>34534.559999999998</v>
       </c>
       <c r="U112" s="80">
-        <f t="shared" si="3"/>
-        <v>189.75032967032965</v>
+        <f t="shared" si="4"/>
+        <v>332.06307692307689</v>
       </c>
     </row>
     <row r="113" spans="1:23" x14ac:dyDescent="0.25">
@@ -24690,7 +24641,7 @@
         <v>0</v>
       </c>
       <c r="U113" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -24750,8 +24701,8 @@
         <v>1546.5300000000002</v>
       </c>
       <c r="U114" s="80">
-        <f t="shared" si="3"/>
-        <v>8.497417582417583</v>
+        <f t="shared" si="4"/>
+        <v>14.87048076923077</v>
       </c>
     </row>
     <row r="115" spans="1:23" x14ac:dyDescent="0.25">
@@ -24810,7 +24761,7 @@
         <v>0</v>
       </c>
       <c r="U115" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -24870,7 +24821,7 @@
         <v>0</v>
       </c>
       <c r="U116" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -24930,7 +24881,7 @@
         <v>0</v>
       </c>
       <c r="U117" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -24990,8 +24941,8 @@
         <v>2797.95</v>
       </c>
       <c r="U118" s="80">
-        <f t="shared" si="3"/>
-        <v>15.373351648351647</v>
+        <f t="shared" si="4"/>
+        <v>26.903365384615384</v>
       </c>
     </row>
     <row r="119" spans="1:23" x14ac:dyDescent="0.25">
@@ -25056,8 +25007,8 @@
         <v>610484.28999999992</v>
       </c>
       <c r="U119" s="80">
-        <f t="shared" si="3"/>
-        <v>3354.3092857142851</v>
+        <f t="shared" si="4"/>
+        <v>5870.0412499999993</v>
       </c>
     </row>
     <row r="120" spans="1:23" x14ac:dyDescent="0.25">
@@ -25122,12 +25073,12 @@
         <v>610484.28999999992</v>
       </c>
       <c r="U120" s="80">
-        <f t="shared" si="3"/>
-        <v>3354.3092857142851</v>
+        <f t="shared" si="4"/>
+        <v>5870.0412499999993</v>
       </c>
       <c r="W120" s="80">
         <f>U120+U143+U151</f>
-        <v>10879.943186813185</v>
+        <v>19039.900576923079</v>
       </c>
     </row>
     <row r="121" spans="1:23" x14ac:dyDescent="0.25">
@@ -25156,7 +25107,7 @@
         <v>0</v>
       </c>
       <c r="U121" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -25216,7 +25167,7 @@
         <v>0</v>
       </c>
       <c r="U122" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -25276,8 +25227,8 @@
         <v>73947.599999999991</v>
       </c>
       <c r="U123" s="80">
-        <f t="shared" si="3"/>
-        <v>406.30549450549449</v>
+        <f t="shared" si="4"/>
+        <v>711.03461538461534</v>
       </c>
     </row>
     <row r="124" spans="1:23" x14ac:dyDescent="0.25">
@@ -25336,8 +25287,8 @@
         <v>142076.88</v>
       </c>
       <c r="U124" s="80">
-        <f t="shared" si="3"/>
-        <v>780.64219780219787</v>
+        <f t="shared" si="4"/>
+        <v>1366.1238461538462</v>
       </c>
     </row>
     <row r="125" spans="1:23" ht="31.5" x14ac:dyDescent="0.25">
@@ -25396,7 +25347,7 @@
         <v>0</v>
       </c>
       <c r="U125" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -25456,7 +25407,7 @@
         <v>0</v>
       </c>
       <c r="U126" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -25516,7 +25467,7 @@
         <v>0</v>
       </c>
       <c r="U127" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -25576,7 +25527,7 @@
         <v>0</v>
       </c>
       <c r="U128" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -25636,7 +25587,7 @@
         <v>0</v>
       </c>
       <c r="U129" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -25696,8 +25647,8 @@
         <v>-8038</v>
       </c>
       <c r="U130" s="80">
-        <f t="shared" si="3"/>
-        <v>-44.164835164835161</v>
+        <f t="shared" si="4"/>
+        <v>-77.288461538461533</v>
       </c>
     </row>
     <row r="131" spans="1:21" x14ac:dyDescent="0.25">
@@ -25756,7 +25707,7 @@
         <v>0</v>
       </c>
       <c r="U131" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -25816,7 +25767,7 @@
         <v>0</v>
       </c>
       <c r="U132" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -25876,7 +25827,7 @@
         <v>0</v>
       </c>
       <c r="U133" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -25936,7 +25887,7 @@
         <v>0</v>
       </c>
       <c r="U134" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -25996,7 +25947,7 @@
         <v>0</v>
       </c>
       <c r="U135" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -26056,7 +26007,7 @@
         <v>0</v>
       </c>
       <c r="U136" s="80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -26112,11 +26063,11 @@
         <v>0</v>
       </c>
       <c r="T137" s="80">
-        <f t="shared" ref="T137:T200" si="4">IFERROR(B137+E137+H137+K137+N137+Q137, "NA")</f>
+        <f t="shared" ref="T137:T200" si="5">IFERROR(B137+E137+H137+K137+N137+Q137, "NA")</f>
         <v>0</v>
       </c>
       <c r="U137" s="80">
-        <f t="shared" ref="U137:U200" si="5">(T137/$V$1)/7</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -26172,11 +26123,11 @@
         <v>0</v>
       </c>
       <c r="T138" s="80">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="U138" s="80">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="U138" s="80">
-        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -26232,12 +26183,12 @@
         <v>4.7290061959126717E-2</v>
       </c>
       <c r="T139" s="80">
+        <f t="shared" si="5"/>
+        <v>440915.44</v>
+      </c>
+      <c r="U139" s="80">
         <f t="shared" si="4"/>
-        <v>440915.44</v>
-      </c>
-      <c r="U139" s="80">
-        <f t="shared" si="5"/>
-        <v>2422.6123076923077</v>
+        <v>4239.5715384615387</v>
       </c>
     </row>
     <row r="140" spans="1:21" x14ac:dyDescent="0.25">
@@ -26292,11 +26243,11 @@
         <v>0</v>
       </c>
       <c r="T140" s="80">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="U140" s="80">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="U140" s="80">
-        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -26352,12 +26303,12 @@
         <v>2.575100851712453E-2</v>
       </c>
       <c r="T141" s="80">
+        <f t="shared" si="5"/>
+        <v>246314.38999999998</v>
+      </c>
+      <c r="U141" s="80">
         <f t="shared" si="4"/>
-        <v>246314.38999999998</v>
-      </c>
-      <c r="U141" s="80">
-        <f t="shared" si="5"/>
-        <v>1353.3757692307693</v>
+        <v>2368.407596153846</v>
       </c>
     </row>
     <row r="142" spans="1:21" x14ac:dyDescent="0.25">
@@ -26412,12 +26363,12 @@
         <v>1.2194785520668432E-2</v>
       </c>
       <c r="T142" s="80">
+        <f t="shared" si="5"/>
+        <v>103515</v>
+      </c>
+      <c r="U142" s="80">
         <f t="shared" si="4"/>
-        <v>103515</v>
-      </c>
-      <c r="U142" s="80">
-        <f t="shared" si="5"/>
-        <v>568.76373626373629</v>
+        <v>995.33653846153845</v>
       </c>
     </row>
     <row r="143" spans="1:21" x14ac:dyDescent="0.25">
@@ -26478,12 +26429,12 @@
         <v>0.11883158542729114</v>
       </c>
       <c r="T143" s="80">
+        <f t="shared" si="5"/>
+        <v>998731.31</v>
+      </c>
+      <c r="U143" s="80">
         <f t="shared" si="4"/>
-        <v>998731.31</v>
-      </c>
-      <c r="U143" s="80">
-        <f t="shared" si="5"/>
-        <v>5487.53467032967</v>
+        <v>9603.1856730769232</v>
       </c>
     </row>
     <row r="144" spans="1:21" x14ac:dyDescent="0.25">
@@ -26508,11 +26459,11 @@
       <c r="Q144" s="72"/>
       <c r="R144" s="73"/>
       <c r="T144" s="80">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="U144" s="80">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="U144" s="80">
-        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -26568,11 +26519,11 @@
         <v>0</v>
       </c>
       <c r="T145" s="80">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="U145" s="80">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="U145" s="80">
-        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -26628,12 +26579,12 @@
         <v>3.1885698564379561E-2</v>
       </c>
       <c r="T146" s="80">
+        <f t="shared" si="5"/>
+        <v>212769.00999999998</v>
+      </c>
+      <c r="U146" s="80">
         <f t="shared" si="4"/>
-        <v>212769.00999999998</v>
-      </c>
-      <c r="U146" s="80">
-        <f t="shared" si="5"/>
-        <v>1169.0604945054945</v>
+        <v>2045.8558653846153</v>
       </c>
     </row>
     <row r="147" spans="1:21" x14ac:dyDescent="0.25">
@@ -26688,12 +26639,12 @@
         <v>1.9259716327100723E-3</v>
       </c>
       <c r="T147" s="80">
+        <f t="shared" si="5"/>
+        <v>38159.67</v>
+      </c>
+      <c r="U147" s="80">
         <f t="shared" si="4"/>
-        <v>38159.67</v>
-      </c>
-      <c r="U147" s="80">
-        <f t="shared" si="5"/>
-        <v>209.66851648351647</v>
+        <v>366.91990384615383</v>
       </c>
     </row>
     <row r="148" spans="1:21" x14ac:dyDescent="0.25">
@@ -26748,12 +26699,12 @@
         <v>2.7230407493332026E-3</v>
       </c>
       <c r="T148" s="80">
+        <f t="shared" si="5"/>
+        <v>26432.370000000003</v>
+      </c>
+      <c r="U148" s="80">
         <f t="shared" si="4"/>
-        <v>26432.370000000003</v>
-      </c>
-      <c r="U148" s="80">
-        <f t="shared" si="5"/>
-        <v>145.23280219780222</v>
+        <v>254.15740384615387</v>
       </c>
     </row>
     <row r="149" spans="1:21" x14ac:dyDescent="0.25">
@@ -26808,12 +26759,12 @@
         <v>3.855230386184716E-3</v>
       </c>
       <c r="T149" s="80">
+        <f t="shared" si="5"/>
+        <v>30530</v>
+      </c>
+      <c r="U149" s="80">
         <f t="shared" si="4"/>
-        <v>30530</v>
-      </c>
-      <c r="U149" s="80">
-        <f t="shared" si="5"/>
-        <v>167.74725274725276</v>
+        <v>293.55769230769232</v>
       </c>
     </row>
     <row r="150" spans="1:21" x14ac:dyDescent="0.25">
@@ -26868,12 +26819,12 @@
         <v>4.7287322691822904E-3</v>
       </c>
       <c r="T150" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>63043.01</v>
       </c>
       <c r="U150" s="80">
-        <f t="shared" si="5"/>
-        <v>346.39016483516485</v>
+        <f t="shared" ref="U150:U156" si="6">(T150/$V$1)/4</f>
+        <v>606.18278846153851</v>
       </c>
     </row>
     <row r="151" spans="1:21" x14ac:dyDescent="0.25">
@@ -26934,12 +26885,12 @@
         <v>4.5118673601789838E-2</v>
       </c>
       <c r="T151" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>370934.06</v>
       </c>
       <c r="U151" s="80">
-        <f t="shared" si="5"/>
-        <v>2038.0992307692306</v>
+        <f t="shared" si="6"/>
+        <v>3566.6736538461537</v>
       </c>
     </row>
     <row r="152" spans="1:21" x14ac:dyDescent="0.25">
@@ -26994,11 +26945,11 @@
         <v>0</v>
       </c>
       <c r="T152" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="U152" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -27054,12 +27005,12 @@
         <v>1.1786000335762086E-2</v>
       </c>
       <c r="T153" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>82274.98</v>
       </c>
       <c r="U153" s="80">
-        <f t="shared" si="5"/>
-        <v>452.06032967032968</v>
+        <f t="shared" si="6"/>
+        <v>791.10557692307691</v>
       </c>
     </row>
     <row r="154" spans="1:21" x14ac:dyDescent="0.25">
@@ -27114,12 +27065,12 @@
         <v>1.9234702491458043E-4</v>
       </c>
       <c r="T154" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1788.63</v>
       </c>
       <c r="U154" s="80">
-        <f t="shared" si="5"/>
-        <v>9.827637362637363</v>
+        <f t="shared" si="6"/>
+        <v>17.198365384615386</v>
       </c>
     </row>
     <row r="155" spans="1:21" x14ac:dyDescent="0.25">
@@ -27174,12 +27125,12 @@
         <v>-8.9458703263873764E-6</v>
       </c>
       <c r="T155" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>33.700000000000017</v>
       </c>
       <c r="U155" s="80">
-        <f t="shared" si="5"/>
-        <v>0.18516483516483526</v>
+        <f t="shared" si="6"/>
+        <v>0.32403846153846172</v>
       </c>
     </row>
     <row r="156" spans="1:21" x14ac:dyDescent="0.25">
@@ -27234,11 +27185,11 @@
         <v>0</v>
       </c>
       <c r="T156" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="U156" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -27300,11 +27251,11 @@
         <v>0.39069146654150411</v>
       </c>
       <c r="T157" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>3982090.75</v>
       </c>
       <c r="U157" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="U137:U200" si="7">(T157/$V$1)/7</f>
         <v>21879.619505494506</v>
       </c>
     </row>
@@ -27330,11 +27281,11 @@
       <c r="Q158" s="72"/>
       <c r="R158" s="73"/>
       <c r="T158" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="U158" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -27360,11 +27311,11 @@
       <c r="Q159" s="72"/>
       <c r="R159" s="73"/>
       <c r="T159" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="U159" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -27420,11 +27371,11 @@
         <v>0</v>
       </c>
       <c r="T160" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="U160" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -27480,11 +27431,11 @@
         <v>9.4432635999737813E-7</v>
       </c>
       <c r="T161" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>28.08</v>
       </c>
       <c r="U161" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.15428571428571428</v>
       </c>
     </row>
@@ -27540,11 +27491,11 @@
         <v>1.1936717706256934E-4</v>
       </c>
       <c r="T162" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>15861.32</v>
       </c>
       <c r="U162" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>87.150109890109889</v>
       </c>
     </row>
@@ -27600,11 +27551,11 @@
         <v>0</v>
       </c>
       <c r="T163" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>25546.41</v>
       </c>
       <c r="U163" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>140.36489010989013</v>
       </c>
     </row>
@@ -27660,11 +27611,11 @@
         <v>0</v>
       </c>
       <c r="T164" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>4000.52</v>
       </c>
       <c r="U164" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>21.98087912087912</v>
       </c>
     </row>
@@ -27720,11 +27671,11 @@
         <v>6.9346714375379975E-6</v>
       </c>
       <c r="T165" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>4282.0999999999995</v>
       </c>
       <c r="U165" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>23.528021978021975</v>
       </c>
     </row>
@@ -27780,11 +27731,11 @@
         <v>3.2215801900283073E-3</v>
       </c>
       <c r="T166" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>23991.940000000002</v>
       </c>
       <c r="U166" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>131.82384615384618</v>
       </c>
     </row>
@@ -27840,11 +27791,11 @@
         <v>2.3054971176528355E-3</v>
       </c>
       <c r="T167" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>17993.730000000003</v>
       </c>
       <c r="U167" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>98.866648351648365</v>
       </c>
     </row>
@@ -27900,11 +27851,11 @@
         <v>6.7782664830886618E-3</v>
       </c>
       <c r="T168" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>73699.940000000017</v>
       </c>
       <c r="U168" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>404.94472527472539</v>
       </c>
     </row>
@@ -27960,11 +27911,11 @@
         <v>3.6702577571959163E-4</v>
       </c>
       <c r="T169" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>3742.88</v>
       </c>
       <c r="U169" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>20.565274725274726</v>
       </c>
     </row>
@@ -28020,11 +27971,11 @@
         <v>2.6713911434600641E-3</v>
       </c>
       <c r="T170" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>26272.66</v>
       </c>
       <c r="U170" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>144.35527472527471</v>
       </c>
     </row>
@@ -28080,11 +28031,11 @@
         <v>1.0976676602253493E-3</v>
       </c>
       <c r="T171" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>29054.15</v>
       </c>
       <c r="U171" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>159.63818681318682</v>
       </c>
     </row>
@@ -28140,11 +28091,11 @@
         <v>0</v>
       </c>
       <c r="T172" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="U172" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -28200,11 +28151,11 @@
         <v>0</v>
       </c>
       <c r="T173" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="U173" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -28260,11 +28211,11 @@
         <v>0</v>
       </c>
       <c r="T174" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="U174" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -28320,11 +28271,11 @@
         <v>3.4541656099162108E-3</v>
       </c>
       <c r="T175" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>28102.33</v>
       </c>
       <c r="U175" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>154.4084065934066</v>
       </c>
     </row>
@@ -28380,11 +28331,11 @@
         <v>3.5356011434191908E-3</v>
       </c>
       <c r="T176" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>26920.400000000001</v>
       </c>
       <c r="U176" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>147.91428571428574</v>
       </c>
     </row>
@@ -28440,11 +28391,11 @@
         <v>3.8021318520798249E-3</v>
       </c>
       <c r="T177" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>21729.399999999998</v>
       </c>
       <c r="U177" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>119.39230769230768</v>
       </c>
     </row>
@@ -28500,11 +28451,11 @@
         <v>3.2311820427879755E-4</v>
       </c>
       <c r="T178" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>30899.310000000005</v>
       </c>
       <c r="U178" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>169.7764285714286</v>
       </c>
     </row>
@@ -28560,11 +28511,11 @@
         <v>1.4026706573081664E-3</v>
       </c>
       <c r="T179" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>10355.58</v>
       </c>
       <c r="U179" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>56.898791208791202</v>
       </c>
     </row>
@@ -28620,11 +28571,11 @@
         <v>5.8284399626891605E-3</v>
       </c>
       <c r="T180" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>54461.990000000005</v>
       </c>
       <c r="U180" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>299.24170329670329</v>
       </c>
     </row>
@@ -28680,11 +28631,11 @@
         <v>0</v>
       </c>
       <c r="T181" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="U181" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -28740,11 +28691,11 @@
         <v>6.4250235470661297E-5</v>
       </c>
       <c r="T182" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>399.49</v>
       </c>
       <c r="U182" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>2.1949999999999998</v>
       </c>
     </row>
@@ -28800,11 +28751,11 @@
         <v>1.8824965771593535E-3</v>
       </c>
       <c r="T183" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>15237.73</v>
       </c>
       <c r="U183" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>83.723791208791212</v>
       </c>
     </row>
@@ -28860,11 +28811,11 @@
         <v>3.8788745881754901E-4</v>
       </c>
       <c r="T184" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>5306.33</v>
       </c>
       <c r="U184" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>29.155659340659337</v>
       </c>
     </row>
@@ -28920,11 +28871,11 @@
         <v>0</v>
       </c>
       <c r="T185" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="U185" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -28980,11 +28931,11 @@
         <v>0</v>
       </c>
       <c r="T186" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="U186" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -29040,11 +28991,11 @@
         <v>2.2789262248058863E-4</v>
       </c>
       <c r="T187" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>2183.71</v>
       </c>
       <c r="U187" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>11.998406593406594</v>
       </c>
     </row>
@@ -29100,11 +29051,11 @@
         <v>1.9252723986877844E-3</v>
       </c>
       <c r="T188" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>18622.71</v>
       </c>
       <c r="U188" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>102.32258241758242</v>
       </c>
     </row>
@@ -29160,11 +29111,11 @@
         <v>3.6196173550662862E-3</v>
       </c>
       <c r="T189" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>31038.239999999998</v>
       </c>
       <c r="U189" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>170.5397802197802</v>
       </c>
     </row>
@@ -29220,11 +29171,11 @@
         <v>0</v>
       </c>
       <c r="T190" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1243.45</v>
       </c>
       <c r="U190" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>6.8321428571428573</v>
       </c>
     </row>
@@ -29280,11 +29231,11 @@
         <v>0</v>
       </c>
       <c r="T191" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="U191" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -29340,11 +29291,11 @@
         <v>1.5283381491694968E-3</v>
       </c>
       <c r="T192" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>17653.29</v>
       </c>
       <c r="U192" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>96.996098901098904</v>
       </c>
     </row>
@@ -29400,11 +29351,11 @@
         <v>1.4903964135724725E-2</v>
       </c>
       <c r="T193" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>129076.53</v>
       </c>
       <c r="U193" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>709.21170329670326</v>
       </c>
     </row>
@@ -29460,11 +29411,11 @@
         <v>9.8002189640527902E-3</v>
       </c>
       <c r="T194" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>62157.31</v>
       </c>
       <c r="U194" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>341.52368131868127</v>
       </c>
     </row>
@@ -29520,11 +29471,11 @@
         <v>8.2629998219404166E-4</v>
       </c>
       <c r="T195" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>7739.7800000000007</v>
       </c>
       <c r="U195" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>42.526263736263736</v>
       </c>
     </row>
@@ -29580,11 +29531,11 @@
         <v>9.7403717403430928E-2</v>
       </c>
       <c r="T196" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>935408.21</v>
       </c>
       <c r="U196" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>5139.605549450549</v>
       </c>
     </row>
@@ -29640,11 +29591,11 @@
         <v>2.1175977978078609E-4</v>
       </c>
       <c r="T197" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>2995.2799999999997</v>
       </c>
       <c r="U197" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>16.457582417582415</v>
       </c>
     </row>
@@ -29700,11 +29651,11 @@
         <v>0</v>
       </c>
       <c r="T198" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="U198" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -29760,11 +29711,11 @@
         <v>0</v>
       </c>
       <c r="T199" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="U199" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -29820,11 +29771,11 @@
         <v>0</v>
       </c>
       <c r="T200" s="80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="U200" s="80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -29880,11 +29831,11 @@
         <v>5.025546298746352E-4</v>
       </c>
       <c r="T201" s="80">
-        <f t="shared" ref="T201:T264" si="6">IFERROR(B201+E201+H201+K201+N201+Q201, "NA")</f>
+        <f t="shared" ref="T201:T264" si="8">IFERROR(B201+E201+H201+K201+N201+Q201, "NA")</f>
         <v>2810.66</v>
       </c>
       <c r="U201" s="80">
-        <f t="shared" ref="U201:U264" si="7">(T201/$V$1)/7</f>
+        <f t="shared" ref="U201:U264" si="9">(T201/$V$1)/7</f>
         <v>15.443186813186813</v>
       </c>
     </row>
@@ -29940,11 +29891,11 @@
         <v>0</v>
       </c>
       <c r="T202" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U202" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -30000,11 +29951,11 @@
         <v>0</v>
       </c>
       <c r="T203" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U203" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -30060,11 +30011,11 @@
         <v>0</v>
       </c>
       <c r="T204" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U204" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -30120,11 +30071,11 @@
         <v>0</v>
       </c>
       <c r="T205" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U205" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -30180,11 +30131,11 @@
         <v>0</v>
       </c>
       <c r="T206" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U206" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -30240,11 +30191,11 @@
         <v>0</v>
       </c>
       <c r="T207" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U207" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -30300,11 +30251,11 @@
         <v>0</v>
       </c>
       <c r="T208" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U208" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -30366,11 +30317,11 @@
         <v>0.16819907166663592</v>
       </c>
       <c r="T209" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1628815.4600000002</v>
       </c>
       <c r="U209" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>8949.5354945054951</v>
       </c>
     </row>
@@ -30426,11 +30377,11 @@
         <v>0</v>
       </c>
       <c r="T210" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U210" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -30492,11 +30443,11 @@
         <v>0.16819907166663592</v>
       </c>
       <c r="T211" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1628815.4600000002</v>
       </c>
       <c r="U211" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>8949.5354945054951</v>
       </c>
     </row>
@@ -30522,11 +30473,11 @@
       <c r="Q212" s="72"/>
       <c r="R212" s="73"/>
       <c r="T212" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U212" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -30552,11 +30503,11 @@
       <c r="Q213" s="72"/>
       <c r="R213" s="73"/>
       <c r="T213" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U213" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -30612,11 +30563,11 @@
         <v>0</v>
       </c>
       <c r="T214" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U214" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -30672,11 +30623,11 @@
         <v>3.0306734430276771E-2</v>
       </c>
       <c r="T215" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>353594.51</v>
       </c>
       <c r="U215" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>1942.826978021978</v>
       </c>
     </row>
@@ -30732,11 +30683,11 @@
         <v>3.2366605773955935E-4</v>
       </c>
       <c r="T216" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>5104</v>
       </c>
       <c r="U216" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>28.043956043956047</v>
       </c>
     </row>
@@ -30792,11 +30743,11 @@
         <v>1.8089890599214505E-2</v>
       </c>
       <c r="T217" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>77639.430000000008</v>
       </c>
       <c r="U217" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>426.59027472527475</v>
       </c>
     </row>
@@ -30852,11 +30803,11 @@
         <v>-1.9189288323000158E-5</v>
       </c>
       <c r="T218" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>6234.84</v>
       </c>
       <c r="U218" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>34.25736263736264</v>
       </c>
     </row>
@@ -30912,11 +30863,11 @@
         <v>2.3433775801654327E-2</v>
       </c>
       <c r="T219" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>144630.38</v>
       </c>
       <c r="U219" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>794.67241758241755</v>
       </c>
     </row>
@@ -30972,11 +30923,11 @@
         <v>6.1460507979676685E-5</v>
       </c>
       <c r="T220" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>3343.92</v>
       </c>
       <c r="U220" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>18.373186813186813</v>
       </c>
     </row>
@@ -31032,11 +30983,11 @@
         <v>0</v>
       </c>
       <c r="T221" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U221" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -31092,11 +31043,11 @@
         <v>0</v>
       </c>
       <c r="T222" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1601.1299999999999</v>
       </c>
       <c r="U222" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>8.797417582417582</v>
       </c>
     </row>
@@ -31152,11 +31103,11 @@
         <v>5.355988438763755E-6</v>
       </c>
       <c r="T223" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>7.43</v>
       </c>
       <c r="U223" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>4.0824175824175822E-2</v>
       </c>
     </row>
@@ -31212,11 +31163,11 @@
         <v>1.0268648090200496E-4</v>
       </c>
       <c r="T224" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>692.71</v>
       </c>
       <c r="U224" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>3.8060989010989013</v>
       </c>
     </row>
@@ -31272,11 +31223,11 @@
         <v>0</v>
       </c>
       <c r="T225" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U225" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -31332,11 +31283,11 @@
         <v>-2.1222113006353293E-5</v>
       </c>
       <c r="T226" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>-136.44</v>
       </c>
       <c r="U226" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-0.74967032967032965</v>
       </c>
     </row>
@@ -31392,11 +31343,11 @@
         <v>1.8994872430411385E-3</v>
       </c>
       <c r="T227" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>21583.73</v>
       </c>
       <c r="U227" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>118.59192307692308</v>
       </c>
     </row>
@@ -31452,11 +31403,11 @@
         <v>6.8276237547444012E-4</v>
       </c>
       <c r="T228" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>4424.13</v>
       </c>
       <c r="U228" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>24.308406593406595</v>
       </c>
     </row>
@@ -31512,11 +31463,11 @@
         <v>0</v>
       </c>
       <c r="T229" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>111</v>
       </c>
       <c r="U229" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.60989010989010983</v>
       </c>
     </row>
@@ -31572,11 +31523,11 @@
         <v>3.6042990839594584E-3</v>
       </c>
       <c r="T230" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>14911.8</v>
       </c>
       <c r="U230" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>81.932967032967028</v>
       </c>
     </row>
@@ -31632,11 +31583,11 @@
         <v>0</v>
       </c>
       <c r="T231" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U231" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -31692,11 +31643,11 @@
         <v>0</v>
       </c>
       <c r="T232" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>500</v>
       </c>
       <c r="U232" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>2.7472527472527473</v>
       </c>
     </row>
@@ -31752,11 +31703,11 @@
         <v>6.5901004451114734E-5</v>
       </c>
       <c r="T233" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>91.42</v>
       </c>
       <c r="U233" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.50230769230769234</v>
       </c>
     </row>
@@ -31812,11 +31763,11 @@
         <v>3.2083307865956722E-4</v>
       </c>
       <c r="T234" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>791.53</v>
       </c>
       <c r="U234" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>4.3490659340659343</v>
       </c>
     </row>
@@ -31872,11 +31823,11 @@
         <v>1.0105733771605529E-4</v>
       </c>
       <c r="T235" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>6540.71</v>
       </c>
       <c r="U235" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>35.93796703296703</v>
       </c>
     </row>
@@ -31932,11 +31883,11 @@
         <v>2.360300485224439E-2</v>
       </c>
       <c r="T236" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>204779.23</v>
       </c>
       <c r="U236" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>1125.1606043956044</v>
       </c>
     </row>
@@ -31992,11 +31943,11 @@
         <v>3.9337320202333532E-4</v>
       </c>
       <c r="T237" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>14802.460000000001</v>
       </c>
       <c r="U237" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>81.332197802197811</v>
       </c>
     </row>
@@ -32052,11 +32003,11 @@
         <v>1.151933987233443E-5</v>
       </c>
       <c r="T238" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>2156.79</v>
       </c>
       <c r="U238" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>11.850494505494506</v>
       </c>
     </row>
@@ -32112,11 +32063,11 @@
         <v>0</v>
       </c>
       <c r="T239" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U239" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -32172,11 +32123,11 @@
         <v>0</v>
       </c>
       <c r="T240" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U240" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -32238,11 +32189,11 @@
         <v>0.10296539598231809</v>
       </c>
       <c r="T241" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>863404.71000000008</v>
       </c>
       <c r="U241" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>4743.9819230769235</v>
       </c>
     </row>
@@ -32268,11 +32219,11 @@
       <c r="Q242" s="72"/>
       <c r="R242" s="73"/>
       <c r="T242" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U242" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -32328,11 +32279,11 @@
         <v>0</v>
       </c>
       <c r="T243" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U243" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -32388,11 +32339,11 @@
         <v>3.4163709297218122E-4</v>
       </c>
       <c r="T244" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>3814.5899999999997</v>
       </c>
       <c r="U244" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>20.959285714285709</v>
       </c>
     </row>
@@ -32448,11 +32399,11 @@
         <v>4.97414899380909E-4</v>
       </c>
       <c r="T245" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>2734.5699999999997</v>
       </c>
       <c r="U245" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>15.025109890109889</v>
       </c>
     </row>
@@ -32508,11 +32459,11 @@
         <v>0</v>
       </c>
       <c r="T246" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U246" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -32568,11 +32519,11 @@
         <v>3.5474232444145785E-3</v>
       </c>
       <c r="T247" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>26354.32</v>
       </c>
       <c r="U247" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>144.80395604395605</v>
       </c>
     </row>
@@ -32628,11 +32579,11 @@
         <v>6.1721459233355345E-4</v>
       </c>
       <c r="T248" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>4524.6000000000004</v>
       </c>
       <c r="U248" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>24.860439560439563</v>
       </c>
     </row>
@@ -32688,11 +32639,11 @@
         <v>3.1739457733346989E-3</v>
       </c>
       <c r="T249" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>28295.75</v>
       </c>
       <c r="U249" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>155.47115384615384</v>
       </c>
     </row>
@@ -32748,11 +32699,11 @@
         <v>0</v>
       </c>
       <c r="T250" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U250" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -32808,11 +32759,11 @@
         <v>0</v>
       </c>
       <c r="T251" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U251" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -32874,11 +32825,11 @@
         <v>8.1776356024359214E-3</v>
       </c>
       <c r="T252" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>65723.83</v>
       </c>
       <c r="U252" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>361.11994505494511</v>
       </c>
     </row>
@@ -32904,11 +32855,11 @@
       <c r="Q253" s="72"/>
       <c r="R253" s="73"/>
       <c r="T253" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U253" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -32964,11 +32915,11 @@
         <v>0</v>
       </c>
       <c r="T254" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U254" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -33024,11 +32975,11 @@
         <v>0</v>
       </c>
       <c r="T255" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U255" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -33084,11 +33035,11 @@
         <v>4.9063514071799964E-2</v>
       </c>
       <c r="T256" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>456490.04</v>
       </c>
       <c r="U256" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>2508.1870329670332</v>
       </c>
     </row>
@@ -33144,11 +33095,11 @@
         <v>0</v>
       </c>
       <c r="T257" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U257" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -33204,11 +33155,11 @@
         <v>5.803267537886788E-3</v>
       </c>
       <c r="T258" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>22943.86</v>
       </c>
       <c r="U258" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>126.06516483516484</v>
       </c>
     </row>
@@ -33264,11 +33215,11 @@
         <v>0</v>
       </c>
       <c r="T259" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U259" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -33324,11 +33275,11 @@
         <v>0</v>
       </c>
       <c r="T260" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U260" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -33384,11 +33335,11 @@
         <v>1.8358944317233911E-2</v>
       </c>
       <c r="T261" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>151388.83000000002</v>
       </c>
       <c r="U261" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>831.8067582417583</v>
       </c>
     </row>
@@ -33444,11 +33395,11 @@
         <v>6.5854436906949984E-3</v>
       </c>
       <c r="T262" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>56233.119999999995</v>
       </c>
       <c r="U262" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>308.97318681318677</v>
       </c>
     </row>
@@ -33510,11 +33461,11 @@
         <v>7.9811169617615654E-2</v>
       </c>
       <c r="T263" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>687055.85</v>
       </c>
       <c r="U263" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>3775.0321428571428</v>
       </c>
     </row>
@@ -33540,11 +33491,11 @@
       <c r="Q264" s="72"/>
       <c r="R264" s="73"/>
       <c r="T264" s="80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U264" s="80">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
@@ -33600,11 +33551,11 @@
         <v>0</v>
       </c>
       <c r="T265" s="80">
-        <f t="shared" ref="T265:T327" si="8">IFERROR(B265+E265+H265+K265+N265+Q265, "NA")</f>
+        <f t="shared" ref="T265:T327" si="10">IFERROR(B265+E265+H265+K265+N265+Q265, "NA")</f>
         <v>0</v>
       </c>
       <c r="U265" s="80">
-        <f t="shared" ref="U265:U327" si="9">(T265/$V$1)/7</f>
+        <f t="shared" ref="U265:U327" si="11">(T265/$V$1)/7</f>
         <v>0</v>
       </c>
     </row>
@@ -33660,11 +33611,11 @@
         <v>0</v>
       </c>
       <c r="T266" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U266" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -33720,11 +33671,11 @@
         <v>0</v>
       </c>
       <c r="T267" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U267" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -33780,11 +33731,11 @@
         <v>-7.3527701312772943E-6</v>
       </c>
       <c r="T268" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>-33.08</v>
       </c>
       <c r="U268" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>-0.18175824175824173</v>
       </c>
     </row>
@@ -33840,11 +33791,11 @@
         <v>0</v>
       </c>
       <c r="T269" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U269" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -33900,11 +33851,11 @@
         <v>0</v>
       </c>
       <c r="T270" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U270" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -33960,11 +33911,11 @@
         <v>0</v>
       </c>
       <c r="T271" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U271" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -34020,11 +33971,11 @@
         <v>0</v>
       </c>
       <c r="T272" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U272" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -34080,11 +34031,11 @@
         <v>0</v>
       </c>
       <c r="T273" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U273" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -34140,11 +34091,11 @@
         <v>0</v>
       </c>
       <c r="T274" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U274" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -34200,11 +34151,11 @@
         <v>0</v>
       </c>
       <c r="T275" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U275" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -34260,11 +34211,11 @@
         <v>0</v>
       </c>
       <c r="T276" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U276" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -34320,11 +34271,11 @@
         <v>0</v>
       </c>
       <c r="T277" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U277" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -34380,11 +34331,11 @@
         <v>-3.6517467979605173E-2</v>
       </c>
       <c r="T278" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>-415848.28</v>
       </c>
       <c r="U278" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>-2284.8806593406593</v>
       </c>
     </row>
@@ -34440,11 +34391,11 @@
         <v>0</v>
       </c>
       <c r="T279" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U279" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -34500,11 +34451,11 @@
         <v>0</v>
       </c>
       <c r="T280" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U280" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -34560,11 +34511,11 @@
         <v>0</v>
       </c>
       <c r="T281" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U281" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -34620,11 +34571,11 @@
         <v>0</v>
       </c>
       <c r="T282" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U282" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -34686,11 +34637,11 @@
         <v>-3.6524820749736446E-2</v>
       </c>
       <c r="T283" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>-415881.36</v>
       </c>
       <c r="U283" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>-2285.0624175824173</v>
       </c>
     </row>
@@ -34752,11 +34703,11 @@
         <v>0.15442938045263321</v>
       </c>
       <c r="T284" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>1200303.03</v>
       </c>
       <c r="U284" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>6595.0715934065938</v>
       </c>
     </row>
@@ -34782,11 +34733,11 @@
       <c r="Q285" s="72"/>
       <c r="R285" s="73"/>
       <c r="T285" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U285" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -34812,11 +34763,11 @@
       <c r="Q286" s="72"/>
       <c r="R286" s="73"/>
       <c r="T286" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U286" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -34872,11 +34823,11 @@
         <v>0</v>
       </c>
       <c r="T287" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U287" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -34932,11 +34883,11 @@
         <v>0</v>
       </c>
       <c r="T288" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U288" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -34992,11 +34943,11 @@
         <v>4.8021806759152158E-3</v>
       </c>
       <c r="T289" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>68669.119999999995</v>
       </c>
       <c r="U289" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>377.30285714285714</v>
       </c>
     </row>
@@ -35052,11 +35003,11 @@
         <v>5.2216929757552419E-2</v>
       </c>
       <c r="T290" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>590935.91</v>
       </c>
       <c r="U290" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>3246.9006043956042</v>
       </c>
     </row>
@@ -35112,11 +35063,11 @@
         <v>0</v>
       </c>
       <c r="T291" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>74</v>
       </c>
       <c r="U291" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0.40659340659340659</v>
       </c>
     </row>
@@ -35172,11 +35123,11 @@
         <v>1.4417196335837833E-3</v>
       </c>
       <c r="T292" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>15742</v>
       </c>
       <c r="U292" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>86.494505494505489</v>
       </c>
     </row>
@@ -35232,11 +35183,11 @@
         <v>4.5102757017035072E-4</v>
       </c>
       <c r="T293" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>1522.53</v>
       </c>
       <c r="U293" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>8.3655494505494499</v>
       </c>
     </row>
@@ -35292,11 +35243,11 @@
         <v>2.2804328218229814E-3</v>
       </c>
       <c r="T294" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>39694.439999999995</v>
       </c>
       <c r="U294" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>218.10131868131865</v>
       </c>
     </row>
@@ -35352,11 +35303,11 @@
         <v>0</v>
       </c>
       <c r="T295" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U295" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -35412,11 +35363,11 @@
         <v>0</v>
       </c>
       <c r="T296" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U296" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -35472,11 +35423,11 @@
         <v>0</v>
       </c>
       <c r="T297" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>482.48</v>
       </c>
       <c r="U297" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>2.6509890109890111</v>
       </c>
     </row>
@@ -35532,11 +35483,11 @@
         <v>0</v>
       </c>
       <c r="T298" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U298" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -35592,11 +35543,11 @@
         <v>0</v>
       </c>
       <c r="T299" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U299" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -35652,11 +35603,11 @@
         <v>0</v>
       </c>
       <c r="T300" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U300" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -35712,11 +35663,11 @@
         <v>0</v>
       </c>
       <c r="T301" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U301" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -35772,11 +35723,11 @@
         <v>0</v>
       </c>
       <c r="T302" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U302" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -35832,11 +35783,11 @@
         <v>0</v>
       </c>
       <c r="T303" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U303" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -35892,11 +35843,11 @@
         <v>0</v>
       </c>
       <c r="T304" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U304" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -35952,11 +35903,11 @@
         <v>0</v>
       </c>
       <c r="T305" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U305" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -36012,11 +35963,11 @@
         <v>0</v>
       </c>
       <c r="T306" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U306" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -36072,11 +36023,11 @@
         <v>0</v>
       </c>
       <c r="T307" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U307" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -36132,11 +36083,11 @@
         <v>0</v>
       </c>
       <c r="T308" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U308" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -36192,11 +36143,11 @@
         <v>0</v>
       </c>
       <c r="T309" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U309" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -36252,11 +36203,11 @@
         <v>0</v>
       </c>
       <c r="T310" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U310" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -36312,11 +36263,11 @@
         <v>0</v>
       </c>
       <c r="T311" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U311" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -36372,11 +36323,11 @@
         <v>0</v>
       </c>
       <c r="T312" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U312" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -36432,11 +36383,11 @@
         <v>0</v>
       </c>
       <c r="T313" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U313" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -36498,11 +36449,11 @@
         <v>6.1192290459044757E-2</v>
       </c>
       <c r="T314" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>717120.4800000001</v>
       </c>
       <c r="U314" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>3940.2224175824181</v>
       </c>
     </row>
@@ -36528,11 +36479,11 @@
       <c r="Q315" s="72"/>
       <c r="R315" s="73"/>
       <c r="T315" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U315" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -36588,11 +36539,11 @@
         <v>0</v>
       </c>
       <c r="T316" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U316" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -36648,11 +36599,11 @@
         <v>0</v>
       </c>
       <c r="T317" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U317" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -36708,11 +36659,11 @@
         <v>0</v>
       </c>
       <c r="T318" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U318" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -36768,11 +36719,11 @@
         <v>0</v>
       </c>
       <c r="T319" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>170</v>
       </c>
       <c r="U319" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0.93406593406593408</v>
       </c>
     </row>
@@ -36828,11 +36779,11 @@
         <v>0</v>
       </c>
       <c r="T320" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U320" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -36888,11 +36839,11 @@
         <v>0</v>
       </c>
       <c r="T321" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U321" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -36948,11 +36899,11 @@
         <v>0</v>
       </c>
       <c r="T322" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U322" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -37008,11 +36959,11 @@
         <v>0</v>
       </c>
       <c r="T323" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U323" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
@@ -37074,11 +37025,11 @@
         <v>0</v>
       </c>
       <c r="T324" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>170</v>
       </c>
       <c r="U324" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0.93406593406593408</v>
       </c>
     </row>
@@ -37140,11 +37091,11 @@
         <v>6.1192290459044757E-2</v>
       </c>
       <c r="T325" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>717290.4800000001</v>
       </c>
       <c r="U325" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>3941.1564835164841</v>
       </c>
     </row>
@@ -37206,11 +37157,11 @@
         <v>0.22548779088018195</v>
       </c>
       <c r="T326" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>3910740.629999999</v>
       </c>
       <c r="U326" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>21487.58587912087</v>
       </c>
     </row>
@@ -37248,11 +37199,11 @@
       </c>
       <c r="R327" s="90"/>
       <c r="T327" s="80">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>11439240.35</v>
       </c>
       <c r="U327" s="80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>62852.968956043951</v>
       </c>
     </row>

</xml_diff>